<commit_message>
Clear the workbook's stale notes and counts
All 348 'v3 addition' Notes cells are empty, Start Here reads 917
questions, Core (387) and 172 patterns, and the Dashboard reads All 917
questions. Master data, formulas, formatting, dropdowns and freeze panes
are unchanged.
</commit_message>
<xml_diff>
--- a/DSA_Master_Sheet.xlsx
+++ b/DSA_Master_Sheet.xlsx
@@ -892,14 +892,14 @@
       </c>
       <c r="C8" s="36" t="inlineStr">
         <is>
-          <t>922 questions is not a plan, it is a wall. The Tier column splits them into three tracks, and the Step column orders them: work down it, and see Path Stages for the ranges.</t>
+          <t>917 questions is not a plan, it is a wall. The Tier column splits them into three tracks, and the Step column orders them: work down it, and see Path Stages for the ranges.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="27.75" customHeight="1" s="32">
       <c r="C9" s="36" t="inlineStr">
         <is>
-          <t>Core (373) - at least two problems per pattern, every pattern in the sheet. Finish this and you have touched every idea an interview can ask. This is your actual target.</t>
+          <t>Core (387) - at least two problems per pattern, every pattern in the sheet. Finish this and you have touched every idea an interview can ask. This is your actual target.</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="C30" s="36" t="inlineStr">
         <is>
-          <t>Per-pattern totals, done count and average confidence across all 168 patterns.</t>
+          <t>Per-pattern totals, done count and average confidence across all 172 patterns.</t>
         </is>
       </c>
     </row>
@@ -3345,11 +3345,7 @@
         <f>IF(OR($J19="Attempted",$J19="Revisit"),"DUE",IF($N19="","",IF($N19&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P19" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P19" s="61" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="32">
       <c r="A20" s="61" t="n">
@@ -3411,11 +3407,7 @@
         <f>IF(OR($J20="Attempted",$J20="Revisit"),"DUE",IF($N20="","",IF($N20&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P20" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P20" s="61" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="32">
       <c r="A21" s="61" t="n">
@@ -3477,11 +3469,7 @@
         <f>IF(OR($J21="Attempted",$J21="Revisit"),"DUE",IF($N21="","",IF($N21&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P21" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P21" s="61" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="32">
       <c r="A22" s="61" t="n">
@@ -3729,11 +3717,7 @@
         <f>IF(OR($J25="Attempted",$J25="Revisit"),"DUE",IF($N25="","",IF($N25&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P25" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P25" s="61" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1" s="32">
       <c r="A26" s="61" t="n">
@@ -3857,11 +3841,7 @@
         <f>IF(OR($J27="Attempted",$J27="Revisit"),"DUE",IF($N27="","",IF($N27&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P27" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P27" s="61" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1" s="32">
       <c r="A28" s="61" t="n">
@@ -3923,11 +3903,7 @@
         <f>IF(OR($J28="Attempted",$J28="Revisit"),"DUE",IF($N28="","",IF($N28&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P28" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P28" s="61" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1" s="32">
       <c r="A29" s="61" t="n">
@@ -3989,11 +3965,7 @@
         <f>IF(OR($J29="Attempted",$J29="Revisit"),"DUE",IF($N29="","",IF($N29&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P29" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P29" s="61" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1" s="32">
       <c r="A30" s="61" t="n">
@@ -4241,11 +4213,7 @@
         <f>IF(OR($J33="Attempted",$J33="Revisit"),"DUE",IF($N33="","",IF($N33&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P33" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P33" s="61" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1" s="32">
       <c r="A34" s="61" t="n">
@@ -4555,11 +4523,7 @@
         <f>IF(OR($J38="Attempted",$J38="Revisit"),"DUE",IF($N38="","",IF($N38&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P38" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P38" s="61" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1" s="32">
       <c r="A39" s="61" t="n">
@@ -5551,11 +5515,7 @@
         <f>IF(OR($J54="Attempted",$J54="Revisit"),"DUE",IF($N54="","",IF($N54&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P54" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P54" s="61" t="n"/>
     </row>
     <row r="55" ht="15" customHeight="1" s="32">
       <c r="A55" s="61" t="n">
@@ -5927,11 +5887,7 @@
         <f>IF(OR($J60="Attempted",$J60="Revisit"),"DUE",IF($N60="","",IF($N60&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P60" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P60" s="61" t="n"/>
     </row>
     <row r="61" ht="15" customHeight="1" s="32">
       <c r="A61" s="61" t="n">
@@ -6117,11 +6073,7 @@
         <f>IF(OR($J63="Attempted",$J63="Revisit"),"DUE",IF($N63="","",IF($N63&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P63" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P63" s="61" t="n"/>
     </row>
     <row r="64" ht="15" customHeight="1" s="32">
       <c r="A64" s="61" t="n">
@@ -6183,11 +6135,7 @@
         <f>IF(OR($J64="Attempted",$J64="Revisit"),"DUE",IF($N64="","",IF($N64&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P64" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P64" s="61" t="n"/>
     </row>
     <row r="65" ht="15" customHeight="1" s="32">
       <c r="A65" s="61" t="n">
@@ -6249,11 +6197,7 @@
         <f>IF(OR($J65="Attempted",$J65="Revisit"),"DUE",IF($N65="","",IF($N65&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P65" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P65" s="61" t="n"/>
     </row>
     <row r="66" ht="15" customHeight="1" s="32">
       <c r="A66" s="61" t="n">
@@ -6439,11 +6383,7 @@
         <f>IF(OR($J68="Attempted",$J68="Revisit"),"DUE",IF($N68="","",IF($N68&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P68" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P68" s="61" t="n"/>
     </row>
     <row r="69" ht="15" customHeight="1" s="32">
       <c r="A69" s="61" t="n">
@@ -6505,11 +6445,7 @@
         <f>IF(OR($J69="Attempted",$J69="Revisit"),"DUE",IF($N69="","",IF($N69&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P69" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P69" s="61" t="n"/>
     </row>
     <row r="70" ht="15" customHeight="1" s="32">
       <c r="A70" s="61" t="n">
@@ -7439,11 +7375,7 @@
         <f>IF(OR($J84="Attempted",$J84="Revisit"),"DUE",IF($N84="","",IF($N84&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P84" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P84" s="61" t="n"/>
     </row>
     <row r="85" ht="15" customHeight="1" s="32">
       <c r="A85" s="61" t="n">
@@ -7505,11 +7437,7 @@
         <f>IF(OR($J85="Attempted",$J85="Revisit"),"DUE",IF($N85="","",IF($N85&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P85" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P85" s="61" t="n"/>
     </row>
     <row r="86" ht="15" customHeight="1" s="32">
       <c r="A86" s="61" t="n">
@@ -7571,11 +7499,7 @@
         <f>IF(OR($J86="Attempted",$J86="Revisit"),"DUE",IF($N86="","",IF($N86&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P86" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P86" s="61" t="n"/>
     </row>
     <row r="87" ht="15" customHeight="1" s="32">
       <c r="A87" s="61" t="n">
@@ -7761,11 +7685,7 @@
         <f>IF(OR($J89="Attempted",$J89="Revisit"),"DUE",IF($N89="","",IF($N89&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P89" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P89" s="61" t="n"/>
     </row>
     <row r="90" ht="15" customHeight="1" s="32">
       <c r="A90" s="61" t="n">
@@ -8013,11 +7933,7 @@
         <f>IF(OR($J93="Attempted",$J93="Revisit"),"DUE",IF($N93="","",IF($N93&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P93" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P93" s="61" t="n"/>
     </row>
     <row r="94" ht="15" customHeight="1" s="32">
       <c r="A94" s="61" t="n">
@@ -8451,11 +8367,7 @@
         <f>IF(OR($J100="Attempted",$J100="Revisit"),"DUE",IF($N100="","",IF($N100&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P100" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P100" s="61" t="n"/>
     </row>
     <row r="101" ht="15" customHeight="1" s="32">
       <c r="A101" s="61" t="n">
@@ -8517,11 +8429,7 @@
         <f>IF(OR($J101="Attempted",$J101="Revisit"),"DUE",IF($N101="","",IF($N101&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P101" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P101" s="61" t="n"/>
     </row>
     <row r="102" ht="15" customHeight="1" s="32">
       <c r="A102" s="61" t="n">
@@ -8583,11 +8491,7 @@
         <f>IF(OR($J102="Attempted",$J102="Revisit"),"DUE",IF($N102="","",IF($N102&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P102" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P102" s="61" t="n"/>
     </row>
     <row r="103" ht="15" customHeight="1" s="32">
       <c r="A103" s="61" t="n">
@@ -8711,11 +8615,7 @@
         <f>IF(OR($J104="Attempted",$J104="Revisit"),"DUE",IF($N104="","",IF($N104&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P104" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P104" s="61" t="n"/>
     </row>
     <row r="105" ht="15" customHeight="1" s="32">
       <c r="A105" s="61" t="n">
@@ -8777,11 +8677,7 @@
         <f>IF(OR($J105="Attempted",$J105="Revisit"),"DUE",IF($N105="","",IF($N105&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P105" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P105" s="61" t="n"/>
     </row>
     <row r="106" ht="15" customHeight="1" s="32">
       <c r="A106" s="61" t="n">
@@ -8843,11 +8739,7 @@
         <f>IF(OR($J106="Attempted",$J106="Revisit"),"DUE",IF($N106="","",IF($N106&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P106" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P106" s="61" t="n"/>
     </row>
     <row r="107" ht="15" customHeight="1" s="32">
       <c r="A107" s="61" t="n">
@@ -8909,11 +8801,7 @@
         <f>IF(OR($J107="Attempted",$J107="Revisit"),"DUE",IF($N107="","",IF($N107&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P107" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P107" s="61" t="n"/>
     </row>
     <row r="108" ht="15" customHeight="1" s="32">
       <c r="A108" s="61" t="n">
@@ -8975,11 +8863,7 @@
         <f>IF(OR($J108="Attempted",$J108="Revisit"),"DUE",IF($N108="","",IF($N108&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P108" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P108" s="61" t="n"/>
     </row>
     <row r="109" ht="15" customHeight="1" s="32">
       <c r="A109" s="61" t="n">
@@ -9661,11 +9545,7 @@
         <f>IF(OR($J119="Attempted",$J119="Revisit"),"DUE",IF($N119="","",IF($N119&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P119" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P119" s="61" t="n"/>
     </row>
     <row r="120" ht="15" customHeight="1" s="32">
       <c r="A120" s="61" t="n">
@@ -9727,11 +9607,7 @@
         <f>IF(OR($J120="Attempted",$J120="Revisit"),"DUE",IF($N120="","",IF($N120&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P120" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P120" s="61" t="n"/>
     </row>
     <row r="121" ht="15" customHeight="1" s="32">
       <c r="A121" s="61" t="n">
@@ -9793,11 +9669,7 @@
         <f>IF(OR($J121="Attempted",$J121="Revisit"),"DUE",IF($N121="","",IF($N121&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P121" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P121" s="61" t="n"/>
     </row>
     <row r="122" ht="15" customHeight="1" s="32">
       <c r="A122" s="61" t="n">
@@ -9859,11 +9731,7 @@
         <f>IF(OR($J122="Attempted",$J122="Revisit"),"DUE",IF($N122="","",IF($N122&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P122" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P122" s="61" t="n"/>
     </row>
     <row r="123" ht="15" customHeight="1" s="32">
       <c r="A123" s="61" t="n">
@@ -9925,11 +9793,7 @@
         <f>IF(OR($J123="Attempted",$J123="Revisit"),"DUE",IF($N123="","",IF($N123&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P123" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P123" s="61" t="n"/>
     </row>
     <row r="124" ht="15" customHeight="1" s="32">
       <c r="A124" s="61" t="n">
@@ -9991,11 +9855,7 @@
         <f>IF(OR($J124="Attempted",$J124="Revisit"),"DUE",IF($N124="","",IF($N124&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P124" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P124" s="61" t="n"/>
     </row>
     <row r="125" ht="15" customHeight="1" s="32">
       <c r="A125" s="61" t="n">
@@ -10181,11 +10041,7 @@
         <f>IF(OR($J127="Attempted",$J127="Revisit"),"DUE",IF($N127="","",IF($N127&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P127" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P127" s="61" t="n"/>
     </row>
     <row r="128" ht="15" customHeight="1" s="32">
       <c r="A128" s="61" t="n">
@@ -10619,11 +10475,7 @@
         <f>IF(OR($J134="Attempted",$J134="Revisit"),"DUE",IF($N134="","",IF($N134&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P134" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P134" s="61" t="n"/>
     </row>
     <row r="135" ht="15" customHeight="1" s="32">
       <c r="A135" s="61" t="n">
@@ -10685,11 +10537,7 @@
         <f>IF(OR($J135="Attempted",$J135="Revisit"),"DUE",IF($N135="","",IF($N135&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P135" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P135" s="61" t="n"/>
     </row>
     <row r="136" ht="15" customHeight="1" s="32">
       <c r="A136" s="61" t="n">
@@ -10751,11 +10599,7 @@
         <f>IF(OR($J136="Attempted",$J136="Revisit"),"DUE",IF($N136="","",IF($N136&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P136" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P136" s="61" t="n"/>
     </row>
     <row r="137" ht="15" customHeight="1" s="32">
       <c r="A137" s="61" t="n">
@@ -10817,11 +10661,7 @@
         <f>IF(OR($J137="Attempted",$J137="Revisit"),"DUE",IF($N137="","",IF($N137&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P137" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P137" s="61" t="n"/>
     </row>
     <row r="138" ht="15" customHeight="1" s="32">
       <c r="A138" s="61" t="n">
@@ -10883,11 +10723,7 @@
         <f>IF(OR($J138="Attempted",$J138="Revisit"),"DUE",IF($N138="","",IF($N138&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P138" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P138" s="61" t="n"/>
     </row>
     <row r="139" ht="15" customHeight="1" s="32">
       <c r="A139" s="61" t="n">
@@ -10949,11 +10785,7 @@
         <f>IF(OR($J139="Attempted",$J139="Revisit"),"DUE",IF($N139="","",IF($N139&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P139" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P139" s="61" t="n"/>
     </row>
     <row r="140" ht="15" customHeight="1" s="32">
       <c r="A140" s="61" t="n">
@@ -11015,11 +10847,7 @@
         <f>IF(OR($J140="Attempted",$J140="Revisit"),"DUE",IF($N140="","",IF($N140&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P140" s="61" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P140" s="61" t="n"/>
     </row>
     <row r="141" ht="15" customHeight="1" s="32">
       <c r="A141" s="61" t="n">
@@ -11267,11 +11095,7 @@
         <f>IF(OR($J144="Attempted",$J144="Revisit"),"DUE",IF($N144="","",IF($N144&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P144" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P144" s="62" t="n"/>
     </row>
     <row r="145" ht="15" customHeight="1" s="32">
       <c r="A145" s="62" t="n">
@@ -11333,11 +11157,7 @@
         <f>IF(OR($J145="Attempted",$J145="Revisit"),"DUE",IF($N145="","",IF($N145&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P145" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P145" s="62" t="n"/>
     </row>
     <row r="146" ht="15" customHeight="1" s="32">
       <c r="A146" s="62" t="n">
@@ -11399,11 +11219,7 @@
         <f>IF(OR($J146="Attempted",$J146="Revisit"),"DUE",IF($N146="","",IF($N146&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P146" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P146" s="62" t="n"/>
     </row>
     <row r="147" ht="15" customHeight="1" s="32">
       <c r="A147" s="62" t="n">
@@ -11589,11 +11405,7 @@
         <f>IF(OR($J149="Attempted",$J149="Revisit"),"DUE",IF($N149="","",IF($N149&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P149" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P149" s="62" t="n"/>
     </row>
     <row r="150" ht="15" customHeight="1" s="32">
       <c r="A150" s="62" t="n">
@@ -11717,11 +11529,7 @@
         <f>IF(OR($J151="Attempted",$J151="Revisit"),"DUE",IF($N151="","",IF($N151&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P151" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P151" s="62" t="n"/>
     </row>
     <row r="152" ht="15" customHeight="1" s="32">
       <c r="A152" s="62" t="n">
@@ -11907,11 +11715,7 @@
         <f>IF(OR($J154="Attempted",$J154="Revisit"),"DUE",IF($N154="","",IF($N154&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P154" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P154" s="62" t="n"/>
     </row>
     <row r="155" ht="15" customHeight="1" s="32">
       <c r="A155" s="62" t="n">
@@ -12097,11 +11901,7 @@
         <f>IF(OR($J157="Attempted",$J157="Revisit"),"DUE",IF($N157="","",IF($N157&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P157" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P157" s="62" t="n"/>
     </row>
     <row r="158" ht="15" customHeight="1" s="32">
       <c r="A158" s="62" t="n">
@@ -12163,11 +11963,7 @@
         <f>IF(OR($J158="Attempted",$J158="Revisit"),"DUE",IF($N158="","",IF($N158&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P158" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P158" s="62" t="n"/>
     </row>
     <row r="159" ht="15" customHeight="1" s="32">
       <c r="A159" s="62" t="n">
@@ -12229,11 +12025,7 @@
         <f>IF(OR($J159="Attempted",$J159="Revisit"),"DUE",IF($N159="","",IF($N159&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P159" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P159" s="62" t="n"/>
     </row>
     <row r="160" ht="15" customHeight="1" s="32">
       <c r="A160" s="62" t="n">
@@ -12915,11 +12707,7 @@
         <f>IF(OR($J170="Attempted",$J170="Revisit"),"DUE",IF($N170="","",IF($N170&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P170" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P170" s="62" t="n"/>
     </row>
     <row r="171" ht="15" customHeight="1" s="32">
       <c r="A171" s="62" t="n">
@@ -13043,11 +12831,7 @@
         <f>IF(OR($J172="Attempted",$J172="Revisit"),"DUE",IF($N172="","",IF($N172&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P172" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P172" s="62" t="n"/>
     </row>
     <row r="173" ht="15" customHeight="1" s="32">
       <c r="A173" s="62" t="n">
@@ -13295,11 +13079,7 @@
         <f>IF(OR($J176="Attempted",$J176="Revisit"),"DUE",IF($N176="","",IF($N176&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P176" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P176" s="62" t="n"/>
     </row>
     <row r="177" ht="15" customHeight="1" s="32">
       <c r="A177" s="62" t="n">
@@ -13609,11 +13389,7 @@
         <f>IF(OR($J181="Attempted",$J181="Revisit"),"DUE",IF($N181="","",IF($N181&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P181" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P181" s="62" t="n"/>
     </row>
     <row r="182" ht="15" customHeight="1" s="32">
       <c r="A182" s="62" t="n">
@@ -14047,11 +13823,7 @@
         <f>IF(OR($J188="Attempted",$J188="Revisit"),"DUE",IF($N188="","",IF($N188&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P188" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P188" s="62" t="n"/>
     </row>
     <row r="189" ht="15" customHeight="1" s="32">
       <c r="A189" s="62" t="n">
@@ -14237,11 +14009,7 @@
         <f>IF(OR($J191="Attempted",$J191="Revisit"),"DUE",IF($N191="","",IF($N191&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P191" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P191" s="62" t="n"/>
     </row>
     <row r="192" ht="15" customHeight="1" s="32">
       <c r="A192" s="62" t="n">
@@ -14303,11 +14071,7 @@
         <f>IF(OR($J192="Attempted",$J192="Revisit"),"DUE",IF($N192="","",IF($N192&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P192" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P192" s="62" t="n"/>
     </row>
     <row r="193" ht="15" customHeight="1" s="32">
       <c r="A193" s="62" t="n">
@@ -14369,11 +14133,7 @@
         <f>IF(OR($J193="Attempted",$J193="Revisit"),"DUE",IF($N193="","",IF($N193&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P193" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P193" s="62" t="n"/>
     </row>
     <row r="194" ht="15" customHeight="1" s="32">
       <c r="A194" s="62" t="n">
@@ -14559,11 +14319,7 @@
         <f>IF(OR($J196="Attempted",$J196="Revisit"),"DUE",IF($N196="","",IF($N196&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P196" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P196" s="62" t="n"/>
     </row>
     <row r="197" ht="15" customHeight="1" s="32">
       <c r="A197" s="62" t="n">
@@ -14625,11 +14381,7 @@
         <f>IF(OR($J197="Attempted",$J197="Revisit"),"DUE",IF($N197="","",IF($N197&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P197" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P197" s="62" t="n"/>
     </row>
     <row r="198" ht="15" customHeight="1" s="32">
       <c r="A198" s="62" t="n">
@@ -14753,11 +14505,7 @@
         <f>IF(OR($J199="Attempted",$J199="Revisit"),"DUE",IF($N199="","",IF($N199&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P199" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P199" s="62" t="n"/>
     </row>
     <row r="200" ht="15" customHeight="1" s="32">
       <c r="A200" s="62" t="n">
@@ -15191,11 +14939,7 @@
         <f>IF(OR($J206="Attempted",$J206="Revisit"),"DUE",IF($N206="","",IF($N206&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P206" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P206" s="62" t="n"/>
     </row>
     <row r="207" ht="15" customHeight="1" s="32">
       <c r="A207" s="62" t="n">
@@ -15257,11 +15001,7 @@
         <f>IF(OR($J207="Attempted",$J207="Revisit"),"DUE",IF($N207="","",IF($N207&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P207" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P207" s="62" t="n"/>
     </row>
     <row r="208" ht="15" customHeight="1" s="32">
       <c r="A208" s="62" t="n">
@@ -15323,11 +15063,7 @@
         <f>IF(OR($J208="Attempted",$J208="Revisit"),"DUE",IF($N208="","",IF($N208&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P208" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P208" s="62" t="n"/>
     </row>
     <row r="209" ht="15" customHeight="1" s="32">
       <c r="A209" s="62" t="n">
@@ -15389,11 +15125,7 @@
         <f>IF(OR($J209="Attempted",$J209="Revisit"),"DUE",IF($N209="","",IF($N209&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P209" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P209" s="62" t="n"/>
     </row>
     <row r="210" ht="15" customHeight="1" s="32">
       <c r="A210" s="62" t="n">
@@ -15517,11 +15249,7 @@
         <f>IF(OR($J211="Attempted",$J211="Revisit"),"DUE",IF($N211="","",IF($N211&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P211" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P211" s="62" t="n"/>
     </row>
     <row r="212" ht="15" customHeight="1" s="32">
       <c r="A212" s="62" t="n">
@@ -15769,11 +15497,7 @@
         <f>IF(OR($J215="Attempted",$J215="Revisit"),"DUE",IF($N215="","",IF($N215&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P215" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P215" s="62" t="n"/>
     </row>
     <row r="216" ht="15" customHeight="1" s="32">
       <c r="A216" s="62" t="n">
@@ -15835,11 +15559,7 @@
         <f>IF(OR($J216="Attempted",$J216="Revisit"),"DUE",IF($N216="","",IF($N216&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P216" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P216" s="62" t="n"/>
     </row>
     <row r="217" ht="15" customHeight="1" s="32">
       <c r="A217" s="62" t="n">
@@ -16025,11 +15745,7 @@
         <f>IF(OR($J219="Attempted",$J219="Revisit"),"DUE",IF($N219="","",IF($N219&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P219" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P219" s="62" t="n"/>
     </row>
     <row r="220" ht="15" customHeight="1" s="32">
       <c r="A220" s="62" t="n">
@@ -16215,11 +15931,7 @@
         <f>IF(OR($J222="Attempted",$J222="Revisit"),"DUE",IF($N222="","",IF($N222&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P222" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P222" s="62" t="n"/>
     </row>
     <row r="223" ht="15" customHeight="1" s="32">
       <c r="A223" s="62" t="n">
@@ -16281,11 +15993,7 @@
         <f>IF(OR($J223="Attempted",$J223="Revisit"),"DUE",IF($N223="","",IF($N223&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P223" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P223" s="62" t="n"/>
     </row>
     <row r="224" ht="15" customHeight="1" s="32">
       <c r="A224" s="62" t="n">
@@ -16347,11 +16055,7 @@
         <f>IF(OR($J224="Attempted",$J224="Revisit"),"DUE",IF($N224="","",IF($N224&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P224" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P224" s="62" t="n"/>
     </row>
     <row r="225" ht="15" customHeight="1" s="32">
       <c r="A225" s="62" t="n">
@@ -16413,11 +16117,7 @@
         <f>IF(OR($J225="Attempted",$J225="Revisit"),"DUE",IF($N225="","",IF($N225&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P225" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P225" s="62" t="n"/>
     </row>
     <row r="226" ht="15" customHeight="1" s="32">
       <c r="A226" s="62" t="n">
@@ -16479,11 +16179,7 @@
         <f>IF(OR($J226="Attempted",$J226="Revisit"),"DUE",IF($N226="","",IF($N226&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P226" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P226" s="62" t="n"/>
     </row>
     <row r="227" ht="15" customHeight="1" s="32">
       <c r="A227" s="62" t="n">
@@ -16545,11 +16241,7 @@
         <f>IF(OR($J227="Attempted",$J227="Revisit"),"DUE",IF($N227="","",IF($N227&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P227" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P227" s="62" t="n"/>
     </row>
     <row r="228" ht="15" customHeight="1" s="32">
       <c r="A228" s="62" t="n">
@@ -16611,11 +16303,7 @@
         <f>IF(OR($J228="Attempted",$J228="Revisit"),"DUE",IF($N228="","",IF($N228&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P228" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P228" s="62" t="n"/>
     </row>
     <row r="229" ht="15" customHeight="1" s="32">
       <c r="A229" s="62" t="n">
@@ -17421,11 +17109,7 @@
         <f>IF(OR($J241="Attempted",$J241="Revisit"),"DUE",IF($N241="","",IF($N241&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P241" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P241" s="62" t="n"/>
     </row>
     <row r="242" ht="15" customHeight="1" s="32">
       <c r="A242" s="62" t="n">
@@ -17487,11 +17171,7 @@
         <f>IF(OR($J242="Attempted",$J242="Revisit"),"DUE",IF($N242="","",IF($N242&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P242" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P242" s="62" t="n"/>
     </row>
     <row r="243" ht="15" customHeight="1" s="32">
       <c r="A243" s="62" t="n">
@@ -17553,11 +17233,7 @@
         <f>IF(OR($J243="Attempted",$J243="Revisit"),"DUE",IF($N243="","",IF($N243&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P243" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P243" s="62" t="n"/>
     </row>
     <row r="244" ht="15" customHeight="1" s="32">
       <c r="A244" s="62" t="n">
@@ -17619,11 +17295,7 @@
         <f>IF(OR($J244="Attempted",$J244="Revisit"),"DUE",IF($N244="","",IF($N244&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P244" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P244" s="62" t="n"/>
     </row>
     <row r="245" ht="15" customHeight="1" s="32">
       <c r="A245" s="62" t="n">
@@ -17685,11 +17357,7 @@
         <f>IF(OR($J245="Attempted",$J245="Revisit"),"DUE",IF($N245="","",IF($N245&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P245" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P245" s="62" t="n"/>
     </row>
     <row r="246" ht="15" customHeight="1" s="32">
       <c r="A246" s="62" t="n">
@@ -17751,11 +17419,7 @@
         <f>IF(OR($J246="Attempted",$J246="Revisit"),"DUE",IF($N246="","",IF($N246&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P246" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P246" s="62" t="n"/>
     </row>
     <row r="247" ht="15" customHeight="1" s="32">
       <c r="A247" s="62" t="n">
@@ -18127,11 +17791,7 @@
         <f>IF(OR($J252="Attempted",$J252="Revisit"),"DUE",IF($N252="","",IF($N252&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P252" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P252" s="62" t="n"/>
     </row>
     <row r="253" ht="15" customHeight="1" s="32">
       <c r="A253" s="62" t="n">
@@ -18751,11 +18411,7 @@
         <f>IF(OR($J262="Attempted",$J262="Revisit"),"DUE",IF($N262="","",IF($N262&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P262" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P262" s="62" t="n"/>
     </row>
     <row r="263" ht="15" customHeight="1" s="32">
       <c r="A263" s="62" t="n">
@@ -18817,11 +18473,7 @@
         <f>IF(OR($J263="Attempted",$J263="Revisit"),"DUE",IF($N263="","",IF($N263&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P263" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P263" s="62" t="n"/>
     </row>
     <row r="264" ht="15" customHeight="1" s="32">
       <c r="A264" s="62" t="n">
@@ -18883,11 +18535,7 @@
         <f>IF(OR($J264="Attempted",$J264="Revisit"),"DUE",IF($N264="","",IF($N264&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P264" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P264" s="62" t="n"/>
     </row>
     <row r="265" ht="15" customHeight="1" s="32">
       <c r="A265" s="62" t="n">
@@ -18949,11 +18597,7 @@
         <f>IF(OR($J265="Attempted",$J265="Revisit"),"DUE",IF($N265="","",IF($N265&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P265" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P265" s="62" t="n"/>
     </row>
     <row r="266" ht="15" customHeight="1" s="32">
       <c r="A266" s="62" t="n">
@@ -19015,11 +18659,7 @@
         <f>IF(OR($J266="Attempted",$J266="Revisit"),"DUE",IF($N266="","",IF($N266&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P266" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P266" s="62" t="n"/>
     </row>
     <row r="267" ht="15" customHeight="1" s="32">
       <c r="A267" s="62" t="n">
@@ -19081,11 +18721,7 @@
         <f>IF(OR($J267="Attempted",$J267="Revisit"),"DUE",IF($N267="","",IF($N267&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P267" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P267" s="62" t="n"/>
     </row>
     <row r="268" ht="15" customHeight="1" s="32">
       <c r="A268" s="62" t="n">
@@ -19147,11 +18783,7 @@
         <f>IF(OR($J268="Attempted",$J268="Revisit"),"DUE",IF($N268="","",IF($N268&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P268" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P268" s="62" t="n"/>
     </row>
     <row r="269" ht="15" customHeight="1" s="32">
       <c r="A269" s="62" t="n">
@@ -19213,11 +18845,7 @@
         <f>IF(OR($J269="Attempted",$J269="Revisit"),"DUE",IF($N269="","",IF($N269&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P269" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P269" s="62" t="n"/>
     </row>
     <row r="270" ht="15" customHeight="1" s="32">
       <c r="A270" s="62" t="n">
@@ -19279,11 +18907,7 @@
         <f>IF(OR($J270="Attempted",$J270="Revisit"),"DUE",IF($N270="","",IF($N270&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P270" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P270" s="62" t="n"/>
     </row>
     <row r="271" ht="15" customHeight="1" s="32">
       <c r="A271" s="62" t="n">
@@ -19345,11 +18969,7 @@
         <f>IF(OR($J271="Attempted",$J271="Revisit"),"DUE",IF($N271="","",IF($N271&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P271" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P271" s="62" t="n"/>
     </row>
     <row r="272" ht="15" customHeight="1" s="32">
       <c r="A272" s="62" t="n">
@@ -19535,11 +19155,7 @@
         <f>IF(OR($J274="Attempted",$J274="Revisit"),"DUE",IF($N274="","",IF($N274&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P274" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P274" s="62" t="n"/>
     </row>
     <row r="275" ht="15" customHeight="1" s="32">
       <c r="A275" s="62" t="n">
@@ -19725,11 +19341,7 @@
         <f>IF(OR($J277="Attempted",$J277="Revisit"),"DUE",IF($N277="","",IF($N277&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P277" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P277" s="62" t="n"/>
     </row>
     <row r="278" ht="15" customHeight="1" s="32">
       <c r="A278" s="62" t="n">
@@ -19791,11 +19403,7 @@
         <f>IF(OR($J278="Attempted",$J278="Revisit"),"DUE",IF($N278="","",IF($N278&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P278" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P278" s="62" t="n"/>
     </row>
     <row r="279" ht="15" customHeight="1" s="32">
       <c r="A279" s="62" t="n">
@@ -19857,11 +19465,7 @@
         <f>IF(OR($J279="Attempted",$J279="Revisit"),"DUE",IF($N279="","",IF($N279&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P279" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P279" s="62" t="n"/>
     </row>
     <row r="280" ht="15" customHeight="1" s="32">
       <c r="A280" s="62" t="n">
@@ -20357,11 +19961,7 @@
         <f>IF(OR($J287="Attempted",$J287="Revisit"),"DUE",IF($N287="","",IF($N287&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P287" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P287" s="62" t="n"/>
     </row>
     <row r="288" ht="15" customHeight="1" s="32">
       <c r="A288" s="62" t="n">
@@ -20423,11 +20023,7 @@
         <f>IF(OR($J288="Attempted",$J288="Revisit"),"DUE",IF($N288="","",IF($N288&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P288" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P288" s="62" t="n"/>
     </row>
     <row r="289" ht="15" customHeight="1" s="32">
       <c r="A289" s="62" t="n">
@@ -20489,11 +20085,7 @@
         <f>IF(OR($J289="Attempted",$J289="Revisit"),"DUE",IF($N289="","",IF($N289&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P289" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P289" s="62" t="n"/>
     </row>
     <row r="290" ht="15" customHeight="1" s="32">
       <c r="A290" s="62" t="n">
@@ -20741,11 +20333,7 @@
         <f>IF(OR($J293="Attempted",$J293="Revisit"),"DUE",IF($N293="","",IF($N293&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P293" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P293" s="62" t="n"/>
     </row>
     <row r="294" ht="15" customHeight="1" s="32">
       <c r="A294" s="62" t="n">
@@ -20807,11 +20395,7 @@
         <f>IF(OR($J294="Attempted",$J294="Revisit"),"DUE",IF($N294="","",IF($N294&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P294" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P294" s="62" t="n"/>
     </row>
     <row r="295" ht="15" customHeight="1" s="32">
       <c r="A295" s="62" t="n">
@@ -20873,11 +20457,7 @@
         <f>IF(OR($J295="Attempted",$J295="Revisit"),"DUE",IF($N295="","",IF($N295&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P295" s="62" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P295" s="62" t="n"/>
     </row>
     <row r="296" ht="15" customHeight="1" s="32">
       <c r="A296" s="63" t="n">
@@ -21745,11 +21325,7 @@
         <f>IF(OR($J309="Attempted",$J309="Revisit"),"DUE",IF($N309="","",IF($N309&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P309" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P309" s="63" t="n"/>
     </row>
     <row r="310" ht="15" customHeight="1" s="32">
       <c r="A310" s="63" t="n">
@@ -21873,11 +21449,7 @@
         <f>IF(OR($J311="Attempted",$J311="Revisit"),"DUE",IF($N311="","",IF($N311&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P311" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P311" s="63" t="n"/>
     </row>
     <row r="312" ht="15" customHeight="1" s="32">
       <c r="A312" s="63" t="n">
@@ -22063,11 +21635,7 @@
         <f>IF(OR($J314="Attempted",$J314="Revisit"),"DUE",IF($N314="","",IF($N314&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P314" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P314" s="63" t="n"/>
     </row>
     <row r="315" ht="15" customHeight="1" s="32">
       <c r="A315" s="63" t="n">
@@ -23989,11 +23557,7 @@
         <f>IF(OR($J345="Attempted",$J345="Revisit"),"DUE",IF($N345="","",IF($N345&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P345" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P345" s="63" t="n"/>
     </row>
     <row r="346" ht="15" customHeight="1" s="32">
       <c r="A346" s="63" t="n">
@@ -24055,11 +23619,7 @@
         <f>IF(OR($J346="Attempted",$J346="Revisit"),"DUE",IF($N346="","",IF($N346&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P346" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P346" s="63" t="n"/>
     </row>
     <row r="347" ht="15" customHeight="1" s="32">
       <c r="A347" s="63" t="n">
@@ -24245,11 +23805,7 @@
         <f>IF(OR($J349="Attempted",$J349="Revisit"),"DUE",IF($N349="","",IF($N349&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P349" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P349" s="63" t="n"/>
     </row>
     <row r="350" ht="15" customHeight="1" s="32">
       <c r="A350" s="63" t="n">
@@ -24311,11 +23867,7 @@
         <f>IF(OR($J350="Attempted",$J350="Revisit"),"DUE",IF($N350="","",IF($N350&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P350" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P350" s="63" t="n"/>
     </row>
     <row r="351" ht="15" customHeight="1" s="32">
       <c r="A351" s="63" t="n">
@@ -24377,11 +23929,7 @@
         <f>IF(OR($J351="Attempted",$J351="Revisit"),"DUE",IF($N351="","",IF($N351&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P351" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P351" s="63" t="n"/>
     </row>
     <row r="352" ht="15" customHeight="1" s="32">
       <c r="A352" s="63" t="n">
@@ -24443,11 +23991,7 @@
         <f>IF(OR($J352="Attempted",$J352="Revisit"),"DUE",IF($N352="","",IF($N352&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P352" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P352" s="63" t="n"/>
     </row>
     <row r="353" ht="15" customHeight="1" s="32">
       <c r="A353" s="63" t="n">
@@ -24633,11 +24177,7 @@
         <f>IF(OR($J355="Attempted",$J355="Revisit"),"DUE",IF($N355="","",IF($N355&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P355" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P355" s="63" t="n"/>
     </row>
     <row r="356" ht="15" customHeight="1" s="32">
       <c r="A356" s="63" t="n">
@@ -24699,11 +24239,7 @@
         <f>IF(OR($J356="Attempted",$J356="Revisit"),"DUE",IF($N356="","",IF($N356&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P356" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P356" s="63" t="n"/>
     </row>
     <row r="357" ht="15" customHeight="1" s="32">
       <c r="A357" s="63" t="n">
@@ -24765,11 +24301,7 @@
         <f>IF(OR($J357="Attempted",$J357="Revisit"),"DUE",IF($N357="","",IF($N357&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P357" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P357" s="63" t="n"/>
     </row>
     <row r="358" ht="15" customHeight="1" s="32">
       <c r="A358" s="63" t="n">
@@ -25761,11 +25293,7 @@
         <f>IF(OR($J373="Attempted",$J373="Revisit"),"DUE",IF($N373="","",IF($N373&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P373" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P373" s="63" t="n"/>
     </row>
     <row r="374" ht="15" customHeight="1" s="32">
       <c r="A374" s="63" t="n">
@@ -26013,11 +25541,7 @@
         <f>IF(OR($J377="Attempted",$J377="Revisit"),"DUE",IF($N377="","",IF($N377&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P377" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P377" s="63" t="n"/>
     </row>
     <row r="378" ht="15" customHeight="1" s="32">
       <c r="A378" s="63" t="n">
@@ -26079,11 +25603,7 @@
         <f>IF(OR($J378="Attempted",$J378="Revisit"),"DUE",IF($N378="","",IF($N378&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P378" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P378" s="63" t="n"/>
     </row>
     <row r="379" ht="15" customHeight="1" s="32">
       <c r="A379" s="63" t="n">
@@ -26145,11 +25665,7 @@
         <f>IF(OR($J379="Attempted",$J379="Revisit"),"DUE",IF($N379="","",IF($N379&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P379" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P379" s="63" t="n"/>
     </row>
     <row r="380" ht="15" customHeight="1" s="32">
       <c r="A380" s="63" t="n">
@@ -26211,11 +25727,7 @@
         <f>IF(OR($J380="Attempted",$J380="Revisit"),"DUE",IF($N380="","",IF($N380&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P380" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P380" s="63" t="n"/>
     </row>
     <row r="381" ht="15" customHeight="1" s="32">
       <c r="A381" s="63" t="n">
@@ -26587,11 +26099,7 @@
         <f>IF(OR($J386="Attempted",$J386="Revisit"),"DUE",IF($N386="","",IF($N386&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P386" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P386" s="63" t="n"/>
     </row>
     <row r="387" ht="15" customHeight="1" s="32">
       <c r="A387" s="63" t="n">
@@ -26653,11 +26161,7 @@
         <f>IF(OR($J387="Attempted",$J387="Revisit"),"DUE",IF($N387="","",IF($N387&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P387" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P387" s="63" t="n"/>
     </row>
     <row r="388" ht="15" customHeight="1" s="32">
       <c r="A388" s="63" t="n">
@@ -26719,11 +26223,7 @@
         <f>IF(OR($J388="Attempted",$J388="Revisit"),"DUE",IF($N388="","",IF($N388&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P388" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P388" s="63" t="n"/>
     </row>
     <row r="389" ht="15" customHeight="1" s="32">
       <c r="A389" s="63" t="n">
@@ -26909,11 +26409,7 @@
         <f>IF(OR($J391="Attempted",$J391="Revisit"),"DUE",IF($N391="","",IF($N391&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P391" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P391" s="63" t="n"/>
     </row>
     <row r="392" ht="15" customHeight="1" s="32">
       <c r="A392" s="63" t="n">
@@ -27161,11 +26657,7 @@
         <f>IF(OR($J395="Attempted",$J395="Revisit"),"DUE",IF($N395="","",IF($N395&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P395" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P395" s="63" t="n"/>
     </row>
     <row r="396" ht="15" customHeight="1" s="32">
       <c r="A396" s="63" t="n">
@@ -27413,11 +26905,7 @@
         <f>IF(OR($J399="Attempted",$J399="Revisit"),"DUE",IF($N399="","",IF($N399&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P399" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P399" s="63" t="n"/>
     </row>
     <row r="400" ht="15" customHeight="1" s="32">
       <c r="A400" s="63" t="n">
@@ -27479,11 +26967,7 @@
         <f>IF(OR($J400="Attempted",$J400="Revisit"),"DUE",IF($N400="","",IF($N400&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P400" s="63" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P400" s="63" t="n"/>
     </row>
     <row r="401" ht="15" customHeight="1" s="32">
       <c r="A401" s="63" t="n">
@@ -27793,11 +27277,7 @@
         <f>IF(OR($J405="Attempted",$J405="Revisit"),"DUE",IF($N405="","",IF($N405&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P405" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P405" s="64" t="n"/>
     </row>
     <row r="406" ht="15" customHeight="1" s="32">
       <c r="A406" s="64" t="n">
@@ -27983,11 +27463,7 @@
         <f>IF(OR($J408="Attempted",$J408="Revisit"),"DUE",IF($N408="","",IF($N408&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P408" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P408" s="64" t="n"/>
     </row>
     <row r="409" ht="15" customHeight="1" s="32">
       <c r="A409" s="64" t="n">
@@ -28111,11 +27587,7 @@
         <f>IF(OR($J410="Attempted",$J410="Revisit"),"DUE",IF($N410="","",IF($N410&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P410" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P410" s="64" t="n"/>
     </row>
     <row r="411" ht="15" customHeight="1" s="32">
       <c r="A411" s="64" t="n">
@@ -28177,11 +27649,7 @@
         <f>IF(OR($J411="Attempted",$J411="Revisit"),"DUE",IF($N411="","",IF($N411&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P411" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P411" s="64" t="n"/>
     </row>
     <row r="412" ht="15" customHeight="1" s="32">
       <c r="A412" s="64" t="n">
@@ -28243,11 +27711,7 @@
         <f>IF(OR($J412="Attempted",$J412="Revisit"),"DUE",IF($N412="","",IF($N412&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P412" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P412" s="64" t="n"/>
     </row>
     <row r="413" ht="15" customHeight="1" s="32">
       <c r="A413" s="64" t="n">
@@ -28371,11 +27835,7 @@
         <f>IF(OR($J414="Attempted",$J414="Revisit"),"DUE",IF($N414="","",IF($N414&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P414" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P414" s="64" t="n"/>
     </row>
     <row r="415" ht="15" customHeight="1" s="32">
       <c r="A415" s="64" t="n">
@@ -28437,11 +27897,7 @@
         <f>IF(OR($J415="Attempted",$J415="Revisit"),"DUE",IF($N415="","",IF($N415&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P415" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P415" s="64" t="n"/>
     </row>
     <row r="416" ht="15" customHeight="1" s="32">
       <c r="A416" s="64" t="n">
@@ -28627,11 +28083,7 @@
         <f>IF(OR($J418="Attempted",$J418="Revisit"),"DUE",IF($N418="","",IF($N418&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P418" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P418" s="64" t="n"/>
     </row>
     <row r="419" ht="15" customHeight="1" s="32">
       <c r="A419" s="64" t="n">
@@ -28693,11 +28145,7 @@
         <f>IF(OR($J419="Attempted",$J419="Revisit"),"DUE",IF($N419="","",IF($N419&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P419" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P419" s="64" t="n"/>
     </row>
     <row r="420" ht="15" customHeight="1" s="32">
       <c r="A420" s="64" t="n">
@@ -30247,11 +29695,7 @@
         <f>IF(OR($J444="Attempted",$J444="Revisit"),"DUE",IF($N444="","",IF($N444&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P444" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P444" s="64" t="n"/>
     </row>
     <row r="445" ht="15" customHeight="1" s="32">
       <c r="A445" s="64" t="n">
@@ -30313,11 +29757,7 @@
         <f>IF(OR($J445="Attempted",$J445="Revisit"),"DUE",IF($N445="","",IF($N445&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P445" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P445" s="64" t="n"/>
     </row>
     <row r="446" ht="15" customHeight="1" s="32">
       <c r="A446" s="64" t="n">
@@ -30379,11 +29819,7 @@
         <f>IF(OR($J446="Attempted",$J446="Revisit"),"DUE",IF($N446="","",IF($N446&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P446" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P446" s="64" t="n"/>
     </row>
     <row r="447" ht="15" customHeight="1" s="32">
       <c r="A447" s="64" t="n">
@@ -30507,11 +29943,7 @@
         <f>IF(OR($J448="Attempted",$J448="Revisit"),"DUE",IF($N448="","",IF($N448&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P448" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P448" s="64" t="n"/>
     </row>
     <row r="449" ht="15" customHeight="1" s="32">
       <c r="A449" s="64" t="n">
@@ -30573,11 +30005,7 @@
         <f>IF(OR($J449="Attempted",$J449="Revisit"),"DUE",IF($N449="","",IF($N449&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P449" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P449" s="64" t="n"/>
     </row>
     <row r="450" ht="15" customHeight="1" s="32">
       <c r="A450" s="64" t="n">
@@ -30639,11 +30067,7 @@
         <f>IF(OR($J450="Attempted",$J450="Revisit"),"DUE",IF($N450="","",IF($N450&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P450" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P450" s="64" t="n"/>
     </row>
     <row r="451" ht="15" customHeight="1" s="32">
       <c r="A451" s="64" t="n">
@@ -30705,11 +30129,7 @@
         <f>IF(OR($J451="Attempted",$J451="Revisit"),"DUE",IF($N451="","",IF($N451&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P451" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P451" s="64" t="n"/>
     </row>
     <row r="452" ht="15" customHeight="1" s="32">
       <c r="A452" s="64" t="n">
@@ -30771,11 +30191,7 @@
         <f>IF(OR($J452="Attempted",$J452="Revisit"),"DUE",IF($N452="","",IF($N452&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P452" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P452" s="64" t="n"/>
     </row>
     <row r="453" ht="15" customHeight="1" s="32">
       <c r="A453" s="64" t="n">
@@ -30837,11 +30253,7 @@
         <f>IF(OR($J453="Attempted",$J453="Revisit"),"DUE",IF($N453="","",IF($N453&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P453" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P453" s="64" t="n"/>
     </row>
     <row r="454" ht="15" customHeight="1" s="32">
       <c r="A454" s="64" t="n">
@@ -30903,11 +30315,7 @@
         <f>IF(OR($J454="Attempted",$J454="Revisit"),"DUE",IF($N454="","",IF($N454&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P454" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P454" s="64" t="n"/>
     </row>
     <row r="455" ht="15" customHeight="1" s="32">
       <c r="A455" s="64" t="n">
@@ -30969,11 +30377,7 @@
         <f>IF(OR($J455="Attempted",$J455="Revisit"),"DUE",IF($N455="","",IF($N455&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P455" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P455" s="64" t="n"/>
     </row>
     <row r="456" ht="15" customHeight="1" s="32">
       <c r="A456" s="64" t="n">
@@ -31035,11 +30439,7 @@
         <f>IF(OR($J456="Attempted",$J456="Revisit"),"DUE",IF($N456="","",IF($N456&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P456" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P456" s="64" t="n"/>
     </row>
     <row r="457" ht="15" customHeight="1" s="32">
       <c r="A457" s="64" t="n">
@@ -31101,11 +30501,7 @@
         <f>IF(OR($J457="Attempted",$J457="Revisit"),"DUE",IF($N457="","",IF($N457&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P457" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P457" s="64" t="n"/>
     </row>
     <row r="458" ht="15" customHeight="1" s="32">
       <c r="A458" s="64" t="n">
@@ -31167,11 +30563,7 @@
         <f>IF(OR($J458="Attempted",$J458="Revisit"),"DUE",IF($N458="","",IF($N458&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P458" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P458" s="64" t="n"/>
     </row>
     <row r="459" ht="15" customHeight="1" s="32">
       <c r="A459" s="64" t="n">
@@ -31419,11 +30811,7 @@
         <f>IF(OR($J462="Attempted",$J462="Revisit"),"DUE",IF($N462="","",IF($N462&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P462" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P462" s="64" t="n"/>
     </row>
     <row r="463" ht="15" customHeight="1" s="32">
       <c r="A463" s="64" t="n">
@@ -31485,11 +30873,7 @@
         <f>IF(OR($J463="Attempted",$J463="Revisit"),"DUE",IF($N463="","",IF($N463&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P463" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P463" s="64" t="n"/>
     </row>
     <row r="464" ht="15" customHeight="1" s="32">
       <c r="A464" s="64" t="n">
@@ -31551,11 +30935,7 @@
         <f>IF(OR($J464="Attempted",$J464="Revisit"),"DUE",IF($N464="","",IF($N464&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P464" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P464" s="64" t="n"/>
     </row>
     <row r="465" ht="15" customHeight="1" s="32">
       <c r="A465" s="64" t="n">
@@ -31617,11 +30997,7 @@
         <f>IF(OR($J465="Attempted",$J465="Revisit"),"DUE",IF($N465="","",IF($N465&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P465" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P465" s="64" t="n"/>
     </row>
     <row r="466" ht="15" customHeight="1" s="32">
       <c r="A466" s="64" t="n">
@@ -31683,11 +31059,7 @@
         <f>IF(OR($J466="Attempted",$J466="Revisit"),"DUE",IF($N466="","",IF($N466&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P466" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P466" s="64" t="n"/>
     </row>
     <row r="467" ht="15" customHeight="1" s="32">
       <c r="A467" s="64" t="n">
@@ -31811,11 +31183,7 @@
         <f>IF(OR($J468="Attempted",$J468="Revisit"),"DUE",IF($N468="","",IF($N468&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P468" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P468" s="64" t="n"/>
     </row>
     <row r="469" ht="15" customHeight="1" s="32">
       <c r="A469" s="64" t="n">
@@ -31877,11 +31245,7 @@
         <f>IF(OR($J469="Attempted",$J469="Revisit"),"DUE",IF($N469="","",IF($N469&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P469" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P469" s="64" t="n"/>
     </row>
     <row r="470" ht="15" customHeight="1" s="32">
       <c r="A470" s="64" t="n">
@@ -31943,11 +31307,7 @@
         <f>IF(OR($J470="Attempted",$J470="Revisit"),"DUE",IF($N470="","",IF($N470&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P470" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P470" s="64" t="n"/>
     </row>
     <row r="471" ht="15" customHeight="1" s="32">
       <c r="A471" s="64" t="n">
@@ -32009,11 +31369,7 @@
         <f>IF(OR($J471="Attempted",$J471="Revisit"),"DUE",IF($N471="","",IF($N471&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P471" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P471" s="64" t="n"/>
     </row>
     <row r="472" ht="15" customHeight="1" s="32">
       <c r="A472" s="64" t="n">
@@ -32261,11 +31617,7 @@
         <f>IF(OR($J475="Attempted",$J475="Revisit"),"DUE",IF($N475="","",IF($N475&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P475" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P475" s="64" t="n"/>
     </row>
     <row r="476" ht="15" customHeight="1" s="32">
       <c r="A476" s="64" t="n">
@@ -32327,11 +31679,7 @@
         <f>IF(OR($J476="Attempted",$J476="Revisit"),"DUE",IF($N476="","",IF($N476&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P476" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P476" s="64" t="n"/>
     </row>
     <row r="477" ht="15" customHeight="1" s="32">
       <c r="A477" s="64" t="n">
@@ -32393,11 +31741,7 @@
         <f>IF(OR($J477="Attempted",$J477="Revisit"),"DUE",IF($N477="","",IF($N477&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P477" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P477" s="64" t="n"/>
     </row>
     <row r="478" ht="15" customHeight="1" s="32">
       <c r="A478" s="64" t="n">
@@ -32459,11 +31803,7 @@
         <f>IF(OR($J478="Attempted",$J478="Revisit"),"DUE",IF($N478="","",IF($N478&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P478" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P478" s="64" t="n"/>
     </row>
     <row r="479" ht="15" customHeight="1" s="32">
       <c r="A479" s="64" t="n">
@@ -32525,11 +31865,7 @@
         <f>IF(OR($J479="Attempted",$J479="Revisit"),"DUE",IF($N479="","",IF($N479&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P479" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P479" s="64" t="n"/>
     </row>
     <row r="480" ht="15" customHeight="1" s="32">
       <c r="A480" s="64" t="n">
@@ -32591,11 +31927,7 @@
         <f>IF(OR($J480="Attempted",$J480="Revisit"),"DUE",IF($N480="","",IF($N480&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P480" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P480" s="64" t="n"/>
     </row>
     <row r="481" ht="15" customHeight="1" s="32">
       <c r="A481" s="64" t="n">
@@ -32657,11 +31989,7 @@
         <f>IF(OR($J481="Attempted",$J481="Revisit"),"DUE",IF($N481="","",IF($N481&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P481" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P481" s="64" t="n"/>
     </row>
     <row r="482" ht="15" customHeight="1" s="32">
       <c r="A482" s="64" t="n">
@@ -32723,11 +32051,7 @@
         <f>IF(OR($J482="Attempted",$J482="Revisit"),"DUE",IF($N482="","",IF($N482&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P482" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P482" s="64" t="n"/>
     </row>
     <row r="483" ht="15" customHeight="1" s="32">
       <c r="A483" s="64" t="n">
@@ -32789,11 +32113,7 @@
         <f>IF(OR($J483="Attempted",$J483="Revisit"),"DUE",IF($N483="","",IF($N483&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P483" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P483" s="64" t="n"/>
     </row>
     <row r="484" ht="15" customHeight="1" s="32">
       <c r="A484" s="64" t="n">
@@ -32855,11 +32175,7 @@
         <f>IF(OR($J484="Attempted",$J484="Revisit"),"DUE",IF($N484="","",IF($N484&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P484" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P484" s="64" t="n"/>
     </row>
     <row r="485" ht="15" customHeight="1" s="32">
       <c r="A485" s="64" t="n">
@@ -32921,11 +32237,7 @@
         <f>IF(OR($J485="Attempted",$J485="Revisit"),"DUE",IF($N485="","",IF($N485&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P485" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P485" s="64" t="n"/>
     </row>
     <row r="486" ht="15" customHeight="1" s="32">
       <c r="A486" s="64" t="n">
@@ -32987,11 +32299,7 @@
         <f>IF(OR($J486="Attempted",$J486="Revisit"),"DUE",IF($N486="","",IF($N486&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P486" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P486" s="64" t="n"/>
     </row>
     <row r="487" ht="15" customHeight="1" s="32">
       <c r="A487" s="64" t="n">
@@ -33053,11 +32361,7 @@
         <f>IF(OR($J487="Attempted",$J487="Revisit"),"DUE",IF($N487="","",IF($N487&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P487" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P487" s="64" t="n"/>
     </row>
     <row r="488" ht="15" customHeight="1" s="32">
       <c r="A488" s="64" t="n">
@@ -33119,11 +32423,7 @@
         <f>IF(OR($J488="Attempted",$J488="Revisit"),"DUE",IF($N488="","",IF($N488&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P488" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P488" s="64" t="n"/>
     </row>
     <row r="489" ht="15" customHeight="1" s="32">
       <c r="A489" s="64" t="n">
@@ -33185,11 +32485,7 @@
         <f>IF(OR($J489="Attempted",$J489="Revisit"),"DUE",IF($N489="","",IF($N489&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P489" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P489" s="64" t="n"/>
     </row>
     <row r="490" ht="15" customHeight="1" s="32">
       <c r="A490" s="64" t="n">
@@ -33251,11 +32547,7 @@
         <f>IF(OR($J490="Attempted",$J490="Revisit"),"DUE",IF($N490="","",IF($N490&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P490" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P490" s="64" t="n"/>
     </row>
     <row r="491" ht="15" customHeight="1" s="32">
       <c r="A491" s="64" t="n">
@@ -33565,11 +32857,7 @@
         <f>IF(OR($J495="Attempted",$J495="Revisit"),"DUE",IF($N495="","",IF($N495&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P495" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P495" s="64" t="n"/>
     </row>
     <row r="496" ht="15" customHeight="1" s="32">
       <c r="A496" s="64" t="n">
@@ -33631,11 +32919,7 @@
         <f>IF(OR($J496="Attempted",$J496="Revisit"),"DUE",IF($N496="","",IF($N496&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P496" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P496" s="64" t="n"/>
     </row>
     <row r="497" ht="15" customHeight="1" s="32">
       <c r="A497" s="64" t="n">
@@ -33697,11 +32981,7 @@
         <f>IF(OR($J497="Attempted",$J497="Revisit"),"DUE",IF($N497="","",IF($N497&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P497" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P497" s="64" t="n"/>
     </row>
     <row r="498" ht="15" customHeight="1" s="32">
       <c r="A498" s="64" t="n">
@@ -33763,11 +33043,7 @@
         <f>IF(OR($J498="Attempted",$J498="Revisit"),"DUE",IF($N498="","",IF($N498&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P498" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P498" s="64" t="n"/>
     </row>
     <row r="499" ht="15" customHeight="1" s="32">
       <c r="A499" s="64" t="n">
@@ -33829,11 +33105,7 @@
         <f>IF(OR($J499="Attempted",$J499="Revisit"),"DUE",IF($N499="","",IF($N499&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P499" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P499" s="64" t="n"/>
     </row>
     <row r="500" ht="15" customHeight="1" s="32">
       <c r="A500" s="64" t="n">
@@ -33895,11 +33167,7 @@
         <f>IF(OR($J500="Attempted",$J500="Revisit"),"DUE",IF($N500="","",IF($N500&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P500" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P500" s="64" t="n"/>
     </row>
     <row r="501" ht="15" customHeight="1" s="32">
       <c r="A501" s="64" t="n">
@@ -33961,11 +33229,7 @@
         <f>IF(OR($J501="Attempted",$J501="Revisit"),"DUE",IF($N501="","",IF($N501&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P501" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P501" s="64" t="n"/>
     </row>
     <row r="502" ht="15" customHeight="1" s="32">
       <c r="A502" s="64" t="n">
@@ -34027,11 +33291,7 @@
         <f>IF(OR($J502="Attempted",$J502="Revisit"),"DUE",IF($N502="","",IF($N502&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P502" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P502" s="64" t="n"/>
     </row>
     <row r="503" ht="15" customHeight="1" s="32">
       <c r="A503" s="64" t="n">
@@ -34093,11 +33353,7 @@
         <f>IF(OR($J503="Attempted",$J503="Revisit"),"DUE",IF($N503="","",IF($N503&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P503" s="64" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P503" s="64" t="n"/>
     </row>
     <row r="504" ht="15" customHeight="1" s="32">
       <c r="A504" s="65" t="n">
@@ -34283,11 +33539,7 @@
         <f>IF(OR($J506="Attempted",$J506="Revisit"),"DUE",IF($N506="","",IF($N506&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P506" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P506" s="65" t="n"/>
     </row>
     <row r="507" ht="15" customHeight="1" s="32">
       <c r="A507" s="65" t="n">
@@ -34473,11 +33725,7 @@
         <f>IF(OR($J509="Attempted",$J509="Revisit"),"DUE",IF($N509="","",IF($N509&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P509" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P509" s="65" t="n"/>
     </row>
     <row r="510" ht="15" customHeight="1" s="32">
       <c r="A510" s="65" t="n">
@@ -35283,11 +34531,7 @@
         <f>IF(OR($J522="Attempted",$J522="Revisit"),"DUE",IF($N522="","",IF($N522&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P522" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P522" s="65" t="n"/>
     </row>
     <row r="523" ht="15" customHeight="1" s="32">
       <c r="A523" s="65" t="n">
@@ -36031,11 +35275,7 @@
         <f>IF(OR($J534="Attempted",$J534="Revisit"),"DUE",IF($N534="","",IF($N534&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P534" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P534" s="65" t="n"/>
     </row>
     <row r="535" ht="15" customHeight="1" s="32">
       <c r="A535" s="65" t="n">
@@ -36345,11 +35585,7 @@
         <f>IF(OR($J539="Attempted",$J539="Revisit"),"DUE",IF($N539="","",IF($N539&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P539" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P539" s="65" t="n"/>
     </row>
     <row r="540" ht="15" customHeight="1" s="32">
       <c r="A540" s="65" t="n">
@@ -36411,11 +35647,7 @@
         <f>IF(OR($J540="Attempted",$J540="Revisit"),"DUE",IF($N540="","",IF($N540&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P540" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P540" s="65" t="n"/>
     </row>
     <row r="541" ht="15" customHeight="1" s="32">
       <c r="A541" s="65" t="n">
@@ -36477,11 +35709,7 @@
         <f>IF(OR($J541="Attempted",$J541="Revisit"),"DUE",IF($N541="","",IF($N541&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P541" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P541" s="65" t="n"/>
     </row>
     <row r="542" ht="15" customHeight="1" s="32">
       <c r="A542" s="65" t="n">
@@ -36543,11 +35771,7 @@
         <f>IF(OR($J542="Attempted",$J542="Revisit"),"DUE",IF($N542="","",IF($N542&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P542" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P542" s="65" t="n"/>
     </row>
     <row r="543" ht="15" customHeight="1" s="32">
       <c r="A543" s="65" t="n">
@@ -36733,11 +35957,7 @@
         <f>IF(OR($J545="Attempted",$J545="Revisit"),"DUE",IF($N545="","",IF($N545&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P545" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P545" s="65" t="n"/>
     </row>
     <row r="546" ht="15" customHeight="1" s="32">
       <c r="A546" s="65" t="n">
@@ -39713,11 +38933,7 @@
         <f>IF(OR($J593="Attempted",$J593="Revisit"),"DUE",IF($N593="","",IF($N593&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P593" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P593" s="65" t="n"/>
     </row>
     <row r="594">
       <c r="A594" s="65" t="n">
@@ -39841,11 +39057,7 @@
         <f>IF(OR($J595="Attempted",$J595="Revisit"),"DUE",IF($N595="","",IF($N595&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P595" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P595" s="65" t="n"/>
     </row>
     <row r="596">
       <c r="A596" s="65" t="n">
@@ -39907,11 +39119,7 @@
         <f>IF(OR($J596="Attempted",$J596="Revisit"),"DUE",IF($N596="","",IF($N596&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P596" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P596" s="65" t="n"/>
     </row>
     <row r="597">
       <c r="A597" s="65" t="n">
@@ -39973,11 +39181,7 @@
         <f>IF(OR($J597="Attempted",$J597="Revisit"),"DUE",IF($N597="","",IF($N597&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P597" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P597" s="65" t="n"/>
     </row>
     <row r="598">
       <c r="A598" s="65" t="n">
@@ -40039,11 +39243,7 @@
         <f>IF(OR($J598="Attempted",$J598="Revisit"),"DUE",IF($N598="","",IF($N598&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P598" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P598" s="65" t="n"/>
     </row>
     <row r="599">
       <c r="A599" s="65" t="n">
@@ -40105,11 +39305,7 @@
         <f>IF(OR($J599="Attempted",$J599="Revisit"),"DUE",IF($N599="","",IF($N599&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P599" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P599" s="65" t="n"/>
     </row>
     <row r="600">
       <c r="A600" s="65" t="n">
@@ -40171,11 +39367,7 @@
         <f>IF(OR($J600="Attempted",$J600="Revisit"),"DUE",IF($N600="","",IF($N600&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P600" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P600" s="65" t="n"/>
     </row>
     <row r="601">
       <c r="A601" s="65" t="n">
@@ -40237,11 +39429,7 @@
         <f>IF(OR($J601="Attempted",$J601="Revisit"),"DUE",IF($N601="","",IF($N601&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P601" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P601" s="65" t="n"/>
     </row>
     <row r="602">
       <c r="A602" s="65" t="n">
@@ -40303,11 +39491,7 @@
         <f>IF(OR($J602="Attempted",$J602="Revisit"),"DUE",IF($N602="","",IF($N602&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P602" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P602" s="65" t="n"/>
     </row>
     <row r="603">
       <c r="A603" s="65" t="n">
@@ -40493,11 +39677,7 @@
         <f>IF(OR($J605="Attempted",$J605="Revisit"),"DUE",IF($N605="","",IF($N605&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P605" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P605" s="65" t="n"/>
     </row>
     <row r="606">
       <c r="A606" s="65" t="n">
@@ -40993,11 +40173,7 @@
         <f>IF(OR($J613="Attempted",$J613="Revisit"),"DUE",IF($N613="","",IF($N613&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P613" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P613" s="65" t="n"/>
     </row>
     <row r="614">
       <c r="A614" s="65" t="n">
@@ -41059,11 +40235,7 @@
         <f>IF(OR($J614="Attempted",$J614="Revisit"),"DUE",IF($N614="","",IF($N614&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P614" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P614" s="65" t="n"/>
     </row>
     <row r="615">
       <c r="A615" s="65" t="n">
@@ -41125,11 +40297,7 @@
         <f>IF(OR($J615="Attempted",$J615="Revisit"),"DUE",IF($N615="","",IF($N615&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P615" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P615" s="65" t="n"/>
     </row>
     <row r="616">
       <c r="A616" s="65" t="n">
@@ -41191,11 +40359,7 @@
         <f>IF(OR($J616="Attempted",$J616="Revisit"),"DUE",IF($N616="","",IF($N616&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P616" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P616" s="65" t="n"/>
     </row>
     <row r="617">
       <c r="A617" s="65" t="n">
@@ -41257,11 +40421,7 @@
         <f>IF(OR($J617="Attempted",$J617="Revisit"),"DUE",IF($N617="","",IF($N617&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P617" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P617" s="65" t="n"/>
     </row>
     <row r="618">
       <c r="A618" s="65" t="n">
@@ -41323,11 +40483,7 @@
         <f>IF(OR($J618="Attempted",$J618="Revisit"),"DUE",IF($N618="","",IF($N618&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P618" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P618" s="65" t="n"/>
     </row>
     <row r="619">
       <c r="A619" s="65" t="n">
@@ -41451,11 +40607,7 @@
         <f>IF(OR($J620="Attempted",$J620="Revisit"),"DUE",IF($N620="","",IF($N620&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P620" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P620" s="65" t="n"/>
     </row>
     <row r="621">
       <c r="A621" s="65" t="n">
@@ -41827,11 +40979,7 @@
         <f>IF(OR($J626="Attempted",$J626="Revisit"),"DUE",IF($N626="","",IF($N626&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P626" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P626" s="65" t="n"/>
     </row>
     <row r="627">
       <c r="A627" s="65" t="n">
@@ -41893,11 +41041,7 @@
         <f>IF(OR($J627="Attempted",$J627="Revisit"),"DUE",IF($N627="","",IF($N627&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P627" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P627" s="65" t="n"/>
     </row>
     <row r="628">
       <c r="A628" s="65" t="n">
@@ -41959,11 +41103,7 @@
         <f>IF(OR($J628="Attempted",$J628="Revisit"),"DUE",IF($N628="","",IF($N628&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P628" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P628" s="65" t="n"/>
     </row>
     <row r="629">
       <c r="A629" s="65" t="n">
@@ -42025,11 +41165,7 @@
         <f>IF(OR($J629="Attempted",$J629="Revisit"),"DUE",IF($N629="","",IF($N629&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P629" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P629" s="65" t="n"/>
     </row>
     <row r="630">
       <c r="A630" s="65" t="n">
@@ -42091,11 +41227,7 @@
         <f>IF(OR($J630="Attempted",$J630="Revisit"),"DUE",IF($N630="","",IF($N630&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P630" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P630" s="65" t="n"/>
     </row>
     <row r="631">
       <c r="A631" s="65" t="n">
@@ -42157,11 +41289,7 @@
         <f>IF(OR($J631="Attempted",$J631="Revisit"),"DUE",IF($N631="","",IF($N631&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P631" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P631" s="65" t="n"/>
     </row>
     <row r="632">
       <c r="A632" s="65" t="n">
@@ -42223,11 +41351,7 @@
         <f>IF(OR($J632="Attempted",$J632="Revisit"),"DUE",IF($N632="","",IF($N632&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P632" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P632" s="65" t="n"/>
     </row>
     <row r="633">
       <c r="A633" s="65" t="n">
@@ -42289,11 +41413,7 @@
         <f>IF(OR($J633="Attempted",$J633="Revisit"),"DUE",IF($N633="","",IF($N633&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P633" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P633" s="65" t="n"/>
     </row>
     <row r="634">
       <c r="A634" s="65" t="n">
@@ -42355,11 +41475,7 @@
         <f>IF(OR($J634="Attempted",$J634="Revisit"),"DUE",IF($N634="","",IF($N634&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P634" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P634" s="65" t="n"/>
     </row>
     <row r="635">
       <c r="A635" s="65" t="n">
@@ -42421,11 +41537,7 @@
         <f>IF(OR($J635="Attempted",$J635="Revisit"),"DUE",IF($N635="","",IF($N635&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P635" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P635" s="65" t="n"/>
     </row>
     <row r="636">
       <c r="A636" s="65" t="n">
@@ -42611,11 +41723,7 @@
         <f>IF(OR($J638="Attempted",$J638="Revisit"),"DUE",IF($N638="","",IF($N638&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P638" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P638" s="65" t="n"/>
     </row>
     <row r="639">
       <c r="A639" s="65" t="n">
@@ -42677,11 +41785,7 @@
         <f>IF(OR($J639="Attempted",$J639="Revisit"),"DUE",IF($N639="","",IF($N639&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P639" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P639" s="65" t="n"/>
     </row>
     <row r="640">
       <c r="A640" s="65" t="n">
@@ -43363,11 +42467,7 @@
         <f>IF(OR($J650="Attempted",$J650="Revisit"),"DUE",IF($N650="","",IF($N650&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P650" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P650" s="65" t="n"/>
     </row>
     <row r="651">
       <c r="A651" s="65" t="n">
@@ -43429,11 +42529,7 @@
         <f>IF(OR($J651="Attempted",$J651="Revisit"),"DUE",IF($N651="","",IF($N651&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P651" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P651" s="65" t="n"/>
     </row>
     <row r="652">
       <c r="A652" s="65" t="n">
@@ -43495,11 +42591,7 @@
         <f>IF(OR($J652="Attempted",$J652="Revisit"),"DUE",IF($N652="","",IF($N652&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P652" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P652" s="65" t="n"/>
     </row>
     <row r="653">
       <c r="A653" s="65" t="n">
@@ -43561,11 +42653,7 @@
         <f>IF(OR($J653="Attempted",$J653="Revisit"),"DUE",IF($N653="","",IF($N653&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P653" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P653" s="65" t="n"/>
     </row>
     <row r="654">
       <c r="A654" s="65" t="n">
@@ -43627,11 +42715,7 @@
         <f>IF(OR($J654="Attempted",$J654="Revisit"),"DUE",IF($N654="","",IF($N654&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P654" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P654" s="65" t="n"/>
     </row>
     <row r="655">
       <c r="A655" s="65" t="n">
@@ -43755,11 +42839,7 @@
         <f>IF(OR($J656="Attempted",$J656="Revisit"),"DUE",IF($N656="","",IF($N656&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P656" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P656" s="65" t="n"/>
     </row>
     <row r="657">
       <c r="A657" s="65" t="n">
@@ -43821,11 +42901,7 @@
         <f>IF(OR($J657="Attempted",$J657="Revisit"),"DUE",IF($N657="","",IF($N657&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P657" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P657" s="65" t="n"/>
     </row>
     <row r="658">
       <c r="A658" s="65" t="n">
@@ -43887,11 +42963,7 @@
         <f>IF(OR($J658="Attempted",$J658="Revisit"),"DUE",IF($N658="","",IF($N658&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P658" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P658" s="65" t="n"/>
     </row>
     <row r="659">
       <c r="A659" s="65" t="n">
@@ -43953,11 +43025,7 @@
         <f>IF(OR($J659="Attempted",$J659="Revisit"),"DUE",IF($N659="","",IF($N659&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P659" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P659" s="65" t="n"/>
     </row>
     <row r="660">
       <c r="A660" s="65" t="n">
@@ -44019,11 +43087,7 @@
         <f>IF(OR($J660="Attempted",$J660="Revisit"),"DUE",IF($N660="","",IF($N660&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P660" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P660" s="65" t="n"/>
     </row>
     <row r="661">
       <c r="A661" s="65" t="n">
@@ -44085,11 +43149,7 @@
         <f>IF(OR($J661="Attempted",$J661="Revisit"),"DUE",IF($N661="","",IF($N661&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P661" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P661" s="65" t="n"/>
     </row>
     <row r="662">
       <c r="A662" s="65" t="n">
@@ -44151,11 +43211,7 @@
         <f>IF(OR($J662="Attempted",$J662="Revisit"),"DUE",IF($N662="","",IF($N662&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P662" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P662" s="65" t="n"/>
     </row>
     <row r="663">
       <c r="A663" s="65" t="n">
@@ -44403,11 +43459,7 @@
         <f>IF(OR($J666="Attempted",$J666="Revisit"),"DUE",IF($N666="","",IF($N666&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P666" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P666" s="65" t="n"/>
     </row>
     <row r="667">
       <c r="A667" s="65" t="n">
@@ -44469,11 +43521,7 @@
         <f>IF(OR($J667="Attempted",$J667="Revisit"),"DUE",IF($N667="","",IF($N667&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P667" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P667" s="65" t="n"/>
     </row>
     <row r="668">
       <c r="A668" s="65" t="n">
@@ -44535,11 +43583,7 @@
         <f>IF(OR($J668="Attempted",$J668="Revisit"),"DUE",IF($N668="","",IF($N668&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P668" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P668" s="65" t="n"/>
     </row>
     <row r="669">
       <c r="A669" s="65" t="n">
@@ -44601,11 +43645,7 @@
         <f>IF(OR($J669="Attempted",$J669="Revisit"),"DUE",IF($N669="","",IF($N669&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P669" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P669" s="65" t="n"/>
     </row>
     <row r="670">
       <c r="A670" s="65" t="n">
@@ -44667,11 +43707,7 @@
         <f>IF(OR($J670="Attempted",$J670="Revisit"),"DUE",IF($N670="","",IF($N670&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P670" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P670" s="65" t="n"/>
     </row>
     <row r="671">
       <c r="A671" s="65" t="n">
@@ -44733,11 +43769,7 @@
         <f>IF(OR($J671="Attempted",$J671="Revisit"),"DUE",IF($N671="","",IF($N671&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P671" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P671" s="65" t="n"/>
     </row>
     <row r="672">
       <c r="A672" s="65" t="n">
@@ -44799,11 +43831,7 @@
         <f>IF(OR($J672="Attempted",$J672="Revisit"),"DUE",IF($N672="","",IF($N672&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P672" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P672" s="65" t="n"/>
     </row>
     <row r="673">
       <c r="A673" s="65" t="n">
@@ -44865,11 +43893,7 @@
         <f>IF(OR($J673="Attempted",$J673="Revisit"),"DUE",IF($N673="","",IF($N673&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P673" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P673" s="65" t="n"/>
     </row>
     <row r="674">
       <c r="A674" s="65" t="n">
@@ -44931,11 +43955,7 @@
         <f>IF(OR($J674="Attempted",$J674="Revisit"),"DUE",IF($N674="","",IF($N674&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P674" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P674" s="65" t="n"/>
     </row>
     <row r="675">
       <c r="A675" s="65" t="n">
@@ -44997,11 +44017,7 @@
         <f>IF(OR($J675="Attempted",$J675="Revisit"),"DUE",IF($N675="","",IF($N675&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P675" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P675" s="65" t="n"/>
     </row>
     <row r="676">
       <c r="A676" s="65" t="n">
@@ -45063,11 +44079,7 @@
         <f>IF(OR($J676="Attempted",$J676="Revisit"),"DUE",IF($N676="","",IF($N676&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P676" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P676" s="65" t="n"/>
     </row>
     <row r="677">
       <c r="A677" s="65" t="n">
@@ -45253,11 +44265,7 @@
         <f>IF(OR($J679="Attempted",$J679="Revisit"),"DUE",IF($N679="","",IF($N679&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P679" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P679" s="65" t="n"/>
     </row>
     <row r="680">
       <c r="A680" s="65" t="n">
@@ -45319,11 +44327,7 @@
         <f>IF(OR($J680="Attempted",$J680="Revisit"),"DUE",IF($N680="","",IF($N680&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P680" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P680" s="65" t="n"/>
     </row>
     <row r="681">
       <c r="A681" s="65" t="n">
@@ -45385,11 +44389,7 @@
         <f>IF(OR($J681="Attempted",$J681="Revisit"),"DUE",IF($N681="","",IF($N681&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P681" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P681" s="65" t="n"/>
     </row>
     <row r="682">
       <c r="A682" s="65" t="n">
@@ -45699,11 +44699,7 @@
         <f>IF(OR($J686="Attempted",$J686="Revisit"),"DUE",IF($N686="","",IF($N686&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P686" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P686" s="65" t="n"/>
     </row>
     <row r="687">
       <c r="A687" s="65" t="n">
@@ -45765,11 +44761,7 @@
         <f>IF(OR($J687="Attempted",$J687="Revisit"),"DUE",IF($N687="","",IF($N687&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P687" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P687" s="65" t="n"/>
     </row>
     <row r="688">
       <c r="A688" s="65" t="n">
@@ -45831,11 +44823,7 @@
         <f>IF(OR($J688="Attempted",$J688="Revisit"),"DUE",IF($N688="","",IF($N688&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P688" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P688" s="65" t="n"/>
     </row>
     <row r="689">
       <c r="A689" s="65" t="n">
@@ -45897,11 +44885,7 @@
         <f>IF(OR($J689="Attempted",$J689="Revisit"),"DUE",IF($N689="","",IF($N689&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P689" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P689" s="65" t="n"/>
     </row>
     <row r="690">
       <c r="A690" s="65" t="n">
@@ -45963,11 +44947,7 @@
         <f>IF(OR($J690="Attempted",$J690="Revisit"),"DUE",IF($N690="","",IF($N690&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P690" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P690" s="65" t="n"/>
     </row>
     <row r="691">
       <c r="A691" s="65" t="n">
@@ -46029,11 +45009,7 @@
         <f>IF(OR($J691="Attempted",$J691="Revisit"),"DUE",IF($N691="","",IF($N691&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P691" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P691" s="65" t="n"/>
     </row>
     <row r="692">
       <c r="A692" s="65" t="n">
@@ -46095,11 +45071,7 @@
         <f>IF(OR($J692="Attempted",$J692="Revisit"),"DUE",IF($N692="","",IF($N692&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P692" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P692" s="65" t="n"/>
     </row>
     <row r="693">
       <c r="A693" s="65" t="n">
@@ -46161,11 +45133,7 @@
         <f>IF(OR($J693="Attempted",$J693="Revisit"),"DUE",IF($N693="","",IF($N693&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P693" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P693" s="65" t="n"/>
     </row>
     <row r="694">
       <c r="A694" s="65" t="n">
@@ -46227,11 +45195,7 @@
         <f>IF(OR($J694="Attempted",$J694="Revisit"),"DUE",IF($N694="","",IF($N694&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P694" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P694" s="65" t="n"/>
     </row>
     <row r="695">
       <c r="A695" s="65" t="n">
@@ -46293,11 +45257,7 @@
         <f>IF(OR($J695="Attempted",$J695="Revisit"),"DUE",IF($N695="","",IF($N695&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P695" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P695" s="65" t="n"/>
     </row>
     <row r="696">
       <c r="A696" s="65" t="n">
@@ -46359,11 +45319,7 @@
         <f>IF(OR($J696="Attempted",$J696="Revisit"),"DUE",IF($N696="","",IF($N696&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P696" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P696" s="65" t="n"/>
     </row>
     <row r="697">
       <c r="A697" s="65" t="n">
@@ -46425,11 +45381,7 @@
         <f>IF(OR($J697="Attempted",$J697="Revisit"),"DUE",IF($N697="","",IF($N697&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P697" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P697" s="65" t="n"/>
     </row>
     <row r="698">
       <c r="A698" s="65" t="n">
@@ -46491,11 +45443,7 @@
         <f>IF(OR($J698="Attempted",$J698="Revisit"),"DUE",IF($N698="","",IF($N698&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P698" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P698" s="65" t="n"/>
     </row>
     <row r="699">
       <c r="A699" s="65" t="n">
@@ -46557,11 +45505,7 @@
         <f>IF(OR($J699="Attempted",$J699="Revisit"),"DUE",IF($N699="","",IF($N699&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P699" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P699" s="65" t="n"/>
     </row>
     <row r="700">
       <c r="A700" s="65" t="n">
@@ -46623,11 +45567,7 @@
         <f>IF(OR($J700="Attempted",$J700="Revisit"),"DUE",IF($N700="","",IF($N700&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P700" s="65" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P700" s="65" t="n"/>
     </row>
     <row r="701">
       <c r="A701" s="66" t="n">
@@ -47929,11 +46869,7 @@
         <f>IF(OR($J721="Attempted",$J721="Revisit"),"DUE",IF($N721="","",IF($N721&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P721" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P721" s="66" t="n"/>
     </row>
     <row r="722">
       <c r="A722" s="66" t="n">
@@ -48615,11 +47551,7 @@
         <f>IF(OR($J732="Attempted",$J732="Revisit"),"DUE",IF($N732="","",IF($N732&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P732" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P732" s="66" t="n"/>
     </row>
     <row r="733">
       <c r="A733" s="66" t="n">
@@ -48681,11 +47613,7 @@
         <f>IF(OR($J733="Attempted",$J733="Revisit"),"DUE",IF($N733="","",IF($N733&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P733" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P733" s="66" t="n"/>
     </row>
     <row r="734">
       <c r="A734" s="66" t="n">
@@ -48871,11 +47799,7 @@
         <f>IF(OR($J736="Attempted",$J736="Revisit"),"DUE",IF($N736="","",IF($N736&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P736" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P736" s="66" t="n"/>
     </row>
     <row r="737">
       <c r="A737" s="66" t="n">
@@ -48937,11 +47861,7 @@
         <f>IF(OR($J737="Attempted",$J737="Revisit"),"DUE",IF($N737="","",IF($N737&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P737" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P737" s="66" t="n"/>
     </row>
     <row r="738">
       <c r="A738" s="66" t="n">
@@ -49003,11 +47923,7 @@
         <f>IF(OR($J738="Attempted",$J738="Revisit"),"DUE",IF($N738="","",IF($N738&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P738" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P738" s="66" t="n"/>
     </row>
     <row r="739">
       <c r="A739" s="66" t="n">
@@ -49379,11 +48295,7 @@
         <f>IF(OR($J744="Attempted",$J744="Revisit"),"DUE",IF($N744="","",IF($N744&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P744" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P744" s="66" t="n"/>
     </row>
     <row r="745">
       <c r="A745" s="66" t="n">
@@ -49569,11 +48481,7 @@
         <f>IF(OR($J747="Attempted",$J747="Revisit"),"DUE",IF($N747="","",IF($N747&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P747" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P747" s="66" t="n"/>
     </row>
     <row r="748">
       <c r="A748" s="66" t="n">
@@ -49759,11 +48667,7 @@
         <f>IF(OR($J750="Attempted",$J750="Revisit"),"DUE",IF($N750="","",IF($N750&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P750" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P750" s="66" t="n"/>
     </row>
     <row r="751">
       <c r="A751" s="66" t="n">
@@ -49825,11 +48729,7 @@
         <f>IF(OR($J751="Attempted",$J751="Revisit"),"DUE",IF($N751="","",IF($N751&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P751" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P751" s="66" t="n"/>
     </row>
     <row r="752">
       <c r="A752" s="66" t="n">
@@ -50077,11 +48977,7 @@
         <f>IF(OR($J755="Attempted",$J755="Revisit"),"DUE",IF($N755="","",IF($N755&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P755" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P755" s="66" t="n"/>
     </row>
     <row r="756">
       <c r="A756" s="66" t="n">
@@ -50391,11 +49287,7 @@
         <f>IF(OR($J760="Attempted",$J760="Revisit"),"DUE",IF($N760="","",IF($N760&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P760" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P760" s="66" t="n"/>
     </row>
     <row r="761">
       <c r="A761" s="66" t="n">
@@ -50519,11 +49411,7 @@
         <f>IF(OR($J762="Attempted",$J762="Revisit"),"DUE",IF($N762="","",IF($N762&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P762" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P762" s="66" t="n"/>
     </row>
     <row r="763">
       <c r="A763" s="66" t="n">
@@ -51267,11 +50155,7 @@
         <f>IF(OR($J774="Attempted",$J774="Revisit"),"DUE",IF($N774="","",IF($N774&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P774" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P774" s="66" t="n"/>
     </row>
     <row r="775">
       <c r="A775" s="66" t="n">
@@ -53007,11 +51891,7 @@
         <f>IF(OR($J802="Attempted",$J802="Revisit"),"DUE",IF($N802="","",IF($N802&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P802" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P802" s="66" t="n"/>
     </row>
     <row r="803">
       <c r="A803" s="66" t="n">
@@ -53073,11 +51953,7 @@
         <f>IF(OR($J803="Attempted",$J803="Revisit"),"DUE",IF($N803="","",IF($N803&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P803" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P803" s="66" t="n"/>
     </row>
     <row r="804">
       <c r="A804" s="66" t="n">
@@ -53139,11 +52015,7 @@
         <f>IF(OR($J804="Attempted",$J804="Revisit"),"DUE",IF($N804="","",IF($N804&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P804" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P804" s="66" t="n"/>
     </row>
     <row r="805">
       <c r="A805" s="66" t="n">
@@ -53453,11 +52325,7 @@
         <f>IF(OR($J809="Attempted",$J809="Revisit"),"DUE",IF($N809="","",IF($N809&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P809" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P809" s="66" t="n"/>
     </row>
     <row r="810">
       <c r="A810" s="66" t="n">
@@ -53519,11 +52387,7 @@
         <f>IF(OR($J810="Attempted",$J810="Revisit"),"DUE",IF($N810="","",IF($N810&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P810" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P810" s="66" t="n"/>
     </row>
     <row r="811">
       <c r="A811" s="66" t="n">
@@ -53585,11 +52449,7 @@
         <f>IF(OR($J811="Attempted",$J811="Revisit"),"DUE",IF($N811="","",IF($N811&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P811" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P811" s="66" t="n"/>
     </row>
     <row r="812">
       <c r="A812" s="66" t="n">
@@ -53651,11 +52511,7 @@
         <f>IF(OR($J812="Attempted",$J812="Revisit"),"DUE",IF($N812="","",IF($N812&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P812" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P812" s="66" t="n"/>
     </row>
     <row r="813">
       <c r="A813" s="66" t="n">
@@ -54399,11 +53255,7 @@
         <f>IF(OR($J824="Attempted",$J824="Revisit"),"DUE",IF($N824="","",IF($N824&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P824" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P824" s="66" t="n"/>
     </row>
     <row r="825">
       <c r="A825" s="66" t="n">
@@ -54465,11 +53317,7 @@
         <f>IF(OR($J825="Attempted",$J825="Revisit"),"DUE",IF($N825="","",IF($N825&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P825" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P825" s="66" t="n"/>
     </row>
     <row r="826">
       <c r="A826" s="66" t="n">
@@ -54531,11 +53379,7 @@
         <f>IF(OR($J826="Attempted",$J826="Revisit"),"DUE",IF($N826="","",IF($N826&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P826" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P826" s="66" t="n"/>
     </row>
     <row r="827">
       <c r="A827" s="66" t="n">
@@ -54659,11 +53503,7 @@
         <f>IF(OR($J828="Attempted",$J828="Revisit"),"DUE",IF($N828="","",IF($N828&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P828" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P828" s="66" t="n"/>
     </row>
     <row r="829">
       <c r="A829" s="66" t="n">
@@ -54725,11 +53565,7 @@
         <f>IF(OR($J829="Attempted",$J829="Revisit"),"DUE",IF($N829="","",IF($N829&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P829" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P829" s="66" t="n"/>
     </row>
     <row r="830">
       <c r="A830" s="66" t="n">
@@ -54853,11 +53689,7 @@
         <f>IF(OR($J831="Attempted",$J831="Revisit"),"DUE",IF($N831="","",IF($N831&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P831" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P831" s="66" t="n"/>
     </row>
     <row r="832">
       <c r="A832" s="66" t="n">
@@ -54919,11 +53751,7 @@
         <f>IF(OR($J832="Attempted",$J832="Revisit"),"DUE",IF($N832="","",IF($N832&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P832" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P832" s="66" t="n"/>
     </row>
     <row r="833">
       <c r="A833" s="66" t="n">
@@ -54985,11 +53813,7 @@
         <f>IF(OR($J833="Attempted",$J833="Revisit"),"DUE",IF($N833="","",IF($N833&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P833" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P833" s="66" t="n"/>
     </row>
     <row r="834">
       <c r="A834" s="66" t="n">
@@ -55051,11 +53875,7 @@
         <f>IF(OR($J834="Attempted",$J834="Revisit"),"DUE",IF($N834="","",IF($N834&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P834" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P834" s="66" t="n"/>
     </row>
     <row r="835">
       <c r="A835" s="66" t="n">
@@ -55117,11 +53937,7 @@
         <f>IF(OR($J835="Attempted",$J835="Revisit"),"DUE",IF($N835="","",IF($N835&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P835" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P835" s="66" t="n"/>
     </row>
     <row r="836">
       <c r="A836" s="66" t="n">
@@ -55183,11 +53999,7 @@
         <f>IF(OR($J836="Attempted",$J836="Revisit"),"DUE",IF($N836="","",IF($N836&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P836" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P836" s="66" t="n"/>
     </row>
     <row r="837">
       <c r="A837" s="66" t="n">
@@ -55249,11 +54061,7 @@
         <f>IF(OR($J837="Attempted",$J837="Revisit"),"DUE",IF($N837="","",IF($N837&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P837" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P837" s="66" t="n"/>
     </row>
     <row r="838">
       <c r="A838" s="66" t="n">
@@ -55315,11 +54123,7 @@
         <f>IF(OR($J838="Attempted",$J838="Revisit"),"DUE",IF($N838="","",IF($N838&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P838" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P838" s="66" t="n"/>
     </row>
     <row r="839">
       <c r="A839" s="66" t="n">
@@ -55381,11 +54185,7 @@
         <f>IF(OR($J839="Attempted",$J839="Revisit"),"DUE",IF($N839="","",IF($N839&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P839" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P839" s="66" t="n"/>
     </row>
     <row r="840">
       <c r="A840" s="66" t="n">
@@ -55447,11 +54247,7 @@
         <f>IF(OR($J840="Attempted",$J840="Revisit"),"DUE",IF($N840="","",IF($N840&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P840" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P840" s="66" t="n"/>
     </row>
     <row r="841">
       <c r="A841" s="66" t="n">
@@ -55637,11 +54433,7 @@
         <f>IF(OR($J843="Attempted",$J843="Revisit"),"DUE",IF($N843="","",IF($N843&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P843" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P843" s="66" t="n"/>
     </row>
     <row r="844">
       <c r="A844" s="66" t="n">
@@ -55703,11 +54495,7 @@
         <f>IF(OR($J844="Attempted",$J844="Revisit"),"DUE",IF($N844="","",IF($N844&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P844" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P844" s="66" t="n"/>
     </row>
     <row r="845">
       <c r="A845" s="66" t="n">
@@ -55831,11 +54619,7 @@
         <f>IF(OR($J846="Attempted",$J846="Revisit"),"DUE",IF($N846="","",IF($N846&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P846" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P846" s="66" t="n"/>
     </row>
     <row r="847">
       <c r="A847" s="66" t="n">
@@ -55897,11 +54681,7 @@
         <f>IF(OR($J847="Attempted",$J847="Revisit"),"DUE",IF($N847="","",IF($N847&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P847" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P847" s="66" t="n"/>
     </row>
     <row r="848">
       <c r="A848" s="66" t="n">
@@ -55963,11 +54743,7 @@
         <f>IF(OR($J848="Attempted",$J848="Revisit"),"DUE",IF($N848="","",IF($N848&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P848" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P848" s="66" t="n"/>
     </row>
     <row r="849">
       <c r="A849" s="66" t="n">
@@ -56029,11 +54805,7 @@
         <f>IF(OR($J849="Attempted",$J849="Revisit"),"DUE",IF($N849="","",IF($N849&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P849" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P849" s="66" t="n"/>
     </row>
     <row r="850">
       <c r="A850" s="66" t="n">
@@ -56157,11 +54929,7 @@
         <f>IF(OR($J851="Attempted",$J851="Revisit"),"DUE",IF($N851="","",IF($N851&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P851" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P851" s="66" t="n"/>
     </row>
     <row r="852">
       <c r="A852" s="66" t="n">
@@ -56223,11 +54991,7 @@
         <f>IF(OR($J852="Attempted",$J852="Revisit"),"DUE",IF($N852="","",IF($N852&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P852" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P852" s="66" t="n"/>
     </row>
     <row r="853">
       <c r="A853" s="66" t="n">
@@ -56289,11 +55053,7 @@
         <f>IF(OR($J853="Attempted",$J853="Revisit"),"DUE",IF($N853="","",IF($N853&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P853" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P853" s="66" t="n"/>
     </row>
     <row r="854">
       <c r="A854" s="66" t="n">
@@ -56355,11 +55115,7 @@
         <f>IF(OR($J854="Attempted",$J854="Revisit"),"DUE",IF($N854="","",IF($N854&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P854" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P854" s="66" t="n"/>
     </row>
     <row r="855">
       <c r="A855" s="66" t="n">
@@ -56421,11 +55177,7 @@
         <f>IF(OR($J855="Attempted",$J855="Revisit"),"DUE",IF($N855="","",IF($N855&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P855" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P855" s="66" t="n"/>
     </row>
     <row r="856">
       <c r="A856" s="66" t="n">
@@ -56487,11 +55239,7 @@
         <f>IF(OR($J856="Attempted",$J856="Revisit"),"DUE",IF($N856="","",IF($N856&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P856" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P856" s="66" t="n"/>
     </row>
     <row r="857">
       <c r="A857" s="66" t="n">
@@ -56553,11 +55301,7 @@
         <f>IF(OR($J857="Attempted",$J857="Revisit"),"DUE",IF($N857="","",IF($N857&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P857" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P857" s="66" t="n"/>
     </row>
     <row r="858">
       <c r="A858" s="66" t="n">
@@ -56619,11 +55363,7 @@
         <f>IF(OR($J858="Attempted",$J858="Revisit"),"DUE",IF($N858="","",IF($N858&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P858" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P858" s="66" t="n"/>
     </row>
     <row r="859">
       <c r="A859" s="66" t="n">
@@ -56685,11 +55425,7 @@
         <f>IF(OR($J859="Attempted",$J859="Revisit"),"DUE",IF($N859="","",IF($N859&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P859" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P859" s="66" t="n"/>
     </row>
     <row r="860">
       <c r="A860" s="66" t="n">
@@ -56751,11 +55487,7 @@
         <f>IF(OR($J860="Attempted",$J860="Revisit"),"DUE",IF($N860="","",IF($N860&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P860" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P860" s="66" t="n"/>
     </row>
     <row r="861">
       <c r="A861" s="66" t="n">
@@ -56817,11 +55549,7 @@
         <f>IF(OR($J861="Attempted",$J861="Revisit"),"DUE",IF($N861="","",IF($N861&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P861" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P861" s="66" t="n"/>
     </row>
     <row r="862">
       <c r="A862" s="66" t="n">
@@ -56883,11 +55611,7 @@
         <f>IF(OR($J862="Attempted",$J862="Revisit"),"DUE",IF($N862="","",IF($N862&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P862" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P862" s="66" t="n"/>
     </row>
     <row r="863">
       <c r="A863" s="66" t="n">
@@ -57941,11 +56665,7 @@
         <f>IF(OR($J879="Attempted",$J879="Revisit"),"DUE",IF($N879="","",IF($N879&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P879" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P879" s="66" t="n"/>
     </row>
     <row r="880">
       <c r="A880" s="66" t="n">
@@ -58007,11 +56727,7 @@
         <f>IF(OR($J880="Attempted",$J880="Revisit"),"DUE",IF($N880="","",IF($N880&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P880" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P880" s="66" t="n"/>
     </row>
     <row r="881">
       <c r="A881" s="66" t="n">
@@ -58073,11 +56789,7 @@
         <f>IF(OR($J881="Attempted",$J881="Revisit"),"DUE",IF($N881="","",IF($N881&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P881" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P881" s="66" t="n"/>
     </row>
     <row r="882">
       <c r="A882" s="66" t="n">
@@ -58139,11 +56851,7 @@
         <f>IF(OR($J882="Attempted",$J882="Revisit"),"DUE",IF($N882="","",IF($N882&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P882" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P882" s="66" t="n"/>
     </row>
     <row r="883">
       <c r="A883" s="66" t="n">
@@ -58205,11 +56913,7 @@
         <f>IF(OR($J883="Attempted",$J883="Revisit"),"DUE",IF($N883="","",IF($N883&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P883" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P883" s="66" t="n"/>
     </row>
     <row r="884">
       <c r="A884" s="66" t="n">
@@ -58271,11 +56975,7 @@
         <f>IF(OR($J884="Attempted",$J884="Revisit"),"DUE",IF($N884="","",IF($N884&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P884" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P884" s="66" t="n"/>
     </row>
     <row r="885">
       <c r="A885" s="66" t="n">
@@ -58337,11 +57037,7 @@
         <f>IF(OR($J885="Attempted",$J885="Revisit"),"DUE",IF($N885="","",IF($N885&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P885" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P885" s="66" t="n"/>
     </row>
     <row r="886">
       <c r="A886" s="66" t="n">
@@ -58403,11 +57099,7 @@
         <f>IF(OR($J886="Attempted",$J886="Revisit"),"DUE",IF($N886="","",IF($N886&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P886" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P886" s="66" t="n"/>
     </row>
     <row r="887">
       <c r="A887" s="66" t="n">
@@ -58531,11 +57223,7 @@
         <f>IF(OR($J888="Attempted",$J888="Revisit"),"DUE",IF($N888="","",IF($N888&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P888" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P888" s="66" t="n"/>
     </row>
     <row r="889">
       <c r="A889" s="66" t="n">
@@ -58597,11 +57285,7 @@
         <f>IF(OR($J889="Attempted",$J889="Revisit"),"DUE",IF($N889="","",IF($N889&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P889" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P889" s="66" t="n"/>
     </row>
     <row r="890">
       <c r="A890" s="66" t="n">
@@ -58663,11 +57347,7 @@
         <f>IF(OR($J890="Attempted",$J890="Revisit"),"DUE",IF($N890="","",IF($N890&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P890" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P890" s="66" t="n"/>
     </row>
     <row r="891">
       <c r="A891" s="66" t="n">
@@ -58729,11 +57409,7 @@
         <f>IF(OR($J891="Attempted",$J891="Revisit"),"DUE",IF($N891="","",IF($N891&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P891" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P891" s="66" t="n"/>
     </row>
     <row r="892">
       <c r="A892" s="66" t="n">
@@ -58795,11 +57471,7 @@
         <f>IF(OR($J892="Attempted",$J892="Revisit"),"DUE",IF($N892="","",IF($N892&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P892" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P892" s="66" t="n"/>
     </row>
     <row r="893">
       <c r="A893" s="66" t="n">
@@ -58985,11 +57657,7 @@
         <f>IF(OR($J895="Attempted",$J895="Revisit"),"DUE",IF($N895="","",IF($N895&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P895" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P895" s="66" t="n"/>
     </row>
     <row r="896">
       <c r="A896" s="66" t="n">
@@ -59051,11 +57719,7 @@
         <f>IF(OR($J896="Attempted",$J896="Revisit"),"DUE",IF($N896="","",IF($N896&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P896" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P896" s="66" t="n"/>
     </row>
     <row r="897">
       <c r="A897" s="66" t="n">
@@ -59117,11 +57781,7 @@
         <f>IF(OR($J897="Attempted",$J897="Revisit"),"DUE",IF($N897="","",IF($N897&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P897" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P897" s="66" t="n"/>
     </row>
     <row r="898">
       <c r="A898" s="66" t="n">
@@ -59183,11 +57843,7 @@
         <f>IF(OR($J898="Attempted",$J898="Revisit"),"DUE",IF($N898="","",IF($N898&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P898" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P898" s="66" t="n"/>
     </row>
     <row r="899">
       <c r="A899" s="66" t="n">
@@ -59249,11 +57905,7 @@
         <f>IF(OR($J899="Attempted",$J899="Revisit"),"DUE",IF($N899="","",IF($N899&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P899" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P899" s="66" t="n"/>
     </row>
     <row r="900">
       <c r="A900" s="66" t="n">
@@ -59315,11 +57967,7 @@
         <f>IF(OR($J900="Attempted",$J900="Revisit"),"DUE",IF($N900="","",IF($N900&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P900" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P900" s="66" t="n"/>
     </row>
     <row r="901">
       <c r="A901" s="66" t="n">
@@ -59443,11 +58091,7 @@
         <f>IF(OR($J902="Attempted",$J902="Revisit"),"DUE",IF($N902="","",IF($N902&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P902" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P902" s="66" t="n"/>
     </row>
     <row r="903">
       <c r="A903" s="66" t="n">
@@ -59509,11 +58153,7 @@
         <f>IF(OR($J903="Attempted",$J903="Revisit"),"DUE",IF($N903="","",IF($N903&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P903" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P903" s="66" t="n"/>
     </row>
     <row r="904">
       <c r="A904" s="66" t="n">
@@ -59575,11 +58215,7 @@
         <f>IF(OR($J904="Attempted",$J904="Revisit"),"DUE",IF($N904="","",IF($N904&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P904" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P904" s="66" t="n"/>
     </row>
     <row r="905">
       <c r="A905" s="66" t="n">
@@ -59765,11 +58401,7 @@
         <f>IF(OR($J907="Attempted",$J907="Revisit"),"DUE",IF($N907="","",IF($N907&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P907" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P907" s="66" t="n"/>
     </row>
     <row r="908">
       <c r="A908" s="66" t="n">
@@ -59831,11 +58463,7 @@
         <f>IF(OR($J908="Attempted",$J908="Revisit"),"DUE",IF($N908="","",IF($N908&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P908" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P908" s="66" t="n"/>
     </row>
     <row r="909">
       <c r="A909" s="66" t="n">
@@ -60083,11 +58711,7 @@
         <f>IF(OR($J912="Attempted",$J912="Revisit"),"DUE",IF($N912="","",IF($N912&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P912" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P912" s="66" t="n"/>
     </row>
     <row r="913">
       <c r="A913" s="66" t="n">
@@ -60211,11 +58835,7 @@
         <f>IF(OR($J914="Attempted",$J914="Revisit"),"DUE",IF($N914="","",IF($N914&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P914" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P914" s="66" t="n"/>
     </row>
     <row r="915">
       <c r="A915" s="66" t="n">
@@ -60277,11 +58897,7 @@
         <f>IF(OR($J915="Attempted",$J915="Revisit"),"DUE",IF($N915="","",IF($N915&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P915" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P915" s="66" t="n"/>
     </row>
     <row r="916">
       <c r="A916" s="66" t="n">
@@ -60405,11 +59021,7 @@
         <f>IF(OR($J917="Attempted",$J917="Revisit"),"DUE",IF($N917="","",IF($N917&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P917" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P917" s="66" t="n"/>
     </row>
     <row r="918">
       <c r="A918" s="66" t="n">
@@ -60471,11 +59083,7 @@
         <f>IF(OR($J918="Attempted",$J918="Revisit"),"DUE",IF($N918="","",IF($N918&lt;=TODAY(),"DUE","")))</f>
         <v/>
       </c>
-      <c r="P918" s="66" t="inlineStr">
-        <is>
-          <t>v3 addition</t>
-        </is>
-      </c>
+      <c r="P918" s="66" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:P918"/>
@@ -60615,7 +59223,7 @@
     <row r="6" ht="15" customHeight="1" s="32">
       <c r="B6" s="37" t="inlineStr">
         <is>
-          <t>All 922 questions</t>
+          <t>All 917 questions</t>
         </is>
       </c>
       <c r="C6" s="53">

</xml_diff>

<commit_message>
Point Wiggle Sort at its free GeeksforGeeks page
The LeetCode problem is Premium-only, so the Core track's step 45 couldn't
be solved. GeeksforGeeks' Convert To Zig-Zag is the same problem (arr[0] <
arr[1] > arr[2] < ...); the link is verified and the Master tab matches.
</commit_message>
<xml_diff>
--- a/DSA_Master_Sheet.xlsx
+++ b/DSA_Master_Sheet.xlsx
@@ -4995,12 +4995,12 @@
       </c>
       <c r="H46" s="61" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I46" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/wiggle-sort/</t>
+          <t>https://www.geeksforgeeks.org/problems/convert-array-into-zig-zag-fashion1638/1</t>
         </is>
       </c>
       <c r="J46" s="61" t="inlineStr">

</xml_diff>

<commit_message>
Give Core a tree serialization problem and describe Core honestly
Serialize and Deserialize BST moves from Depth to Core, so the Core track
now meets tree serialization; the Hard binary-tree version stays in Depth.
Job Sequencing moves from Greedy's one-problem "Interval greedy" pattern to
Intervals / Scheduling. Steps are renumbered for the whole sheet.

The workbook follows: Master rows reordered, Path Stages ranges, Pattern
Radar and Pattern Coverage lose the empty pattern row, and Start Here's
counts change.

The README and Start Here no longer claim Core covers every pattern with
two problems each. Core is the main track and deliberately skips the
advanced patterns, which live in Depth and Stretch.
</commit_message>
<xml_diff>
--- a/DSA_Master_Sheet.xlsx
+++ b/DSA_Master_Sheet.xlsx
@@ -899,7 +899,7 @@
     <row r="9" ht="27.75" customHeight="1" s="32">
       <c r="C9" s="36" t="inlineStr">
         <is>
-          <t>Core (387) - at least two problems per pattern, every pattern in the sheet. Finish this and you have touched every idea an interview can ask. This is your actual target.</t>
+          <t>Core (388) - the main track. It deliberately skips the advanced patterns (SCC, Euler path, bridges and articulation points, binary lifting, bitmask DP, and everything in Advanced DS); those live in Depth and Stretch. This is your actual target.</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="C30" s="36" t="inlineStr">
         <is>
-          <t>Per-pattern totals, done count and average confidence across all 172 patterns.</t>
+          <t>Per-pattern totals, done count and average confidence across all 171 patterns.</t>
         </is>
       </c>
     </row>
@@ -1565,17 +1565,17 @@
       </c>
       <c r="B14" s="31" t="inlineStr">
         <is>
-          <t>578-653</t>
+          <t>578-654</t>
         </is>
       </c>
       <c r="C14" s="31" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D14" s="31" t="n">
         <v>30</v>
       </c>
       <c r="E14" s="31" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F14" s="31" t="n">
         <v>1</v>
@@ -1594,17 +1594,17 @@
       </c>
       <c r="B15" s="31" t="inlineStr">
         <is>
-          <t>654-739</t>
+          <t>655-739</t>
         </is>
       </c>
       <c r="C15" s="31" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D15" s="31" t="n">
         <v>2</v>
       </c>
       <c r="E15" s="31" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F15" s="31" t="n">
         <v>6</v>
@@ -33991,12 +33991,12 @@
       </c>
       <c r="D514" s="65" t="inlineStr">
         <is>
-          <t>Booking</t>
+          <t>Scheduling</t>
         </is>
       </c>
       <c r="E514" s="65" t="inlineStr">
         <is>
-          <t>The Number of the Smallest Unoccupied Chair</t>
+          <t>Job Sequencing Problem</t>
         </is>
       </c>
       <c r="F514" s="65" t="inlineStr">
@@ -34011,12 +34011,12 @@
       </c>
       <c r="H514" s="65" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I514" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/the-number-of-the-smallest-unoccupied-chair/</t>
+          <t>https://www.geeksforgeeks.org/problems/job-sequencing-problem-1587115620/1</t>
         </is>
       </c>
       <c r="J514" s="65" t="inlineStr">
@@ -34048,17 +34048,17 @@
       </c>
       <c r="C515" s="65" t="inlineStr">
         <is>
-          <t>16. Greedy</t>
+          <t>15. Intervals</t>
         </is>
       </c>
       <c r="D515" s="65" t="inlineStr">
         <is>
-          <t>Sort + pick</t>
+          <t>Booking</t>
         </is>
       </c>
       <c r="E515" s="65" t="inlineStr">
         <is>
-          <t>Two City Scheduling</t>
+          <t>The Number of the Smallest Unoccupied Chair</t>
         </is>
       </c>
       <c r="F515" s="65" t="inlineStr">
@@ -34078,7 +34078,7 @@
       </c>
       <c r="I515" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/two-city-scheduling/</t>
+          <t>https://leetcode.com/problems/the-number-of-the-smallest-unoccupied-chair/</t>
         </is>
       </c>
       <c r="J515" s="65" t="inlineStr">
@@ -34120,7 +34120,7 @@
       </c>
       <c r="E516" s="65" t="inlineStr">
         <is>
-          <t>Advantage Shuffle</t>
+          <t>Two City Scheduling</t>
         </is>
       </c>
       <c r="F516" s="65" t="inlineStr">
@@ -34140,7 +34140,7 @@
       </c>
       <c r="I516" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/advantage-shuffle/</t>
+          <t>https://leetcode.com/problems/two-city-scheduling/</t>
         </is>
       </c>
       <c r="J516" s="65" t="inlineStr">
@@ -34182,7 +34182,7 @@
       </c>
       <c r="E517" s="65" t="inlineStr">
         <is>
-          <t>Maximum Number of Coins You Can Get</t>
+          <t>Advantage Shuffle</t>
         </is>
       </c>
       <c r="F517" s="65" t="inlineStr">
@@ -34202,7 +34202,7 @@
       </c>
       <c r="I517" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/maximum-number-of-coins-you-can-get/</t>
+          <t>https://leetcode.com/problems/advantage-shuffle/</t>
         </is>
       </c>
       <c r="J517" s="65" t="inlineStr">
@@ -34239,12 +34239,12 @@
       </c>
       <c r="D518" s="65" t="inlineStr">
         <is>
-          <t>Classic greedy</t>
+          <t>Sort + pick</t>
         </is>
       </c>
       <c r="E518" s="65" t="inlineStr">
         <is>
-          <t>Fractional Knapsack</t>
+          <t>Maximum Number of Coins You Can Get</t>
         </is>
       </c>
       <c r="F518" s="65" t="inlineStr">
@@ -34259,12 +34259,12 @@
       </c>
       <c r="H518" s="65" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I518" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/fractional-knapsack-1587115620/1</t>
+          <t>https://leetcode.com/problems/maximum-number-of-coins-you-can-get/</t>
         </is>
       </c>
       <c r="J518" s="65" t="inlineStr">
@@ -34306,7 +34306,7 @@
       </c>
       <c r="E519" s="65" t="inlineStr">
         <is>
-          <t>Huffman Encoding</t>
+          <t>Fractional Knapsack</t>
         </is>
       </c>
       <c r="F519" s="65" t="inlineStr">
@@ -34326,7 +34326,7 @@
       </c>
       <c r="I519" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/search/?q=Huffman+Encoding</t>
+          <t>https://www.geeksforgeeks.org/problems/fractional-knapsack-1587115620/1</t>
         </is>
       </c>
       <c r="J519" s="65" t="inlineStr">
@@ -34363,12 +34363,12 @@
       </c>
       <c r="D520" s="65" t="inlineStr">
         <is>
-          <t>Simulation</t>
+          <t>Classic greedy</t>
         </is>
       </c>
       <c r="E520" s="65" t="inlineStr">
         <is>
-          <t>Broken Calculator</t>
+          <t>Huffman Encoding</t>
         </is>
       </c>
       <c r="F520" s="65" t="inlineStr">
@@ -34383,12 +34383,12 @@
       </c>
       <c r="H520" s="65" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I520" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/broken-calculator/</t>
+          <t>https://www.geeksforgeeks.org/search/?q=Huffman+Encoding</t>
         </is>
       </c>
       <c r="J520" s="65" t="inlineStr">
@@ -34430,7 +34430,7 @@
       </c>
       <c r="E521" s="65" t="inlineStr">
         <is>
-          <t>Bag of Tokens</t>
+          <t>Broken Calculator</t>
         </is>
       </c>
       <c r="F521" s="65" t="inlineStr">
@@ -34450,7 +34450,7 @@
       </c>
       <c r="I521" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/bag-of-tokens/</t>
+          <t>https://leetcode.com/problems/broken-calculator/</t>
         </is>
       </c>
       <c r="J521" s="65" t="inlineStr">
@@ -34492,7 +34492,7 @@
       </c>
       <c r="E522" s="65" t="inlineStr">
         <is>
-          <t>Push Dominoes</t>
+          <t>Bag of Tokens</t>
         </is>
       </c>
       <c r="F522" s="65" t="inlineStr">
@@ -34512,7 +34512,7 @@
       </c>
       <c r="I522" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/push-dominoes/</t>
+          <t>https://leetcode.com/problems/bag-of-tokens/</t>
         </is>
       </c>
       <c r="J522" s="65" t="inlineStr">
@@ -34554,7 +34554,7 @@
       </c>
       <c r="E523" s="65" t="inlineStr">
         <is>
-          <t>Minimum Deletions to Make Character Frequencies Unique</t>
+          <t>Push Dominoes</t>
         </is>
       </c>
       <c r="F523" s="65" t="inlineStr">
@@ -34574,7 +34574,7 @@
       </c>
       <c r="I523" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/minimum-deletions-to-make-character-frequencies-unique/</t>
+          <t>https://leetcode.com/problems/push-dominoes/</t>
         </is>
       </c>
       <c r="J523" s="65" t="inlineStr">
@@ -34611,12 +34611,12 @@
       </c>
       <c r="D524" s="65" t="inlineStr">
         <is>
-          <t>Two pass</t>
+          <t>Simulation</t>
         </is>
       </c>
       <c r="E524" s="65" t="inlineStr">
         <is>
-          <t>Best Sightseeing Pair</t>
+          <t>Minimum Deletions to Make Character Frequencies Unique</t>
         </is>
       </c>
       <c r="F524" s="65" t="inlineStr">
@@ -34636,7 +34636,7 @@
       </c>
       <c r="I524" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/best-sightseeing-pair/</t>
+          <t>https://leetcode.com/problems/minimum-deletions-to-make-character-frequencies-unique/</t>
         </is>
       </c>
       <c r="J524" s="65" t="inlineStr">
@@ -34678,12 +34678,12 @@
       </c>
       <c r="E525" s="65" t="inlineStr">
         <is>
-          <t>Candy</t>
+          <t>Best Sightseeing Pair</t>
         </is>
       </c>
       <c r="F525" s="65" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G525" s="65" t="inlineStr">
@@ -34698,7 +34698,7 @@
       </c>
       <c r="I525" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/candy/</t>
+          <t>https://leetcode.com/problems/best-sightseeing-pair/</t>
         </is>
       </c>
       <c r="J525" s="65" t="inlineStr">
@@ -34735,17 +34735,17 @@
       </c>
       <c r="D526" s="65" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Two pass</t>
         </is>
       </c>
       <c r="E526" s="65" t="inlineStr">
         <is>
-          <t>Check If a String Can Break Another String</t>
+          <t>Candy</t>
         </is>
       </c>
       <c r="F526" s="65" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="G526" s="65" t="inlineStr">
@@ -34760,7 +34760,7 @@
       </c>
       <c r="I526" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/check-if-a-string-can-break-another-string/</t>
+          <t>https://leetcode.com/problems/candy/</t>
         </is>
       </c>
       <c r="J526" s="65" t="inlineStr">
@@ -34802,7 +34802,7 @@
       </c>
       <c r="E527" s="65" t="inlineStr">
         <is>
-          <t>Minimum Number of Swaps to Make the String Balanced</t>
+          <t>Check If a String Can Break Another String</t>
         </is>
       </c>
       <c r="F527" s="65" t="inlineStr">
@@ -34822,7 +34822,7 @@
       </c>
       <c r="I527" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/minimum-number-of-swaps-to-make-the-string-balanced/</t>
+          <t>https://leetcode.com/problems/check-if-a-string-can-break-another-string/</t>
         </is>
       </c>
       <c r="J527" s="65" t="inlineStr">
@@ -34859,12 +34859,12 @@
       </c>
       <c r="D528" s="65" t="inlineStr">
         <is>
-          <t>Reachability</t>
+          <t>Validation</t>
         </is>
       </c>
       <c r="E528" s="65" t="inlineStr">
         <is>
-          <t>Jump Game III</t>
+          <t>Minimum Number of Swaps to Make the String Balanced</t>
         </is>
       </c>
       <c r="F528" s="65" t="inlineStr">
@@ -34884,7 +34884,7 @@
       </c>
       <c r="I528" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/jump-game-iii/</t>
+          <t>https://leetcode.com/problems/minimum-number-of-swaps-to-make-the-string-balanced/</t>
         </is>
       </c>
       <c r="J528" s="65" t="inlineStr">
@@ -34926,7 +34926,7 @@
       </c>
       <c r="E529" s="65" t="inlineStr">
         <is>
-          <t>Jump Game VII</t>
+          <t>Jump Game III</t>
         </is>
       </c>
       <c r="F529" s="65" t="inlineStr">
@@ -34946,7 +34946,7 @@
       </c>
       <c r="I529" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/jump-game-vii/</t>
+          <t>https://leetcode.com/problems/jump-game-iii/</t>
         </is>
       </c>
       <c r="J529" s="65" t="inlineStr">
@@ -34988,7 +34988,7 @@
       </c>
       <c r="E530" s="65" t="inlineStr">
         <is>
-          <t>Reach a Number</t>
+          <t>Jump Game VII</t>
         </is>
       </c>
       <c r="F530" s="65" t="inlineStr">
@@ -35008,7 +35008,7 @@
       </c>
       <c r="I530" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/reach-a-number/</t>
+          <t>https://leetcode.com/problems/jump-game-vii/</t>
         </is>
       </c>
       <c r="J530" s="65" t="inlineStr">
@@ -35045,12 +35045,12 @@
       </c>
       <c r="D531" s="65" t="inlineStr">
         <is>
-          <t>Partitioning</t>
+          <t>Reachability</t>
         </is>
       </c>
       <c r="E531" s="65" t="inlineStr">
         <is>
-          <t>Partition Array into Disjoint Intervals</t>
+          <t>Reach a Number</t>
         </is>
       </c>
       <c r="F531" s="65" t="inlineStr">
@@ -35070,7 +35070,7 @@
       </c>
       <c r="I531" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/partition-array-into-disjoint-intervals/</t>
+          <t>https://leetcode.com/problems/reach-a-number/</t>
         </is>
       </c>
       <c r="J531" s="65" t="inlineStr">
@@ -35112,7 +35112,7 @@
       </c>
       <c r="E532" s="65" t="inlineStr">
         <is>
-          <t>Divide Players Into Teams of Equal Skill</t>
+          <t>Partition Array into Disjoint Intervals</t>
         </is>
       </c>
       <c r="F532" s="65" t="inlineStr">
@@ -35132,7 +35132,7 @@
       </c>
       <c r="I532" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/divide-players-into-teams-of-equal-skill/</t>
+          <t>https://leetcode.com/problems/partition-array-into-disjoint-intervals/</t>
         </is>
       </c>
       <c r="J532" s="65" t="inlineStr">
@@ -35174,7 +35174,7 @@
       </c>
       <c r="E533" s="65" t="inlineStr">
         <is>
-          <t>Split Array into Consecutive Subsequences</t>
+          <t>Divide Players Into Teams of Equal Skill</t>
         </is>
       </c>
       <c r="F533" s="65" t="inlineStr">
@@ -35194,7 +35194,7 @@
       </c>
       <c r="I533" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/split-array-into-consecutive-subsequences/</t>
+          <t>https://leetcode.com/problems/divide-players-into-teams-of-equal-skill/</t>
         </is>
       </c>
       <c r="J533" s="65" t="inlineStr">
@@ -35231,12 +35231,12 @@
       </c>
       <c r="D534" s="65" t="inlineStr">
         <is>
-          <t>Reconstruction</t>
+          <t>Partitioning</t>
         </is>
       </c>
       <c r="E534" s="65" t="inlineStr">
         <is>
-          <t>Construct String With Repeat Limit</t>
+          <t>Split Array into Consecutive Subsequences</t>
         </is>
       </c>
       <c r="F534" s="65" t="inlineStr">
@@ -35256,7 +35256,7 @@
       </c>
       <c r="I534" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/construct-string-with-repeat-limit/</t>
+          <t>https://leetcode.com/problems/split-array-into-consecutive-subsequences/</t>
         </is>
       </c>
       <c r="J534" s="65" t="inlineStr">
@@ -35298,7 +35298,7 @@
       </c>
       <c r="E535" s="65" t="inlineStr">
         <is>
-          <t>Remove Duplicate Letters</t>
+          <t>Construct String With Repeat Limit</t>
         </is>
       </c>
       <c r="F535" s="65" t="inlineStr">
@@ -35318,7 +35318,7 @@
       </c>
       <c r="I535" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/remove-duplicate-letters/</t>
+          <t>https://leetcode.com/problems/construct-string-with-repeat-limit/</t>
         </is>
       </c>
       <c r="J535" s="65" t="inlineStr">
@@ -35355,12 +35355,12 @@
       </c>
       <c r="D536" s="65" t="inlineStr">
         <is>
-          <t>Interval greedy</t>
+          <t>Reconstruction</t>
         </is>
       </c>
       <c r="E536" s="65" t="inlineStr">
         <is>
-          <t>Job Sequencing Problem</t>
+          <t>Remove Duplicate Letters</t>
         </is>
       </c>
       <c r="F536" s="65" t="inlineStr">
@@ -35375,12 +35375,12 @@
       </c>
       <c r="H536" s="65" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I536" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/job-sequencing-problem-1587115620/1</t>
+          <t>https://leetcode.com/problems/remove-duplicate-letters/</t>
         </is>
       </c>
       <c r="J536" s="65" t="inlineStr">
@@ -39633,17 +39633,17 @@
       </c>
       <c r="D605" s="65" t="inlineStr">
         <is>
-          <t>BST basics</t>
+          <t>Serialization</t>
         </is>
       </c>
       <c r="E605" s="65" t="inlineStr">
         <is>
-          <t>Search in a Binary Search Tree</t>
+          <t>Serialize and Deserialize BST</t>
         </is>
       </c>
       <c r="F605" s="65" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G605" s="65" t="inlineStr">
@@ -39658,7 +39658,7 @@
       </c>
       <c r="I605" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/search-in-a-binary-search-tree/</t>
+          <t>https://leetcode.com/problems/serialize-and-deserialize-bst/</t>
         </is>
       </c>
       <c r="J605" s="65" t="inlineStr">
@@ -39700,7 +39700,7 @@
       </c>
       <c r="E606" s="65" t="inlineStr">
         <is>
-          <t>Range Sum of BST</t>
+          <t>Search in a Binary Search Tree</t>
         </is>
       </c>
       <c r="F606" s="65" t="inlineStr">
@@ -39720,7 +39720,7 @@
       </c>
       <c r="I606" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/range-sum-of-bst/</t>
+          <t>https://leetcode.com/problems/search-in-a-binary-search-tree/</t>
         </is>
       </c>
       <c r="J606" s="65" t="inlineStr">
@@ -39757,12 +39757,12 @@
       </c>
       <c r="D607" s="65" t="inlineStr">
         <is>
-          <t>BST properties</t>
+          <t>BST basics</t>
         </is>
       </c>
       <c r="E607" s="65" t="inlineStr">
         <is>
-          <t>Two Sum IV - Input is a BST</t>
+          <t>Range Sum of BST</t>
         </is>
       </c>
       <c r="F607" s="65" t="inlineStr">
@@ -39782,7 +39782,7 @@
       </c>
       <c r="I607" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/two-sum-iv-input-is-a-bst/</t>
+          <t>https://leetcode.com/problems/range-sum-of-bst/</t>
         </is>
       </c>
       <c r="J607" s="65" t="inlineStr">
@@ -39824,12 +39824,12 @@
       </c>
       <c r="E608" s="65" t="inlineStr">
         <is>
-          <t>Validate Binary Search Tree</t>
+          <t>Two Sum IV - Input is a BST</t>
         </is>
       </c>
       <c r="F608" s="65" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G608" s="65" t="inlineStr">
@@ -39844,7 +39844,7 @@
       </c>
       <c r="I608" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/validate-binary-search-tree/</t>
+          <t>https://leetcode.com/problems/two-sum-iv-input-is-a-bst/</t>
         </is>
       </c>
       <c r="J608" s="65" t="inlineStr">
@@ -39886,7 +39886,7 @@
       </c>
       <c r="E609" s="65" t="inlineStr">
         <is>
-          <t>Kth Smallest Element in a BST</t>
+          <t>Validate Binary Search Tree</t>
         </is>
       </c>
       <c r="F609" s="65" t="inlineStr">
@@ -39906,7 +39906,7 @@
       </c>
       <c r="I609" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/kth-smallest-element-in-a-bst/</t>
+          <t>https://leetcode.com/problems/validate-binary-search-tree/</t>
         </is>
       </c>
       <c r="J609" s="65" t="inlineStr">
@@ -39938,17 +39938,17 @@
       </c>
       <c r="C610" s="65" t="inlineStr">
         <is>
-          <t>19. Tries</t>
+          <t>18. Trees &amp; BST</t>
         </is>
       </c>
       <c r="D610" s="65" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>BST properties</t>
         </is>
       </c>
       <c r="E610" s="65" t="inlineStr">
         <is>
-          <t>Implement Trie (Prefix Tree)</t>
+          <t>Kth Smallest Element in a BST</t>
         </is>
       </c>
       <c r="F610" s="65" t="inlineStr">
@@ -39968,7 +39968,7 @@
       </c>
       <c r="I610" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/implement-trie-prefix-tree/</t>
+          <t>https://leetcode.com/problems/kth-smallest-element-in-a-bst/</t>
         </is>
       </c>
       <c r="J610" s="65" t="inlineStr">
@@ -40010,7 +40010,7 @@
       </c>
       <c r="E611" s="65" t="inlineStr">
         <is>
-          <t>Design Add and Search Words Data Structure</t>
+          <t>Implement Trie (Prefix Tree)</t>
         </is>
       </c>
       <c r="F611" s="65" t="inlineStr">
@@ -40030,7 +40030,7 @@
       </c>
       <c r="I611" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/design-add-and-search-words-data-structure/</t>
+          <t>https://leetcode.com/problems/implement-trie-prefix-tree/</t>
         </is>
       </c>
       <c r="J611" s="65" t="inlineStr">
@@ -40067,12 +40067,12 @@
       </c>
       <c r="D612" s="65" t="inlineStr">
         <is>
-          <t>Prefix search</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="E612" s="65" t="inlineStr">
         <is>
-          <t>Replace Words</t>
+          <t>Design Add and Search Words Data Structure</t>
         </is>
       </c>
       <c r="F612" s="65" t="inlineStr">
@@ -40092,7 +40092,7 @@
       </c>
       <c r="I612" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/replace-words/</t>
+          <t>https://leetcode.com/problems/design-add-and-search-words-data-structure/</t>
         </is>
       </c>
       <c r="J612" s="65" t="inlineStr">
@@ -40134,7 +40134,7 @@
       </c>
       <c r="E613" s="65" t="inlineStr">
         <is>
-          <t>Longest Word in Dictionary</t>
+          <t>Replace Words</t>
         </is>
       </c>
       <c r="F613" s="65" t="inlineStr">
@@ -40154,7 +40154,7 @@
       </c>
       <c r="I613" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/longest-word-in-dictionary/</t>
+          <t>https://leetcode.com/problems/replace-words/</t>
         </is>
       </c>
       <c r="J613" s="65" t="inlineStr">
@@ -40191,17 +40191,17 @@
       </c>
       <c r="D614" s="65" t="inlineStr">
         <is>
-          <t>Counting</t>
+          <t>Prefix search</t>
         </is>
       </c>
       <c r="E614" s="65" t="inlineStr">
         <is>
-          <t>Count Prefix and Suffix Pairs I</t>
+          <t>Longest Word in Dictionary</t>
         </is>
       </c>
       <c r="F614" s="65" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G614" s="65" t="inlineStr">
@@ -40216,7 +40216,7 @@
       </c>
       <c r="I614" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/count-prefix-and-suffix-pairs-i/</t>
+          <t>https://leetcode.com/problems/longest-word-in-dictionary/</t>
         </is>
       </c>
       <c r="J614" s="65" t="inlineStr">
@@ -40253,17 +40253,17 @@
       </c>
       <c r="D615" s="65" t="inlineStr">
         <is>
-          <t>Trie + grid</t>
+          <t>Counting</t>
         </is>
       </c>
       <c r="E615" s="65" t="inlineStr">
         <is>
-          <t>Word Search II</t>
+          <t>Count Prefix and Suffix Pairs I</t>
         </is>
       </c>
       <c r="F615" s="65" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G615" s="65" t="inlineStr">
@@ -40278,7 +40278,7 @@
       </c>
       <c r="I615" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/word-search-ii/</t>
+          <t>https://leetcode.com/problems/count-prefix-and-suffix-pairs-i/</t>
         </is>
       </c>
       <c r="J615" s="65" t="inlineStr">
@@ -40315,17 +40315,17 @@
       </c>
       <c r="D616" s="65" t="inlineStr">
         <is>
-          <t>Bit trie</t>
+          <t>Trie + grid</t>
         </is>
       </c>
       <c r="E616" s="65" t="inlineStr">
         <is>
-          <t>Maximum XOR of Two Numbers in an Array</t>
+          <t>Word Search II</t>
         </is>
       </c>
       <c r="F616" s="65" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="G616" s="65" t="inlineStr">
@@ -40340,7 +40340,7 @@
       </c>
       <c r="I616" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/maximum-xor-of-two-numbers-in-an-array/</t>
+          <t>https://leetcode.com/problems/word-search-ii/</t>
         </is>
       </c>
       <c r="J616" s="65" t="inlineStr">
@@ -40372,22 +40372,22 @@
       </c>
       <c r="C617" s="65" t="inlineStr">
         <is>
-          <t>20. Graphs</t>
+          <t>19. Tries</t>
         </is>
       </c>
       <c r="D617" s="65" t="inlineStr">
         <is>
-          <t>Representation</t>
+          <t>Bit trie</t>
         </is>
       </c>
       <c r="E617" s="65" t="inlineStr">
         <is>
-          <t>Print Adjacency List</t>
+          <t>Maximum XOR of Two Numbers in an Array</t>
         </is>
       </c>
       <c r="F617" s="65" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G617" s="65" t="inlineStr">
@@ -40397,12 +40397,12 @@
       </c>
       <c r="H617" s="65" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I617" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/print-adjacency-list-1587115620/1</t>
+          <t>https://leetcode.com/problems/maximum-xor-of-two-numbers-in-an-array/</t>
         </is>
       </c>
       <c r="J617" s="65" t="inlineStr">
@@ -40444,7 +40444,7 @@
       </c>
       <c r="E618" s="65" t="inlineStr">
         <is>
-          <t>Convert Adjacency Matrix to Adjacency List</t>
+          <t>Print Adjacency List</t>
         </is>
       </c>
       <c r="F618" s="65" t="inlineStr">
@@ -40464,7 +40464,7 @@
       </c>
       <c r="I618" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/search/?q=Convert+Adjacency+Matrix+to+Adjacency+List</t>
+          <t>https://www.geeksforgeeks.org/problems/print-adjacency-list-1587115620/1</t>
         </is>
       </c>
       <c r="J618" s="65" t="inlineStr">
@@ -40506,7 +40506,7 @@
       </c>
       <c r="E619" s="65" t="inlineStr">
         <is>
-          <t>Transpose of a Directed Graph</t>
+          <t>Convert Adjacency Matrix to Adjacency List</t>
         </is>
       </c>
       <c r="F619" s="65" t="inlineStr">
@@ -40526,7 +40526,7 @@
       </c>
       <c r="I619" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/search/?q=Transpose+of+a+Directed+Graph</t>
+          <t>https://www.geeksforgeeks.org/search/?q=Convert+Adjacency+Matrix+to+Adjacency+List</t>
         </is>
       </c>
       <c r="J619" s="65" t="inlineStr">
@@ -40568,7 +40568,7 @@
       </c>
       <c r="E620" s="65" t="inlineStr">
         <is>
-          <t>Find the Town Judge</t>
+          <t>Transpose of a Directed Graph</t>
         </is>
       </c>
       <c r="F620" s="65" t="inlineStr">
@@ -40583,12 +40583,12 @@
       </c>
       <c r="H620" s="65" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I620" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/find-the-town-judge/</t>
+          <t>https://www.geeksforgeeks.org/search/?q=Transpose+of+a+Directed+Graph</t>
         </is>
       </c>
       <c r="J620" s="65" t="inlineStr">
@@ -40630,7 +40630,7 @@
       </c>
       <c r="E621" s="65" t="inlineStr">
         <is>
-          <t>Find Center of Star Graph</t>
+          <t>Find the Town Judge</t>
         </is>
       </c>
       <c r="F621" s="65" t="inlineStr">
@@ -40650,7 +40650,7 @@
       </c>
       <c r="I621" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/find-center-of-star-graph/</t>
+          <t>https://leetcode.com/problems/find-the-town-judge/</t>
         </is>
       </c>
       <c r="J621" s="65" t="inlineStr">
@@ -40687,12 +40687,12 @@
       </c>
       <c r="D622" s="65" t="inlineStr">
         <is>
-          <t>Traversal</t>
+          <t>Representation</t>
         </is>
       </c>
       <c r="E622" s="65" t="inlineStr">
         <is>
-          <t>DFS of Graph</t>
+          <t>Find Center of Star Graph</t>
         </is>
       </c>
       <c r="F622" s="65" t="inlineStr">
@@ -40707,12 +40707,12 @@
       </c>
       <c r="H622" s="65" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I622" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/depth-first-traversal-for-a-graph/1</t>
+          <t>https://leetcode.com/problems/find-center-of-star-graph/</t>
         </is>
       </c>
       <c r="J622" s="65" t="inlineStr">
@@ -40754,7 +40754,7 @@
       </c>
       <c r="E623" s="65" t="inlineStr">
         <is>
-          <t>BFS of Graph</t>
+          <t>DFS of Graph</t>
         </is>
       </c>
       <c r="F623" s="65" t="inlineStr">
@@ -40774,7 +40774,7 @@
       </c>
       <c r="I623" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/bfs-traversal-of-graph/1</t>
+          <t>https://www.geeksforgeeks.org/problems/depth-first-traversal-for-a-graph/1</t>
         </is>
       </c>
       <c r="J623" s="65" t="inlineStr">
@@ -40816,7 +40816,7 @@
       </c>
       <c r="E624" s="65" t="inlineStr">
         <is>
-          <t>Find if Path Exists in Graph</t>
+          <t>BFS of Graph</t>
         </is>
       </c>
       <c r="F624" s="65" t="inlineStr">
@@ -40831,12 +40831,12 @@
       </c>
       <c r="H624" s="65" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I624" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/find-if-path-exists-in-graph/</t>
+          <t>https://www.geeksforgeeks.org/problems/bfs-traversal-of-graph/1</t>
         </is>
       </c>
       <c r="J624" s="65" t="inlineStr">
@@ -40878,12 +40878,12 @@
       </c>
       <c r="E625" s="65" t="inlineStr">
         <is>
-          <t>Clone Graph</t>
+          <t>Find if Path Exists in Graph</t>
         </is>
       </c>
       <c r="F625" s="65" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G625" s="65" t="inlineStr">
@@ -40898,7 +40898,7 @@
       </c>
       <c r="I625" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/clone-graph/</t>
+          <t>https://leetcode.com/problems/find-if-path-exists-in-graph/</t>
         </is>
       </c>
       <c r="J625" s="65" t="inlineStr">
@@ -40935,17 +40935,17 @@
       </c>
       <c r="D626" s="65" t="inlineStr">
         <is>
-          <t>Grid DFS/BFS</t>
+          <t>Traversal</t>
         </is>
       </c>
       <c r="E626" s="65" t="inlineStr">
         <is>
-          <t>Flood Fill</t>
+          <t>Clone Graph</t>
         </is>
       </c>
       <c r="F626" s="65" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G626" s="65" t="inlineStr">
@@ -40960,7 +40960,7 @@
       </c>
       <c r="I626" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/flood-fill/</t>
+          <t>https://leetcode.com/problems/clone-graph/</t>
         </is>
       </c>
       <c r="J626" s="65" t="inlineStr">
@@ -41002,12 +41002,12 @@
       </c>
       <c r="E627" s="65" t="inlineStr">
         <is>
-          <t>Number of Islands</t>
+          <t>Flood Fill</t>
         </is>
       </c>
       <c r="F627" s="65" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G627" s="65" t="inlineStr">
@@ -41022,7 +41022,7 @@
       </c>
       <c r="I627" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/number-of-islands/</t>
+          <t>https://leetcode.com/problems/flood-fill/</t>
         </is>
       </c>
       <c r="J627" s="65" t="inlineStr">
@@ -41064,7 +41064,7 @@
       </c>
       <c r="E628" s="65" t="inlineStr">
         <is>
-          <t>Max Area of Island</t>
+          <t>Number of Islands</t>
         </is>
       </c>
       <c r="F628" s="65" t="inlineStr">
@@ -41084,7 +41084,7 @@
       </c>
       <c r="I628" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/max-area-of-island/</t>
+          <t>https://leetcode.com/problems/number-of-islands/</t>
         </is>
       </c>
       <c r="J628" s="65" t="inlineStr">
@@ -41126,7 +41126,7 @@
       </c>
       <c r="E629" s="65" t="inlineStr">
         <is>
-          <t>Surrounded Regions</t>
+          <t>Max Area of Island</t>
         </is>
       </c>
       <c r="F629" s="65" t="inlineStr">
@@ -41146,7 +41146,7 @@
       </c>
       <c r="I629" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/surrounded-regions/</t>
+          <t>https://leetcode.com/problems/max-area-of-island/</t>
         </is>
       </c>
       <c r="J629" s="65" t="inlineStr">
@@ -41183,12 +41183,12 @@
       </c>
       <c r="D630" s="65" t="inlineStr">
         <is>
-          <t>Multi-source BFS</t>
+          <t>Grid DFS/BFS</t>
         </is>
       </c>
       <c r="E630" s="65" t="inlineStr">
         <is>
-          <t>Rotting Oranges</t>
+          <t>Surrounded Regions</t>
         </is>
       </c>
       <c r="F630" s="65" t="inlineStr">
@@ -41208,7 +41208,7 @@
       </c>
       <c r="I630" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/rotting-oranges/</t>
+          <t>https://leetcode.com/problems/surrounded-regions/</t>
         </is>
       </c>
       <c r="J630" s="65" t="inlineStr">
@@ -41250,7 +41250,7 @@
       </c>
       <c r="E631" s="65" t="inlineStr">
         <is>
-          <t>01 Matrix</t>
+          <t>Rotting Oranges</t>
         </is>
       </c>
       <c r="F631" s="65" t="inlineStr">
@@ -41270,7 +41270,7 @@
       </c>
       <c r="I631" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/01-matrix/</t>
+          <t>https://leetcode.com/problems/rotting-oranges/</t>
         </is>
       </c>
       <c r="J631" s="65" t="inlineStr">
@@ -41307,12 +41307,12 @@
       </c>
       <c r="D632" s="65" t="inlineStr">
         <is>
-          <t>Connected components</t>
+          <t>Multi-source BFS</t>
         </is>
       </c>
       <c r="E632" s="65" t="inlineStr">
         <is>
-          <t>Number of Provinces</t>
+          <t>01 Matrix</t>
         </is>
       </c>
       <c r="F632" s="65" t="inlineStr">
@@ -41332,7 +41332,7 @@
       </c>
       <c r="I632" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/number-of-provinces/</t>
+          <t>https://leetcode.com/problems/01-matrix/</t>
         </is>
       </c>
       <c r="J632" s="65" t="inlineStr">
@@ -41369,12 +41369,12 @@
       </c>
       <c r="D633" s="65" t="inlineStr">
         <is>
-          <t>Coloring</t>
+          <t>Connected components</t>
         </is>
       </c>
       <c r="E633" s="65" t="inlineStr">
         <is>
-          <t>M-Coloring Problem</t>
+          <t>Number of Provinces</t>
         </is>
       </c>
       <c r="F633" s="65" t="inlineStr">
@@ -41389,12 +41389,12 @@
       </c>
       <c r="H633" s="65" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I633" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/m-coloring-problem-1587115620/1</t>
+          <t>https://leetcode.com/problems/number-of-provinces/</t>
         </is>
       </c>
       <c r="J633" s="65" t="inlineStr">
@@ -41436,7 +41436,7 @@
       </c>
       <c r="E634" s="65" t="inlineStr">
         <is>
-          <t>Is Graph Bipartite?</t>
+          <t>M-Coloring Problem</t>
         </is>
       </c>
       <c r="F634" s="65" t="inlineStr">
@@ -41451,12 +41451,12 @@
       </c>
       <c r="H634" s="65" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I634" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/is-graph-bipartite/</t>
+          <t>https://www.geeksforgeeks.org/problems/m-coloring-problem-1587115620/1</t>
         </is>
       </c>
       <c r="J634" s="65" t="inlineStr">
@@ -41493,12 +41493,12 @@
       </c>
       <c r="D635" s="65" t="inlineStr">
         <is>
-          <t>Cycle detection</t>
+          <t>Coloring</t>
         </is>
       </c>
       <c r="E635" s="65" t="inlineStr">
         <is>
-          <t>Detect Cycle in an Undirected Graph</t>
+          <t>Is Graph Bipartite?</t>
         </is>
       </c>
       <c r="F635" s="65" t="inlineStr">
@@ -41513,12 +41513,12 @@
       </c>
       <c r="H635" s="65" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I635" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/detect-cycle-in-an-undirected-graph/1</t>
+          <t>https://leetcode.com/problems/is-graph-bipartite/</t>
         </is>
       </c>
       <c r="J635" s="65" t="inlineStr">
@@ -41560,7 +41560,7 @@
       </c>
       <c r="E636" s="65" t="inlineStr">
         <is>
-          <t>Detect Cycle in a Directed Graph</t>
+          <t>Detect Cycle in an Undirected Graph</t>
         </is>
       </c>
       <c r="F636" s="65" t="inlineStr">
@@ -41580,7 +41580,7 @@
       </c>
       <c r="I636" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/detect-cycle-in-a-directed-graph/1</t>
+          <t>https://www.geeksforgeeks.org/problems/detect-cycle-in-an-undirected-graph/1</t>
         </is>
       </c>
       <c r="J636" s="65" t="inlineStr">
@@ -41617,12 +41617,12 @@
       </c>
       <c r="D637" s="65" t="inlineStr">
         <is>
-          <t>BFS shortest path</t>
+          <t>Cycle detection</t>
         </is>
       </c>
       <c r="E637" s="65" t="inlineStr">
         <is>
-          <t>Shortest Path in Binary Matrix</t>
+          <t>Detect Cycle in a Directed Graph</t>
         </is>
       </c>
       <c r="F637" s="65" t="inlineStr">
@@ -41637,12 +41637,12 @@
       </c>
       <c r="H637" s="65" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I637" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/shortest-path-in-binary-matrix/</t>
+          <t>https://www.geeksforgeeks.org/problems/detect-cycle-in-a-directed-graph/1</t>
         </is>
       </c>
       <c r="J637" s="65" t="inlineStr">
@@ -41684,7 +41684,7 @@
       </c>
       <c r="E638" s="65" t="inlineStr">
         <is>
-          <t>Shortest Path in Undirected Graph (unit weights)</t>
+          <t>Shortest Path in Binary Matrix</t>
         </is>
       </c>
       <c r="F638" s="65" t="inlineStr">
@@ -41699,12 +41699,12 @@
       </c>
       <c r="H638" s="65" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I638" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/shortest-path-in-undirected-graph-having-unit-distance/1</t>
+          <t>https://leetcode.com/problems/shortest-path-in-binary-matrix/</t>
         </is>
       </c>
       <c r="J638" s="65" t="inlineStr">
@@ -41741,12 +41741,12 @@
       </c>
       <c r="D639" s="65" t="inlineStr">
         <is>
-          <t>Topological sort</t>
+          <t>BFS shortest path</t>
         </is>
       </c>
       <c r="E639" s="65" t="inlineStr">
         <is>
-          <t>Topological Sort</t>
+          <t>Shortest Path in Undirected Graph (unit weights)</t>
         </is>
       </c>
       <c r="F639" s="65" t="inlineStr">
@@ -41766,7 +41766,7 @@
       </c>
       <c r="I639" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/topological-sort/1</t>
+          <t>https://www.geeksforgeeks.org/problems/shortest-path-in-undirected-graph-having-unit-distance/1</t>
         </is>
       </c>
       <c r="J639" s="65" t="inlineStr">
@@ -41808,7 +41808,7 @@
       </c>
       <c r="E640" s="65" t="inlineStr">
         <is>
-          <t>Course Schedule</t>
+          <t>Topological Sort</t>
         </is>
       </c>
       <c r="F640" s="65" t="inlineStr">
@@ -41823,12 +41823,12 @@
       </c>
       <c r="H640" s="65" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I640" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/course-schedule/</t>
+          <t>https://www.geeksforgeeks.org/problems/topological-sort/1</t>
         </is>
       </c>
       <c r="J640" s="65" t="inlineStr">
@@ -41870,7 +41870,7 @@
       </c>
       <c r="E641" s="65" t="inlineStr">
         <is>
-          <t>Course Schedule II</t>
+          <t>Course Schedule</t>
         </is>
       </c>
       <c r="F641" s="65" t="inlineStr">
@@ -41890,7 +41890,7 @@
       </c>
       <c r="I641" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/course-schedule-ii/</t>
+          <t>https://leetcode.com/problems/course-schedule/</t>
         </is>
       </c>
       <c r="J641" s="65" t="inlineStr">
@@ -41927,12 +41927,12 @@
       </c>
       <c r="D642" s="65" t="inlineStr">
         <is>
-          <t>DSU</t>
+          <t>Topological sort</t>
         </is>
       </c>
       <c r="E642" s="65" t="inlineStr">
         <is>
-          <t>Disjoint Set (Union by Rank &amp; Path Compression)</t>
+          <t>Course Schedule II</t>
         </is>
       </c>
       <c r="F642" s="65" t="inlineStr">
@@ -41947,12 +41947,12 @@
       </c>
       <c r="H642" s="65" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I642" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/disjoint-set-union-find/1</t>
+          <t>https://leetcode.com/problems/course-schedule-ii/</t>
         </is>
       </c>
       <c r="J642" s="65" t="inlineStr">
@@ -41994,7 +41994,7 @@
       </c>
       <c r="E643" s="65" t="inlineStr">
         <is>
-          <t>Redundant Connection</t>
+          <t>Disjoint Set (Union by Rank &amp; Path Compression)</t>
         </is>
       </c>
       <c r="F643" s="65" t="inlineStr">
@@ -42009,12 +42009,12 @@
       </c>
       <c r="H643" s="65" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I643" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/redundant-connection/</t>
+          <t>https://www.geeksforgeeks.org/problems/disjoint-set-union-find/1</t>
         </is>
       </c>
       <c r="J643" s="65" t="inlineStr">
@@ -42056,7 +42056,7 @@
       </c>
       <c r="E644" s="65" t="inlineStr">
         <is>
-          <t>Accounts Merge</t>
+          <t>Redundant Connection</t>
         </is>
       </c>
       <c r="F644" s="65" t="inlineStr">
@@ -42076,7 +42076,7 @@
       </c>
       <c r="I644" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/accounts-merge/</t>
+          <t>https://leetcode.com/problems/redundant-connection/</t>
         </is>
       </c>
       <c r="J644" s="65" t="inlineStr">
@@ -42113,12 +42113,12 @@
       </c>
       <c r="D645" s="65" t="inlineStr">
         <is>
-          <t>Dijkstra</t>
+          <t>DSU</t>
         </is>
       </c>
       <c r="E645" s="65" t="inlineStr">
         <is>
-          <t>Implementing Dijkstra Algorithm</t>
+          <t>Accounts Merge</t>
         </is>
       </c>
       <c r="F645" s="65" t="inlineStr">
@@ -42133,12 +42133,12 @@
       </c>
       <c r="H645" s="65" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I645" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/implementing-dijkstra-set-1-adjacency-matrix/1</t>
+          <t>https://leetcode.com/problems/accounts-merge/</t>
         </is>
       </c>
       <c r="J645" s="65" t="inlineStr">
@@ -42180,7 +42180,7 @@
       </c>
       <c r="E646" s="65" t="inlineStr">
         <is>
-          <t>Network Delay Time</t>
+          <t>Implementing Dijkstra Algorithm</t>
         </is>
       </c>
       <c r="F646" s="65" t="inlineStr">
@@ -42195,12 +42195,12 @@
       </c>
       <c r="H646" s="65" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I646" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/network-delay-time/</t>
+          <t>https://www.geeksforgeeks.org/problems/implementing-dijkstra-set-1-adjacency-matrix/1</t>
         </is>
       </c>
       <c r="J646" s="65" t="inlineStr">
@@ -42237,12 +42237,12 @@
       </c>
       <c r="D647" s="65" t="inlineStr">
         <is>
-          <t>Bellman-Ford</t>
+          <t>Dijkstra</t>
         </is>
       </c>
       <c r="E647" s="65" t="inlineStr">
         <is>
-          <t>Distance from the Source (Bellman-Ford)</t>
+          <t>Network Delay Time</t>
         </is>
       </c>
       <c r="F647" s="65" t="inlineStr">
@@ -42257,12 +42257,12 @@
       </c>
       <c r="H647" s="65" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I647" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/distance-from-the-source-bellman-ford-algorithm/1</t>
+          <t>https://leetcode.com/problems/network-delay-time/</t>
         </is>
       </c>
       <c r="J647" s="65" t="inlineStr">
@@ -42304,7 +42304,7 @@
       </c>
       <c r="E648" s="65" t="inlineStr">
         <is>
-          <t>Cheapest Flights Within K Stops</t>
+          <t>Distance from the Source (Bellman-Ford)</t>
         </is>
       </c>
       <c r="F648" s="65" t="inlineStr">
@@ -42319,12 +42319,12 @@
       </c>
       <c r="H648" s="65" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I648" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/cheapest-flights-within-k-stops/</t>
+          <t>https://www.geeksforgeeks.org/problems/distance-from-the-source-bellman-ford-algorithm/1</t>
         </is>
       </c>
       <c r="J648" s="65" t="inlineStr">
@@ -42361,12 +42361,12 @@
       </c>
       <c r="D649" s="65" t="inlineStr">
         <is>
-          <t>Floyd-Warshall</t>
+          <t>Bellman-Ford</t>
         </is>
       </c>
       <c r="E649" s="65" t="inlineStr">
         <is>
-          <t>Floyd Warshall Algorithm</t>
+          <t>Cheapest Flights Within K Stops</t>
         </is>
       </c>
       <c r="F649" s="65" t="inlineStr">
@@ -42381,12 +42381,12 @@
       </c>
       <c r="H649" s="65" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I649" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/implementing-floyd-warshall2042/1</t>
+          <t>https://leetcode.com/problems/cheapest-flights-within-k-stops/</t>
         </is>
       </c>
       <c r="J649" s="65" t="inlineStr">
@@ -42428,7 +42428,7 @@
       </c>
       <c r="E650" s="65" t="inlineStr">
         <is>
-          <t>Find the City With the Smallest Number of Neighbors</t>
+          <t>Floyd Warshall Algorithm</t>
         </is>
       </c>
       <c r="F650" s="65" t="inlineStr">
@@ -42443,12 +42443,12 @@
       </c>
       <c r="H650" s="65" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I650" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/find-the-city-with-the-smallest-number-of-neighbors-at-a-threshold-distance/</t>
+          <t>https://www.geeksforgeeks.org/problems/implementing-floyd-warshall2042/1</t>
         </is>
       </c>
       <c r="J650" s="65" t="inlineStr">
@@ -42485,12 +42485,12 @@
       </c>
       <c r="D651" s="65" t="inlineStr">
         <is>
-          <t>MST</t>
+          <t>Floyd-Warshall</t>
         </is>
       </c>
       <c r="E651" s="65" t="inlineStr">
         <is>
-          <t>Minimum Spanning Tree (Prim's)</t>
+          <t>Find the City With the Smallest Number of Neighbors</t>
         </is>
       </c>
       <c r="F651" s="65" t="inlineStr">
@@ -42505,12 +42505,12 @@
       </c>
       <c r="H651" s="65" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I651" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/minimum-spanning-tree/1</t>
+          <t>https://leetcode.com/problems/find-the-city-with-the-smallest-number-of-neighbors-at-a-threshold-distance/</t>
         </is>
       </c>
       <c r="J651" s="65" t="inlineStr">
@@ -42552,7 +42552,7 @@
       </c>
       <c r="E652" s="65" t="inlineStr">
         <is>
-          <t>Kruskal's Algorithm</t>
+          <t>Minimum Spanning Tree (Prim's)</t>
         </is>
       </c>
       <c r="F652" s="65" t="inlineStr">
@@ -42572,7 +42572,7 @@
       </c>
       <c r="I652" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/minimum-spanning-tree-kruskals-algorithm/1</t>
+          <t>https://www.geeksforgeeks.org/problems/minimum-spanning-tree/1</t>
         </is>
       </c>
       <c r="J652" s="65" t="inlineStr">
@@ -42609,12 +42609,12 @@
       </c>
       <c r="D653" s="65" t="inlineStr">
         <is>
-          <t>Misc</t>
+          <t>MST</t>
         </is>
       </c>
       <c r="E653" s="65" t="inlineStr">
         <is>
-          <t>Graph Valid Tree</t>
+          <t>Kruskal's Algorithm</t>
         </is>
       </c>
       <c r="F653" s="65" t="inlineStr">
@@ -42634,7 +42634,7 @@
       </c>
       <c r="I653" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/is-it-a-tree/1</t>
+          <t>https://www.geeksforgeeks.org/problems/minimum-spanning-tree-kruskals-algorithm/1</t>
         </is>
       </c>
       <c r="J653" s="65" t="inlineStr">
@@ -42676,7 +42676,7 @@
       </c>
       <c r="E654" s="65" t="inlineStr">
         <is>
-          <t>Evaluate Division</t>
+          <t>Graph Valid Tree</t>
         </is>
       </c>
       <c r="F654" s="65" t="inlineStr">
@@ -42691,12 +42691,12 @@
       </c>
       <c r="H654" s="65" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I654" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/evaluate-division/</t>
+          <t>https://www.geeksforgeeks.org/problems/is-it-a-tree/1</t>
         </is>
       </c>
       <c r="J654" s="65" t="inlineStr">
@@ -42723,32 +42723,32 @@
       </c>
       <c r="B655" s="65" t="inlineStr">
         <is>
-          <t>5. Trees &amp; Graphs - Depth</t>
+          <t>5. Trees &amp; Graphs - Core</t>
         </is>
       </c>
       <c r="C655" s="65" t="inlineStr">
         <is>
-          <t>18. Trees &amp; BST</t>
+          <t>20. Graphs</t>
         </is>
       </c>
       <c r="D655" s="65" t="inlineStr">
         <is>
-          <t>Traversal</t>
+          <t>Misc</t>
         </is>
       </c>
       <c r="E655" s="65" t="inlineStr">
         <is>
-          <t>Binary Tree Postorder Traversal</t>
+          <t>Evaluate Division</t>
         </is>
       </c>
       <c r="F655" s="65" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G655" s="65" t="inlineStr">
         <is>
-          <t>Depth</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H655" s="65" t="inlineStr">
@@ -42758,7 +42758,7 @@
       </c>
       <c r="I655" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/binary-tree-postorder-traversal/</t>
+          <t>https://leetcode.com/problems/evaluate-division/</t>
         </is>
       </c>
       <c r="J655" s="65" t="inlineStr">
@@ -42800,12 +42800,12 @@
       </c>
       <c r="E656" s="65" t="inlineStr">
         <is>
-          <t>Morris Inorder Traversal</t>
+          <t>Binary Tree Postorder Traversal</t>
         </is>
       </c>
       <c r="F656" s="65" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G656" s="65" t="inlineStr">
@@ -42815,12 +42815,12 @@
       </c>
       <c r="H656" s="65" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I656" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/inorder-traversal/1</t>
+          <t>https://leetcode.com/problems/binary-tree-postorder-traversal/</t>
         </is>
       </c>
       <c r="J656" s="65" t="inlineStr">
@@ -42857,17 +42857,17 @@
       </c>
       <c r="D657" s="65" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>Traversal</t>
         </is>
       </c>
       <c r="E657" s="65" t="inlineStr">
         <is>
-          <t>Count Complete Tree Nodes</t>
+          <t>Morris Inorder Traversal</t>
         </is>
       </c>
       <c r="F657" s="65" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G657" s="65" t="inlineStr">
@@ -42877,12 +42877,12 @@
       </c>
       <c r="H657" s="65" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I657" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/count-complete-tree-nodes/</t>
+          <t>https://www.geeksforgeeks.org/problems/inorder-traversal/1</t>
         </is>
       </c>
       <c r="J657" s="65" t="inlineStr">
@@ -42924,12 +42924,12 @@
       </c>
       <c r="E658" s="65" t="inlineStr">
         <is>
-          <t>Flip Equivalent Binary Trees</t>
+          <t>Count Complete Tree Nodes</t>
         </is>
       </c>
       <c r="F658" s="65" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G658" s="65" t="inlineStr">
@@ -42944,7 +42944,7 @@
       </c>
       <c r="I658" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/flip-equivalent-binary-trees/</t>
+          <t>https://leetcode.com/problems/count-complete-tree-nodes/</t>
         </is>
       </c>
       <c r="J658" s="65" t="inlineStr">
@@ -42986,7 +42986,7 @@
       </c>
       <c r="E659" s="65" t="inlineStr">
         <is>
-          <t>Check Completeness of a Binary Tree</t>
+          <t>Flip Equivalent Binary Trees</t>
         </is>
       </c>
       <c r="F659" s="65" t="inlineStr">
@@ -43006,7 +43006,7 @@
       </c>
       <c r="I659" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/check-completeness-of-a-binary-tree/</t>
+          <t>https://leetcode.com/problems/flip-equivalent-binary-trees/</t>
         </is>
       </c>
       <c r="J659" s="65" t="inlineStr">
@@ -43043,12 +43043,12 @@
       </c>
       <c r="D660" s="65" t="inlineStr">
         <is>
-          <t>BFS</t>
+          <t>Structure</t>
         </is>
       </c>
       <c r="E660" s="65" t="inlineStr">
         <is>
-          <t>Kth Largest Sum in a Binary Tree</t>
+          <t>Check Completeness of a Binary Tree</t>
         </is>
       </c>
       <c r="F660" s="65" t="inlineStr">
@@ -43068,7 +43068,7 @@
       </c>
       <c r="I660" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/kth-largest-sum-in-a-binary-tree/</t>
+          <t>https://leetcode.com/problems/check-completeness-of-a-binary-tree/</t>
         </is>
       </c>
       <c r="J660" s="65" t="inlineStr">
@@ -43110,7 +43110,7 @@
       </c>
       <c r="E661" s="65" t="inlineStr">
         <is>
-          <t>Binary Tree Level Order Traversal II</t>
+          <t>Kth Largest Sum in a Binary Tree</t>
         </is>
       </c>
       <c r="F661" s="65" t="inlineStr">
@@ -43130,7 +43130,7 @@
       </c>
       <c r="I661" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/binary-tree-level-order-traversal-ii/</t>
+          <t>https://leetcode.com/problems/kth-largest-sum-in-a-binary-tree/</t>
         </is>
       </c>
       <c r="J661" s="65" t="inlineStr">
@@ -43172,7 +43172,7 @@
       </c>
       <c r="E662" s="65" t="inlineStr">
         <is>
-          <t>Binary Tree Zigzag Level Order Traversal</t>
+          <t>Binary Tree Level Order Traversal II</t>
         </is>
       </c>
       <c r="F662" s="65" t="inlineStr">
@@ -43192,7 +43192,7 @@
       </c>
       <c r="I662" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/binary-tree-zigzag-level-order-traversal/</t>
+          <t>https://leetcode.com/problems/binary-tree-level-order-traversal-ii/</t>
         </is>
       </c>
       <c r="J662" s="65" t="inlineStr">
@@ -43234,7 +43234,7 @@
       </c>
       <c r="E663" s="65" t="inlineStr">
         <is>
-          <t>N-ary Tree Level Order Traversal</t>
+          <t>Binary Tree Zigzag Level Order Traversal</t>
         </is>
       </c>
       <c r="F663" s="65" t="inlineStr">
@@ -43254,7 +43254,7 @@
       </c>
       <c r="I663" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/n-ary-tree-level-order-traversal/</t>
+          <t>https://leetcode.com/problems/binary-tree-zigzag-level-order-traversal/</t>
         </is>
       </c>
       <c r="J663" s="65" t="inlineStr">
@@ -43291,12 +43291,12 @@
       </c>
       <c r="D664" s="65" t="inlineStr">
         <is>
-          <t>Views</t>
+          <t>BFS</t>
         </is>
       </c>
       <c r="E664" s="65" t="inlineStr">
         <is>
-          <t>Bottom View of Binary Tree</t>
+          <t>N-ary Tree Level Order Traversal</t>
         </is>
       </c>
       <c r="F664" s="65" t="inlineStr">
@@ -43311,12 +43311,12 @@
       </c>
       <c r="H664" s="65" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I664" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/bottom-view-of-binary-tree/1</t>
+          <t>https://leetcode.com/problems/n-ary-tree-level-order-traversal/</t>
         </is>
       </c>
       <c r="J664" s="65" t="inlineStr">
@@ -43358,7 +43358,7 @@
       </c>
       <c r="E665" s="65" t="inlineStr">
         <is>
-          <t>Boundary Traversal of Binary Tree</t>
+          <t>Bottom View of Binary Tree</t>
         </is>
       </c>
       <c r="F665" s="65" t="inlineStr">
@@ -43378,7 +43378,7 @@
       </c>
       <c r="I665" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/boundary-traversal-of-binary-tree/1</t>
+          <t>https://www.geeksforgeeks.org/problems/bottom-view-of-binary-tree/1</t>
         </is>
       </c>
       <c r="J665" s="65" t="inlineStr">
@@ -43415,12 +43415,12 @@
       </c>
       <c r="D666" s="65" t="inlineStr">
         <is>
-          <t>Path sum</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="E666" s="65" t="inlineStr">
         <is>
-          <t>Path Sum III</t>
+          <t>Boundary Traversal of Binary Tree</t>
         </is>
       </c>
       <c r="F666" s="65" t="inlineStr">
@@ -43435,12 +43435,12 @@
       </c>
       <c r="H666" s="65" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I666" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/path-sum-iii/</t>
+          <t>https://www.geeksforgeeks.org/problems/boundary-traversal-of-binary-tree/1</t>
         </is>
       </c>
       <c r="J666" s="65" t="inlineStr">
@@ -43482,7 +43482,7 @@
       </c>
       <c r="E667" s="65" t="inlineStr">
         <is>
-          <t>Sum Root to Leaf Numbers</t>
+          <t>Path Sum III</t>
         </is>
       </c>
       <c r="F667" s="65" t="inlineStr">
@@ -43502,7 +43502,7 @@
       </c>
       <c r="I667" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/sum-root-to-leaf-numbers/</t>
+          <t>https://leetcode.com/problems/path-sum-iii/</t>
         </is>
       </c>
       <c r="J667" s="65" t="inlineStr">
@@ -43539,12 +43539,12 @@
       </c>
       <c r="D668" s="65" t="inlineStr">
         <is>
-          <t>Construction</t>
+          <t>Path sum</t>
         </is>
       </c>
       <c r="E668" s="65" t="inlineStr">
         <is>
-          <t>All Possible Full Binary Trees</t>
+          <t>Sum Root to Leaf Numbers</t>
         </is>
       </c>
       <c r="F668" s="65" t="inlineStr">
@@ -43564,7 +43564,7 @@
       </c>
       <c r="I668" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/all-possible-full-binary-trees/</t>
+          <t>https://leetcode.com/problems/sum-root-to-leaf-numbers/</t>
         </is>
       </c>
       <c r="J668" s="65" t="inlineStr">
@@ -43606,7 +43606,7 @@
       </c>
       <c r="E669" s="65" t="inlineStr">
         <is>
-          <t>Construct Binary Tree from Inorder and Postorder</t>
+          <t>All Possible Full Binary Trees</t>
         </is>
       </c>
       <c r="F669" s="65" t="inlineStr">
@@ -43626,7 +43626,7 @@
       </c>
       <c r="I669" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/construct-binary-tree-from-inorder-and-postorder-traversal/</t>
+          <t>https://leetcode.com/problems/all-possible-full-binary-trees/</t>
         </is>
       </c>
       <c r="J669" s="65" t="inlineStr">
@@ -43668,7 +43668,7 @@
       </c>
       <c r="E670" s="65" t="inlineStr">
         <is>
-          <t>Flatten Binary Tree to Linked List</t>
+          <t>Construct Binary Tree from Inorder and Postorder</t>
         </is>
       </c>
       <c r="F670" s="65" t="inlineStr">
@@ -43688,7 +43688,7 @@
       </c>
       <c r="I670" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/flatten-binary-tree-to-linked-list/</t>
+          <t>https://leetcode.com/problems/construct-binary-tree-from-inorder-and-postorder-traversal/</t>
         </is>
       </c>
       <c r="J670" s="65" t="inlineStr">
@@ -43730,7 +43730,7 @@
       </c>
       <c r="E671" s="65" t="inlineStr">
         <is>
-          <t>Construct Binary Search Tree from Preorder Traversal</t>
+          <t>Flatten Binary Tree to Linked List</t>
         </is>
       </c>
       <c r="F671" s="65" t="inlineStr">
@@ -43750,7 +43750,7 @@
       </c>
       <c r="I671" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/construct-binary-search-tree-from-preorder-traversal/</t>
+          <t>https://leetcode.com/problems/flatten-binary-tree-to-linked-list/</t>
         </is>
       </c>
       <c r="J671" s="65" t="inlineStr">
@@ -43787,12 +43787,12 @@
       </c>
       <c r="D672" s="65" t="inlineStr">
         <is>
-          <t>LCA</t>
+          <t>Construction</t>
         </is>
       </c>
       <c r="E672" s="65" t="inlineStr">
         <is>
-          <t>Lowest Common Ancestor of Deepest Leaves</t>
+          <t>Construct Binary Search Tree from Preorder Traversal</t>
         </is>
       </c>
       <c r="F672" s="65" t="inlineStr">
@@ -43812,7 +43812,7 @@
       </c>
       <c r="I672" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/lowest-common-ancestor-of-deepest-leaves/</t>
+          <t>https://leetcode.com/problems/construct-binary-search-tree-from-preorder-traversal/</t>
         </is>
       </c>
       <c r="J672" s="65" t="inlineStr">
@@ -43854,7 +43854,7 @@
       </c>
       <c r="E673" s="65" t="inlineStr">
         <is>
-          <t>Step-By-Step Directions From a Binary Tree Node to Another</t>
+          <t>Lowest Common Ancestor of Deepest Leaves</t>
         </is>
       </c>
       <c r="F673" s="65" t="inlineStr">
@@ -43874,7 +43874,7 @@
       </c>
       <c r="I673" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/step-by-step-directions-from-a-binary-tree-node-to-another/</t>
+          <t>https://leetcode.com/problems/lowest-common-ancestor-of-deepest-leaves/</t>
         </is>
       </c>
       <c r="J673" s="65" t="inlineStr">
@@ -43916,7 +43916,7 @@
       </c>
       <c r="E674" s="65" t="inlineStr">
         <is>
-          <t>LCA of a Binary Tree with Parent Pointers</t>
+          <t>Step-By-Step Directions From a Binary Tree Node to Another</t>
         </is>
       </c>
       <c r="F674" s="65" t="inlineStr">
@@ -43931,12 +43931,12 @@
       </c>
       <c r="H674" s="65" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I674" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/search/?q=LCA+of+a+Binary+Tree+with+Parent+Pointers</t>
+          <t>https://leetcode.com/problems/step-by-step-directions-from-a-binary-tree-node-to-another/</t>
         </is>
       </c>
       <c r="J674" s="65" t="inlineStr">
@@ -43973,12 +43973,12 @@
       </c>
       <c r="D675" s="65" t="inlineStr">
         <is>
-          <t>Distance</t>
+          <t>LCA</t>
         </is>
       </c>
       <c r="E675" s="65" t="inlineStr">
         <is>
-          <t>Distance Between Two Nodes of a Binary Tree</t>
+          <t>LCA of a Binary Tree with Parent Pointers</t>
         </is>
       </c>
       <c r="F675" s="65" t="inlineStr">
@@ -43998,7 +43998,7 @@
       </c>
       <c r="I675" s="65" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/search/?q=Distance+Between+Two+Nodes+of+a+Binary+Tree</t>
+          <t>https://www.geeksforgeeks.org/search/?q=LCA+of+a+Binary+Tree+with+Parent+Pointers</t>
         </is>
       </c>
       <c r="J675" s="65" t="inlineStr">
@@ -44040,7 +44040,7 @@
       </c>
       <c r="E676" s="65" t="inlineStr">
         <is>
-          <t>Closest Leaf in a Binary Tree</t>
+          <t>Distance Between Two Nodes of a Binary Tree</t>
         </is>
       </c>
       <c r="F676" s="65" t="inlineStr">
@@ -44055,12 +44055,12 @@
       </c>
       <c r="H676" s="65" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I676" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/closest-leaf-in-a-binary-tree/</t>
+          <t>https://www.geeksforgeeks.org/search/?q=Distance+Between+Two+Nodes+of+a+Binary+Tree</t>
         </is>
       </c>
       <c r="J676" s="65" t="inlineStr">
@@ -44097,12 +44097,12 @@
       </c>
       <c r="D677" s="65" t="inlineStr">
         <is>
-          <t>Serialization</t>
+          <t>Distance</t>
         </is>
       </c>
       <c r="E677" s="65" t="inlineStr">
         <is>
-          <t>Serialize and Deserialize BST</t>
+          <t>Closest Leaf in a Binary Tree</t>
         </is>
       </c>
       <c r="F677" s="65" t="inlineStr">
@@ -44122,7 +44122,7 @@
       </c>
       <c r="I677" s="65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/serialize-and-deserialize-bst/</t>
+          <t>https://leetcode.com/problems/closest-leaf-in-a-binary-tree/</t>
         </is>
       </c>
       <c r="J677" s="65" t="inlineStr">
@@ -60329,7 +60329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H177"/>
+  <dimension ref="A1:H176"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" style="31" min="2" max="2"/>
@@ -63819,12 +63819,12 @@
     <row r="113" ht="15" customHeight="1" s="32">
       <c r="B113" s="42" t="inlineStr">
         <is>
-          <t>16. Greedy</t>
+          <t>17. Backtracking</t>
         </is>
       </c>
       <c r="C113" s="42" t="inlineStr">
         <is>
-          <t>Interval greedy</t>
+          <t>Expression</t>
         </is>
       </c>
       <c r="D113" s="43">
@@ -63856,7 +63856,7 @@
       </c>
       <c r="C114" s="42" t="inlineStr">
         <is>
-          <t>Expression</t>
+          <t>Bitmask assignment</t>
         </is>
       </c>
       <c r="D114" s="43">
@@ -63883,12 +63883,12 @@
     <row r="115" ht="15" customHeight="1" s="32">
       <c r="B115" s="42" t="inlineStr">
         <is>
-          <t>17. Backtracking</t>
+          <t>15. Intervals</t>
         </is>
       </c>
       <c r="C115" s="42" t="inlineStr">
         <is>
-          <t>Bitmask assignment</t>
+          <t>Streaming</t>
         </is>
       </c>
       <c r="D115" s="43">
@@ -63915,12 +63915,12 @@
     <row r="116" ht="15" customHeight="1" s="32">
       <c r="B116" s="42" t="inlineStr">
         <is>
-          <t>15. Intervals</t>
+          <t>17. Backtracking</t>
         </is>
       </c>
       <c r="C116" s="42" t="inlineStr">
         <is>
-          <t>Streaming</t>
+          <t>Greedy + backtracking</t>
         </is>
       </c>
       <c r="D116" s="43">
@@ -63947,12 +63947,12 @@
     <row r="117" ht="15" customHeight="1" s="32">
       <c r="B117" s="42" t="inlineStr">
         <is>
-          <t>17. Backtracking</t>
+          <t>18. Trees &amp; BST</t>
         </is>
       </c>
       <c r="C117" s="42" t="inlineStr">
         <is>
-          <t>Greedy + backtracking</t>
+          <t>Traversal</t>
         </is>
       </c>
       <c r="D117" s="43">
@@ -63984,7 +63984,7 @@
       </c>
       <c r="C118" s="42" t="inlineStr">
         <is>
-          <t>Traversal</t>
+          <t>Depth &amp; balance</t>
         </is>
       </c>
       <c r="D118" s="43">
@@ -64016,7 +64016,7 @@
       </c>
       <c r="C119" s="42" t="inlineStr">
         <is>
-          <t>Depth &amp; balance</t>
+          <t>Structure</t>
         </is>
       </c>
       <c r="D119" s="43">
@@ -64048,7 +64048,7 @@
       </c>
       <c r="C120" s="42" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>BFS</t>
         </is>
       </c>
       <c r="D120" s="43">
@@ -64080,7 +64080,7 @@
       </c>
       <c r="C121" s="42" t="inlineStr">
         <is>
-          <t>BFS</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="D121" s="43">
@@ -64112,7 +64112,7 @@
       </c>
       <c r="C122" s="42" t="inlineStr">
         <is>
-          <t>Views</t>
+          <t>Path sum</t>
         </is>
       </c>
       <c r="D122" s="43">
@@ -64144,7 +64144,7 @@
       </c>
       <c r="C123" s="42" t="inlineStr">
         <is>
-          <t>Path sum</t>
+          <t>Construction</t>
         </is>
       </c>
       <c r="D123" s="43">
@@ -64176,7 +64176,7 @@
       </c>
       <c r="C124" s="42" t="inlineStr">
         <is>
-          <t>Construction</t>
+          <t>LCA</t>
         </is>
       </c>
       <c r="D124" s="43">
@@ -64208,7 +64208,7 @@
       </c>
       <c r="C125" s="42" t="inlineStr">
         <is>
-          <t>LCA</t>
+          <t>Distance</t>
         </is>
       </c>
       <c r="D125" s="43">
@@ -64240,7 +64240,7 @@
       </c>
       <c r="C126" s="42" t="inlineStr">
         <is>
-          <t>Distance</t>
+          <t>BST basics</t>
         </is>
       </c>
       <c r="D126" s="43">
@@ -64272,7 +64272,7 @@
       </c>
       <c r="C127" s="42" t="inlineStr">
         <is>
-          <t>BST basics</t>
+          <t>BST properties</t>
         </is>
       </c>
       <c r="D127" s="43">
@@ -64299,12 +64299,12 @@
     <row r="128" ht="15" customHeight="1" s="32">
       <c r="B128" s="42" t="inlineStr">
         <is>
-          <t>18. Trees &amp; BST</t>
+          <t>19. Tries</t>
         </is>
       </c>
       <c r="C128" s="42" t="inlineStr">
         <is>
-          <t>BST properties</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="D128" s="43">
@@ -64336,7 +64336,7 @@
       </c>
       <c r="C129" s="42" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Prefix search</t>
         </is>
       </c>
       <c r="D129" s="43">
@@ -64368,7 +64368,7 @@
       </c>
       <c r="C130" s="42" t="inlineStr">
         <is>
-          <t>Prefix search</t>
+          <t>Counting</t>
         </is>
       </c>
       <c r="D130" s="43">
@@ -64400,7 +64400,7 @@
       </c>
       <c r="C131" s="42" t="inlineStr">
         <is>
-          <t>Counting</t>
+          <t>Trie + grid</t>
         </is>
       </c>
       <c r="D131" s="43">
@@ -64432,7 +64432,7 @@
       </c>
       <c r="C132" s="42" t="inlineStr">
         <is>
-          <t>Trie + grid</t>
+          <t>Bit trie</t>
         </is>
       </c>
       <c r="D132" s="43">
@@ -64459,12 +64459,12 @@
     <row r="133" ht="15" customHeight="1" s="32">
       <c r="B133" s="42" t="inlineStr">
         <is>
-          <t>19. Tries</t>
+          <t>20. Graphs</t>
         </is>
       </c>
       <c r="C133" s="42" t="inlineStr">
         <is>
-          <t>Bit trie</t>
+          <t>Representation</t>
         </is>
       </c>
       <c r="D133" s="43">
@@ -64496,7 +64496,7 @@
       </c>
       <c r="C134" s="42" t="inlineStr">
         <is>
-          <t>Representation</t>
+          <t>Traversal</t>
         </is>
       </c>
       <c r="D134" s="43">
@@ -64528,7 +64528,7 @@
       </c>
       <c r="C135" s="42" t="inlineStr">
         <is>
-          <t>Traversal</t>
+          <t>Grid DFS/BFS</t>
         </is>
       </c>
       <c r="D135" s="43">
@@ -64560,7 +64560,7 @@
       </c>
       <c r="C136" s="42" t="inlineStr">
         <is>
-          <t>Grid DFS/BFS</t>
+          <t>Multi-source BFS</t>
         </is>
       </c>
       <c r="D136" s="43">
@@ -64592,7 +64592,7 @@
       </c>
       <c r="C137" s="42" t="inlineStr">
         <is>
-          <t>Multi-source BFS</t>
+          <t>Connected components</t>
         </is>
       </c>
       <c r="D137" s="43">
@@ -64624,7 +64624,7 @@
       </c>
       <c r="C138" s="42" t="inlineStr">
         <is>
-          <t>Connected components</t>
+          <t>Coloring</t>
         </is>
       </c>
       <c r="D138" s="43">
@@ -64656,7 +64656,7 @@
       </c>
       <c r="C139" s="42" t="inlineStr">
         <is>
-          <t>Coloring</t>
+          <t>Cycle detection</t>
         </is>
       </c>
       <c r="D139" s="43">
@@ -64688,7 +64688,7 @@
       </c>
       <c r="C140" s="42" t="inlineStr">
         <is>
-          <t>Cycle detection</t>
+          <t>BFS shortest path</t>
         </is>
       </c>
       <c r="D140" s="43">
@@ -64720,7 +64720,7 @@
       </c>
       <c r="C141" s="42" t="inlineStr">
         <is>
-          <t>BFS shortest path</t>
+          <t>Topological sort</t>
         </is>
       </c>
       <c r="D141" s="43">
@@ -64752,7 +64752,7 @@
       </c>
       <c r="C142" s="42" t="inlineStr">
         <is>
-          <t>Topological sort</t>
+          <t>DSU</t>
         </is>
       </c>
       <c r="D142" s="43">
@@ -64784,7 +64784,7 @@
       </c>
       <c r="C143" s="42" t="inlineStr">
         <is>
-          <t>DSU</t>
+          <t>Dijkstra</t>
         </is>
       </c>
       <c r="D143" s="43">
@@ -64816,7 +64816,7 @@
       </c>
       <c r="C144" s="42" t="inlineStr">
         <is>
-          <t>Dijkstra</t>
+          <t>Bellman-Ford</t>
         </is>
       </c>
       <c r="D144" s="43">
@@ -64848,7 +64848,7 @@
       </c>
       <c r="C145" s="42" t="inlineStr">
         <is>
-          <t>Bellman-Ford</t>
+          <t>Floyd-Warshall</t>
         </is>
       </c>
       <c r="D145" s="43">
@@ -64880,7 +64880,7 @@
       </c>
       <c r="C146" s="42" t="inlineStr">
         <is>
-          <t>Floyd-Warshall</t>
+          <t>MST</t>
         </is>
       </c>
       <c r="D146" s="43">
@@ -64912,7 +64912,7 @@
       </c>
       <c r="C147" s="42" t="inlineStr">
         <is>
-          <t>MST</t>
+          <t>Misc</t>
         </is>
       </c>
       <c r="D147" s="43">
@@ -64939,12 +64939,12 @@
     <row r="148" ht="15" customHeight="1" s="32">
       <c r="B148" s="42" t="inlineStr">
         <is>
-          <t>20. Graphs</t>
+          <t>18. Trees &amp; BST</t>
         </is>
       </c>
       <c r="C148" s="42" t="inlineStr">
         <is>
-          <t>Misc</t>
+          <t>Serialization</t>
         </is>
       </c>
       <c r="D148" s="43">
@@ -64971,12 +64971,12 @@
     <row r="149" ht="15" customHeight="1" s="32">
       <c r="B149" s="42" t="inlineStr">
         <is>
-          <t>18. Trees &amp; BST</t>
+          <t>20. Graphs</t>
         </is>
       </c>
       <c r="C149" s="42" t="inlineStr">
         <is>
-          <t>Serialization</t>
+          <t>Bridges &amp; APs</t>
         </is>
       </c>
       <c r="D149" s="43">
@@ -65008,7 +65008,7 @@
       </c>
       <c r="C150" s="42" t="inlineStr">
         <is>
-          <t>Bridges &amp; APs</t>
+          <t>SCC</t>
         </is>
       </c>
       <c r="D150" s="43">
@@ -65040,7 +65040,7 @@
       </c>
       <c r="C151" s="42" t="inlineStr">
         <is>
-          <t>SCC</t>
+          <t>Euler path</t>
         </is>
       </c>
       <c r="D151" s="43">
@@ -65072,7 +65072,7 @@
       </c>
       <c r="C152" s="42" t="inlineStr">
         <is>
-          <t>Euler path</t>
+          <t>0-1 BFS</t>
         </is>
       </c>
       <c r="D152" s="43">
@@ -65104,7 +65104,7 @@
       </c>
       <c r="C153" s="42" t="inlineStr">
         <is>
-          <t>0-1 BFS</t>
+          <t>Binary lifting</t>
         </is>
       </c>
       <c r="D153" s="43">
@@ -65131,12 +65131,12 @@
     <row r="154" ht="15" customHeight="1" s="32">
       <c r="B154" s="42" t="inlineStr">
         <is>
-          <t>20. Graphs</t>
+          <t>21. Dynamic Programming</t>
         </is>
       </c>
       <c r="C154" s="42" t="inlineStr">
         <is>
-          <t>Binary lifting</t>
+          <t>1D DP</t>
         </is>
       </c>
       <c r="D154" s="43">
@@ -65168,7 +65168,7 @@
       </c>
       <c r="C155" s="42" t="inlineStr">
         <is>
-          <t>1D DP</t>
+          <t>Grid DP</t>
         </is>
       </c>
       <c r="D155" s="43">
@@ -65200,7 +65200,7 @@
       </c>
       <c r="C156" s="42" t="inlineStr">
         <is>
-          <t>Grid DP</t>
+          <t>0/1 Knapsack</t>
         </is>
       </c>
       <c r="D156" s="43">
@@ -65232,7 +65232,7 @@
       </c>
       <c r="C157" s="42" t="inlineStr">
         <is>
-          <t>0/1 Knapsack</t>
+          <t>Unbounded Knapsack</t>
         </is>
       </c>
       <c r="D157" s="43">
@@ -65264,7 +65264,7 @@
       </c>
       <c r="C158" s="42" t="inlineStr">
         <is>
-          <t>Unbounded Knapsack</t>
+          <t>LIS</t>
         </is>
       </c>
       <c r="D158" s="43">
@@ -65296,7 +65296,7 @@
       </c>
       <c r="C159" s="42" t="inlineStr">
         <is>
-          <t>LIS</t>
+          <t>Stocks DP</t>
         </is>
       </c>
       <c r="D159" s="43">
@@ -65328,7 +65328,7 @@
       </c>
       <c r="C160" s="42" t="inlineStr">
         <is>
-          <t>Stocks DP</t>
+          <t>Squares in matrix</t>
         </is>
       </c>
       <c r="D160" s="43">
@@ -65360,7 +65360,7 @@
       </c>
       <c r="C161" s="42" t="inlineStr">
         <is>
-          <t>Squares in matrix</t>
+          <t>String DP</t>
         </is>
       </c>
       <c r="D161" s="43">
@@ -65392,7 +65392,7 @@
       </c>
       <c r="C162" s="42" t="inlineStr">
         <is>
-          <t>String DP</t>
+          <t>Partition DP</t>
         </is>
       </c>
       <c r="D162" s="43">
@@ -65424,7 +65424,7 @@
       </c>
       <c r="C163" s="42" t="inlineStr">
         <is>
-          <t>Partition DP</t>
+          <t>DP on trees</t>
         </is>
       </c>
       <c r="D163" s="43">
@@ -65456,7 +65456,7 @@
       </c>
       <c r="C164" s="42" t="inlineStr">
         <is>
-          <t>DP on trees</t>
+          <t>Game DP</t>
         </is>
       </c>
       <c r="D164" s="43">
@@ -65488,7 +65488,7 @@
       </c>
       <c r="C165" s="42" t="inlineStr">
         <is>
-          <t>Game DP</t>
+          <t>Counting DP</t>
         </is>
       </c>
       <c r="D165" s="43">
@@ -65515,12 +65515,12 @@
     <row r="166" ht="15" customHeight="1" s="32">
       <c r="B166" s="42" t="inlineStr">
         <is>
-          <t>21. Dynamic Programming</t>
+          <t>22. Design</t>
         </is>
       </c>
       <c r="C166" s="42" t="inlineStr">
         <is>
-          <t>Counting DP</t>
+          <t>Hash structures</t>
         </is>
       </c>
       <c r="D166" s="43">
@@ -65552,7 +65552,7 @@
       </c>
       <c r="C167" s="42" t="inlineStr">
         <is>
-          <t>Hash structures</t>
+          <t>Cache</t>
         </is>
       </c>
       <c r="D167" s="43">
@@ -65584,7 +65584,7 @@
       </c>
       <c r="C168" s="42" t="inlineStr">
         <is>
-          <t>Cache</t>
+          <t>Systems</t>
         </is>
       </c>
       <c r="D168" s="43">
@@ -65616,7 +65616,7 @@
       </c>
       <c r="C169" s="42" t="inlineStr">
         <is>
-          <t>Systems</t>
+          <t>Versioned data</t>
         </is>
       </c>
       <c r="D169" s="43">
@@ -65648,7 +65648,7 @@
       </c>
       <c r="C170" s="42" t="inlineStr">
         <is>
-          <t>Versioned data</t>
+          <t>Randomized / sampling</t>
         </is>
       </c>
       <c r="D170" s="43">
@@ -65675,12 +65675,12 @@
     <row r="171" ht="15" customHeight="1" s="32">
       <c r="B171" s="42" t="inlineStr">
         <is>
-          <t>22. Design</t>
+          <t>23. Advanced DS</t>
         </is>
       </c>
       <c r="C171" s="42" t="inlineStr">
         <is>
-          <t>Randomized / sampling</t>
+          <t>Fenwick tree</t>
         </is>
       </c>
       <c r="D171" s="43">
@@ -65712,7 +65712,7 @@
       </c>
       <c r="C172" s="42" t="inlineStr">
         <is>
-          <t>Fenwick tree</t>
+          <t>Segment tree</t>
         </is>
       </c>
       <c r="D172" s="43">
@@ -65744,7 +65744,7 @@
       </c>
       <c r="C173" s="42" t="inlineStr">
         <is>
-          <t>Segment tree</t>
+          <t>Sparse table</t>
         </is>
       </c>
       <c r="D173" s="43">
@@ -65776,7 +65776,7 @@
       </c>
       <c r="C174" s="42" t="inlineStr">
         <is>
-          <t>Sparse table</t>
+          <t>Sweep line</t>
         </is>
       </c>
       <c r="D174" s="43">
@@ -65808,7 +65808,7 @@
       </c>
       <c r="C175" s="42" t="inlineStr">
         <is>
-          <t>Sweep line</t>
+          <t>Ordered set</t>
         </is>
       </c>
       <c r="D175" s="43">
@@ -65835,12 +65835,12 @@
     <row r="176" ht="15" customHeight="1" s="32">
       <c r="B176" s="42" t="inlineStr">
         <is>
-          <t>23. Advanced DS</t>
+          <t>21. Dynamic Programming</t>
         </is>
       </c>
       <c r="C176" s="42" t="inlineStr">
         <is>
-          <t>Ordered set</t>
+          <t>Bitmask DP</t>
         </is>
       </c>
       <c r="D176" s="43">
@@ -65864,41 +65864,9 @@
         <v/>
       </c>
     </row>
-    <row r="177" ht="15" customHeight="1" s="32">
-      <c r="B177" s="42" t="inlineStr">
-        <is>
-          <t>21. Dynamic Programming</t>
-        </is>
-      </c>
-      <c r="C177" s="42" t="inlineStr">
-        <is>
-          <t>Bitmask DP</t>
-        </is>
-      </c>
-      <c r="D177" s="43">
-        <f>COUNTIFS(Master!$C$2:$C$918,$B177,Master!$D$2:$D$918,$C177)</f>
-        <v/>
-      </c>
-      <c r="E177" s="43">
-        <f>COUNTIFS(Master!$C$2:$C$918,$B177,Master!$D$2:$D$918,$C177,Master!$G$2:$G$918,"Core")</f>
-        <v/>
-      </c>
-      <c r="F177" s="43">
-        <f>COUNTIFS(Master!$C$2:$C$918,$B177,Master!$D$2:$D$918,$C177,Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,$B177,Master!$D$2:$D$918,$C177,Master!$J$2:$J$918,"Mastered")</f>
-        <v/>
-      </c>
-      <c r="G177" s="56">
-        <f>IFERROR(AVERAGEIFS(Master!$K$2:$K$918,Master!$C$2:$C$918,$B177,Master!$D$2:$D$918,$C177,Master!$K$2:$K$918,"&gt;0"),"")</f>
-        <v/>
-      </c>
-      <c r="H177" s="46">
-        <f>IF($F177=0,"Untouched",IF($G177="","No rating",IF($G177&lt;=3,"Weak","Solid")))</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="B5:H177"/>
-  <conditionalFormatting sqref="H6:H177">
+  <autoFilter ref="B5:H176"/>
+  <conditionalFormatting sqref="H6:H176">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="equal" aboveAverage="0" dxfId="17" text="" percent="0" bottom="0">
       <formula>"Untouched"</formula>
     </cfRule>
@@ -65921,7 +65889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E173"/>
+  <dimension ref="A1:E172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="32" min="1" max="1"/>
@@ -67821,7 +67789,7 @@
         <v>3</v>
       </c>
       <c r="D90" s="31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E90" s="31" t="n">
         <v>2</v>
@@ -68208,22 +68176,22 @@
     <row r="109">
       <c r="A109" s="31" t="inlineStr">
         <is>
-          <t>16. Greedy</t>
+          <t>17. Backtracking</t>
         </is>
       </c>
       <c r="B109" s="31" t="inlineStr">
         <is>
-          <t>Interval greedy</t>
+          <t>Expression</t>
         </is>
       </c>
       <c r="C109" s="31" t="n">
         <v>0</v>
       </c>
       <c r="D109" s="31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E109" s="31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="110">
@@ -68234,49 +68202,49 @@
       </c>
       <c r="B110" s="31" t="inlineStr">
         <is>
-          <t>Expression</t>
+          <t>Bitmask assignment</t>
         </is>
       </c>
       <c r="C110" s="31" t="n">
         <v>0</v>
       </c>
       <c r="D110" s="31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E110" s="31" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="31" t="inlineStr">
         <is>
-          <t>17. Backtracking</t>
+          <t>15. Intervals</t>
         </is>
       </c>
       <c r="B111" s="31" t="inlineStr">
         <is>
-          <t>Bitmask assignment</t>
+          <t>Streaming</t>
         </is>
       </c>
       <c r="C111" s="31" t="n">
         <v>0</v>
       </c>
       <c r="D111" s="31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E111" s="31" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="31" t="inlineStr">
         <is>
-          <t>15. Intervals</t>
+          <t>17. Backtracking</t>
         </is>
       </c>
       <c r="B112" s="31" t="inlineStr">
         <is>
-          <t>Streaming</t>
+          <t>Greedy + backtracking</t>
         </is>
       </c>
       <c r="C112" s="31" t="n">
@@ -68286,28 +68254,28 @@
         <v>0</v>
       </c>
       <c r="E112" s="31" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="31" t="inlineStr">
         <is>
-          <t>17. Backtracking</t>
+          <t>18. Trees &amp; BST</t>
         </is>
       </c>
       <c r="B113" s="31" t="inlineStr">
         <is>
-          <t>Greedy + backtracking</t>
+          <t>Traversal</t>
         </is>
       </c>
       <c r="C113" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D113" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E113" s="31" t="n">
         <v>0</v>
-      </c>
-      <c r="D113" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="E113" s="31" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="114">
@@ -68318,14 +68286,14 @@
       </c>
       <c r="B114" s="31" t="inlineStr">
         <is>
-          <t>Traversal</t>
+          <t>Depth &amp; balance</t>
         </is>
       </c>
       <c r="C114" s="31" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D114" s="31" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E114" s="31" t="n">
         <v>0</v>
@@ -68339,14 +68307,14 @@
       </c>
       <c r="B115" s="31" t="inlineStr">
         <is>
-          <t>Depth &amp; balance</t>
+          <t>Structure</t>
         </is>
       </c>
       <c r="C115" s="31" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D115" s="31" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E115" s="31" t="n">
         <v>0</v>
@@ -68360,14 +68328,14 @@
       </c>
       <c r="B116" s="31" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>BFS</t>
         </is>
       </c>
       <c r="C116" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="D116" s="31" t="n">
         <v>4</v>
-      </c>
-      <c r="D116" s="31" t="n">
-        <v>3</v>
       </c>
       <c r="E116" s="31" t="n">
         <v>0</v>
@@ -68381,17 +68349,17 @@
       </c>
       <c r="B117" s="31" t="inlineStr">
         <is>
-          <t>BFS</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="C117" s="31" t="n">
         <v>2</v>
       </c>
       <c r="D117" s="31" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E117" s="31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="118">
@@ -68402,11 +68370,11 @@
       </c>
       <c r="B118" s="31" t="inlineStr">
         <is>
-          <t>Views</t>
+          <t>Path sum</t>
         </is>
       </c>
       <c r="C118" s="31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D118" s="31" t="n">
         <v>2</v>
@@ -68423,17 +68391,17 @@
       </c>
       <c r="B119" s="31" t="inlineStr">
         <is>
-          <t>Path sum</t>
+          <t>Construction</t>
         </is>
       </c>
       <c r="C119" s="31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D119" s="31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E119" s="31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="120">
@@ -68444,14 +68412,14 @@
       </c>
       <c r="B120" s="31" t="inlineStr">
         <is>
-          <t>Construction</t>
+          <t>LCA</t>
         </is>
       </c>
       <c r="C120" s="31" t="n">
         <v>2</v>
       </c>
       <c r="D120" s="31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E120" s="31" t="n">
         <v>0</v>
@@ -68465,14 +68433,14 @@
       </c>
       <c r="B121" s="31" t="inlineStr">
         <is>
-          <t>LCA</t>
+          <t>Distance</t>
         </is>
       </c>
       <c r="C121" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D121" s="31" t="n">
         <v>2</v>
-      </c>
-      <c r="D121" s="31" t="n">
-        <v>3</v>
       </c>
       <c r="E121" s="31" t="n">
         <v>0</v>
@@ -68486,14 +68454,14 @@
       </c>
       <c r="B122" s="31" t="inlineStr">
         <is>
-          <t>Distance</t>
+          <t>BST basics</t>
         </is>
       </c>
       <c r="C122" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="D122" s="31" t="n">
         <v>3</v>
-      </c>
-      <c r="D122" s="31" t="n">
-        <v>2</v>
       </c>
       <c r="E122" s="31" t="n">
         <v>0</v>
@@ -68507,35 +68475,35 @@
       </c>
       <c r="B123" s="31" t="inlineStr">
         <is>
-          <t>BST basics</t>
+          <t>BST properties</t>
         </is>
       </c>
       <c r="C123" s="31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D123" s="31" t="n">
         <v>3</v>
       </c>
       <c r="E123" s="31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="31" t="inlineStr">
         <is>
-          <t>18. Trees &amp; BST</t>
+          <t>19. Tries</t>
         </is>
       </c>
       <c r="B124" s="31" t="inlineStr">
         <is>
-          <t>BST properties</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="C124" s="31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D124" s="31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E124" s="31" t="n">
         <v>1</v>
@@ -68549,7 +68517,7 @@
       </c>
       <c r="B125" s="31" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Prefix search</t>
         </is>
       </c>
       <c r="C125" s="31" t="n">
@@ -68570,14 +68538,14 @@
       </c>
       <c r="B126" s="31" t="inlineStr">
         <is>
-          <t>Prefix search</t>
+          <t>Counting</t>
         </is>
       </c>
       <c r="C126" s="31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D126" s="31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E126" s="31" t="n">
         <v>1</v>
@@ -68591,17 +68559,17 @@
       </c>
       <c r="B127" s="31" t="inlineStr">
         <is>
-          <t>Counting</t>
+          <t>Trie + grid</t>
         </is>
       </c>
       <c r="C127" s="31" t="n">
         <v>1</v>
       </c>
       <c r="D127" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E127" s="31" t="n">
         <v>3</v>
-      </c>
-      <c r="E127" s="31" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="128">
@@ -68612,14 +68580,14 @@
       </c>
       <c r="B128" s="31" t="inlineStr">
         <is>
-          <t>Trie + grid</t>
+          <t>Bit trie</t>
         </is>
       </c>
       <c r="C128" s="31" t="n">
         <v>1</v>
       </c>
       <c r="D128" s="31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E128" s="31" t="n">
         <v>3</v>
@@ -68628,22 +68596,22 @@
     <row r="129">
       <c r="A129" s="31" t="inlineStr">
         <is>
-          <t>19. Tries</t>
+          <t>20. Graphs</t>
         </is>
       </c>
       <c r="B129" s="31" t="inlineStr">
         <is>
-          <t>Bit trie</t>
+          <t>Representation</t>
         </is>
       </c>
       <c r="C129" s="31" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D129" s="31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E129" s="31" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="130">
@@ -68654,14 +68622,14 @@
       </c>
       <c r="B130" s="31" t="inlineStr">
         <is>
-          <t>Representation</t>
+          <t>Traversal</t>
         </is>
       </c>
       <c r="C130" s="31" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D130" s="31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E130" s="31" t="n">
         <v>0</v>
@@ -68675,14 +68643,14 @@
       </c>
       <c r="B131" s="31" t="inlineStr">
         <is>
-          <t>Traversal</t>
+          <t>Grid DFS/BFS</t>
         </is>
       </c>
       <c r="C131" s="31" t="n">
         <v>4</v>
       </c>
       <c r="D131" s="31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E131" s="31" t="n">
         <v>0</v>
@@ -68696,11 +68664,11 @@
       </c>
       <c r="B132" s="31" t="inlineStr">
         <is>
-          <t>Grid DFS/BFS</t>
+          <t>Multi-source BFS</t>
         </is>
       </c>
       <c r="C132" s="31" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D132" s="31" t="n">
         <v>3</v>
@@ -68717,14 +68685,14 @@
       </c>
       <c r="B133" s="31" t="inlineStr">
         <is>
-          <t>Multi-source BFS</t>
+          <t>Connected components</t>
         </is>
       </c>
       <c r="C133" s="31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D133" s="31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E133" s="31" t="n">
         <v>0</v>
@@ -68738,17 +68706,17 @@
       </c>
       <c r="B134" s="31" t="inlineStr">
         <is>
-          <t>Connected components</t>
+          <t>Coloring</t>
         </is>
       </c>
       <c r="C134" s="31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D134" s="31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E134" s="31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="135">
@@ -68759,14 +68727,14 @@
       </c>
       <c r="B135" s="31" t="inlineStr">
         <is>
-          <t>Coloring</t>
+          <t>Cycle detection</t>
         </is>
       </c>
       <c r="C135" s="31" t="n">
         <v>2</v>
       </c>
       <c r="D135" s="31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E135" s="31" t="n">
         <v>2</v>
@@ -68780,7 +68748,7 @@
       </c>
       <c r="B136" s="31" t="inlineStr">
         <is>
-          <t>Cycle detection</t>
+          <t>BFS shortest path</t>
         </is>
       </c>
       <c r="C136" s="31" t="n">
@@ -68801,17 +68769,17 @@
       </c>
       <c r="B137" s="31" t="inlineStr">
         <is>
-          <t>BFS shortest path</t>
+          <t>Topological sort</t>
         </is>
       </c>
       <c r="C137" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D137" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="D137" s="31" t="n">
+      <c r="E137" s="31" t="n">
         <v>1</v>
-      </c>
-      <c r="E137" s="31" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="138">
@@ -68822,17 +68790,17 @@
       </c>
       <c r="B138" s="31" t="inlineStr">
         <is>
-          <t>Topological sort</t>
+          <t>DSU</t>
         </is>
       </c>
       <c r="C138" s="31" t="n">
         <v>3</v>
       </c>
       <c r="D138" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="E138" s="31" t="n">
         <v>2</v>
-      </c>
-      <c r="E138" s="31" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="139">
@@ -68843,17 +68811,17 @@
       </c>
       <c r="B139" s="31" t="inlineStr">
         <is>
-          <t>DSU</t>
+          <t>Dijkstra</t>
         </is>
       </c>
       <c r="C139" s="31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D139" s="31" t="n">
         <v>3</v>
       </c>
       <c r="E139" s="31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="140">
@@ -68864,14 +68832,14 @@
       </c>
       <c r="B140" s="31" t="inlineStr">
         <is>
-          <t>Dijkstra</t>
+          <t>Bellman-Ford</t>
         </is>
       </c>
       <c r="C140" s="31" t="n">
         <v>2</v>
       </c>
       <c r="D140" s="31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E140" s="31" t="n">
         <v>1</v>
@@ -68885,17 +68853,17 @@
       </c>
       <c r="B141" s="31" t="inlineStr">
         <is>
-          <t>Bellman-Ford</t>
+          <t>Floyd-Warshall</t>
         </is>
       </c>
       <c r="C141" s="31" t="n">
         <v>2</v>
       </c>
       <c r="D141" s="31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E141" s="31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="142">
@@ -68906,17 +68874,17 @@
       </c>
       <c r="B142" s="31" t="inlineStr">
         <is>
-          <t>Floyd-Warshall</t>
+          <t>MST</t>
         </is>
       </c>
       <c r="C142" s="31" t="n">
         <v>2</v>
       </c>
       <c r="D142" s="31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E142" s="31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="143">
@@ -68927,35 +68895,35 @@
       </c>
       <c r="B143" s="31" t="inlineStr">
         <is>
-          <t>MST</t>
+          <t>Misc</t>
         </is>
       </c>
       <c r="C143" s="31" t="n">
         <v>2</v>
       </c>
       <c r="D143" s="31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E143" s="31" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="31" t="inlineStr">
         <is>
-          <t>20. Graphs</t>
+          <t>18. Trees &amp; BST</t>
         </is>
       </c>
       <c r="B144" s="31" t="inlineStr">
         <is>
-          <t>Misc</t>
+          <t>Serialization</t>
         </is>
       </c>
       <c r="C144" s="31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D144" s="31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E144" s="31" t="n">
         <v>0</v>
@@ -68964,22 +68932,22 @@
     <row r="145">
       <c r="A145" s="31" t="inlineStr">
         <is>
-          <t>18. Trees &amp; BST</t>
+          <t>20. Graphs</t>
         </is>
       </c>
       <c r="B145" s="31" t="inlineStr">
         <is>
-          <t>Serialization</t>
+          <t>Bridges &amp; APs</t>
         </is>
       </c>
       <c r="C145" s="31" t="n">
         <v>0</v>
       </c>
       <c r="D145" s="31" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E145" s="31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="146">
@@ -68990,17 +68958,17 @@
       </c>
       <c r="B146" s="31" t="inlineStr">
         <is>
-          <t>Bridges &amp; APs</t>
+          <t>SCC</t>
         </is>
       </c>
       <c r="C146" s="31" t="n">
         <v>0</v>
       </c>
       <c r="D146" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E146" s="31" t="n">
         <v>3</v>
-      </c>
-      <c r="E146" s="31" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="147">
@@ -69011,7 +68979,7 @@
       </c>
       <c r="B147" s="31" t="inlineStr">
         <is>
-          <t>SCC</t>
+          <t>Euler path</t>
         </is>
       </c>
       <c r="C147" s="31" t="n">
@@ -69032,7 +69000,7 @@
       </c>
       <c r="B148" s="31" t="inlineStr">
         <is>
-          <t>Euler path</t>
+          <t>0-1 BFS</t>
         </is>
       </c>
       <c r="C148" s="31" t="n">
@@ -69053,38 +69021,38 @@
       </c>
       <c r="B149" s="31" t="inlineStr">
         <is>
-          <t>0-1 BFS</t>
+          <t>Binary lifting</t>
         </is>
       </c>
       <c r="C149" s="31" t="n">
         <v>0</v>
       </c>
       <c r="D149" s="31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E149" s="31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="31" t="inlineStr">
         <is>
-          <t>20. Graphs</t>
+          <t>21. Dynamic Programming</t>
         </is>
       </c>
       <c r="B150" s="31" t="inlineStr">
         <is>
-          <t>Binary lifting</t>
+          <t>1D DP</t>
         </is>
       </c>
       <c r="C150" s="31" t="n">
+        <v>6</v>
+      </c>
+      <c r="D150" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="E150" s="31" t="n">
         <v>0</v>
-      </c>
-      <c r="D150" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="E150" s="31" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="151">
@@ -69095,17 +69063,17 @@
       </c>
       <c r="B151" s="31" t="inlineStr">
         <is>
-          <t>1D DP</t>
+          <t>Grid DP</t>
         </is>
       </c>
       <c r="C151" s="31" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D151" s="31" t="n">
         <v>3</v>
       </c>
       <c r="E151" s="31" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="152">
@@ -69116,17 +69084,17 @@
       </c>
       <c r="B152" s="31" t="inlineStr">
         <is>
-          <t>Grid DP</t>
+          <t>0/1 Knapsack</t>
         </is>
       </c>
       <c r="C152" s="31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D152" s="31" t="n">
         <v>3</v>
       </c>
       <c r="E152" s="31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="153">
@@ -69137,17 +69105,17 @@
       </c>
       <c r="B153" s="31" t="inlineStr">
         <is>
-          <t>0/1 Knapsack</t>
+          <t>Unbounded Knapsack</t>
         </is>
       </c>
       <c r="C153" s="31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D153" s="31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E153" s="31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="154">
@@ -69158,17 +69126,17 @@
       </c>
       <c r="B154" s="31" t="inlineStr">
         <is>
-          <t>Unbounded Knapsack</t>
+          <t>LIS</t>
         </is>
       </c>
       <c r="C154" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="D154" s="31" t="n">
         <v>4</v>
       </c>
-      <c r="D154" s="31" t="n">
-        <v>2</v>
-      </c>
       <c r="E154" s="31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="155">
@@ -69179,17 +69147,17 @@
       </c>
       <c r="B155" s="31" t="inlineStr">
         <is>
-          <t>LIS</t>
+          <t>Stocks DP</t>
         </is>
       </c>
       <c r="C155" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D155" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E155" s="31" t="n">
         <v>2</v>
-      </c>
-      <c r="D155" s="31" t="n">
-        <v>4</v>
-      </c>
-      <c r="E155" s="31" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="156">
@@ -69200,17 +69168,17 @@
       </c>
       <c r="B156" s="31" t="inlineStr">
         <is>
-          <t>Stocks DP</t>
+          <t>Squares in matrix</t>
         </is>
       </c>
       <c r="C156" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="D156" s="31" t="n">
         <v>3</v>
       </c>
-      <c r="D156" s="31" t="n">
+      <c r="E156" s="31" t="n">
         <v>0</v>
-      </c>
-      <c r="E156" s="31" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="157">
@@ -69221,17 +69189,17 @@
       </c>
       <c r="B157" s="31" t="inlineStr">
         <is>
-          <t>Squares in matrix</t>
+          <t>String DP</t>
         </is>
       </c>
       <c r="C157" s="31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D157" s="31" t="n">
         <v>3</v>
       </c>
       <c r="E157" s="31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="158">
@@ -69242,17 +69210,17 @@
       </c>
       <c r="B158" s="31" t="inlineStr">
         <is>
-          <t>String DP</t>
+          <t>Partition DP</t>
         </is>
       </c>
       <c r="C158" s="31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D158" s="31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E158" s="31" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="159">
@@ -69263,7 +69231,7 @@
       </c>
       <c r="B159" s="31" t="inlineStr">
         <is>
-          <t>Partition DP</t>
+          <t>DP on trees</t>
         </is>
       </c>
       <c r="C159" s="31" t="n">
@@ -69273,7 +69241,7 @@
         <v>1</v>
       </c>
       <c r="E159" s="31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="160">
@@ -69284,17 +69252,17 @@
       </c>
       <c r="B160" s="31" t="inlineStr">
         <is>
-          <t>DP on trees</t>
+          <t>Game DP</t>
         </is>
       </c>
       <c r="C160" s="31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D160" s="31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E160" s="31" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="161">
@@ -69305,38 +69273,38 @@
       </c>
       <c r="B161" s="31" t="inlineStr">
         <is>
-          <t>Game DP</t>
+          <t>Counting DP</t>
         </is>
       </c>
       <c r="C161" s="31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D161" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E161" s="31" t="n">
         <v>2</v>
-      </c>
-      <c r="E161" s="31" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="31" t="inlineStr">
         <is>
-          <t>21. Dynamic Programming</t>
+          <t>22. Design</t>
         </is>
       </c>
       <c r="B162" s="31" t="inlineStr">
         <is>
-          <t>Counting DP</t>
+          <t>Hash structures</t>
         </is>
       </c>
       <c r="C162" s="31" t="n">
         <v>2</v>
       </c>
       <c r="D162" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E162" s="31" t="n">
         <v>1</v>
-      </c>
-      <c r="E162" s="31" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="163">
@@ -69347,17 +69315,17 @@
       </c>
       <c r="B163" s="31" t="inlineStr">
         <is>
-          <t>Hash structures</t>
+          <t>Cache</t>
         </is>
       </c>
       <c r="C163" s="31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D163" s="31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E163" s="31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="164">
@@ -69368,14 +69336,14 @@
       </c>
       <c r="B164" s="31" t="inlineStr">
         <is>
-          <t>Cache</t>
+          <t>Systems</t>
         </is>
       </c>
       <c r="C164" s="31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D164" s="31" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E164" s="31" t="n">
         <v>0</v>
@@ -69389,17 +69357,17 @@
       </c>
       <c r="B165" s="31" t="inlineStr">
         <is>
-          <t>Systems</t>
+          <t>Versioned data</t>
         </is>
       </c>
       <c r="C165" s="31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D165" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E165" s="31" t="n">
         <v>2</v>
-      </c>
-      <c r="E165" s="31" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="166">
@@ -69410,41 +69378,41 @@
       </c>
       <c r="B166" s="31" t="inlineStr">
         <is>
-          <t>Versioned data</t>
+          <t>Randomized / sampling</t>
         </is>
       </c>
       <c r="C166" s="31" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D166" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="E166" s="31" t="n">
         <v>1</v>
-      </c>
-      <c r="E166" s="31" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="31" t="inlineStr">
         <is>
-          <t>22. Design</t>
+          <t>23. Advanced DS</t>
         </is>
       </c>
       <c r="B167" s="31" t="inlineStr">
         <is>
-          <t>Randomized / sampling</t>
+          <t>Fenwick tree</t>
         </is>
       </c>
       <c r="C167" s="31" t="n">
         <v>0</v>
       </c>
       <c r="D167" s="31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E167" s="31" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="168">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="168" s="32">
       <c r="A168" s="31" t="inlineStr">
         <is>
           <t>23. Advanced DS</t>
@@ -69452,7 +69420,7 @@
       </c>
       <c r="B168" s="31" t="inlineStr">
         <is>
-          <t>Fenwick tree</t>
+          <t>Segment tree</t>
         </is>
       </c>
       <c r="C168" s="31" t="n">
@@ -69462,7 +69430,7 @@
         <v>3</v>
       </c>
       <c r="E168" s="31" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="169" s="32">
@@ -69473,7 +69441,7 @@
       </c>
       <c r="B169" s="31" t="inlineStr">
         <is>
-          <t>Segment tree</t>
+          <t>Sparse table</t>
         </is>
       </c>
       <c r="C169" s="31" t="n">
@@ -69494,17 +69462,17 @@
       </c>
       <c r="B170" s="31" t="inlineStr">
         <is>
-          <t>Sparse table</t>
+          <t>Sweep line</t>
         </is>
       </c>
       <c r="C170" s="31" t="n">
         <v>0</v>
       </c>
       <c r="D170" s="31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E170" s="31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="171" s="32">
@@ -69515,7 +69483,7 @@
       </c>
       <c r="B171" s="31" t="inlineStr">
         <is>
-          <t>Sweep line</t>
+          <t>Ordered set</t>
         </is>
       </c>
       <c r="C171" s="31" t="n">
@@ -69531,42 +69499,21 @@
     <row r="172" s="32">
       <c r="A172" s="31" t="inlineStr">
         <is>
-          <t>23. Advanced DS</t>
+          <t>21. Dynamic Programming</t>
         </is>
       </c>
       <c r="B172" s="31" t="inlineStr">
         <is>
-          <t>Ordered set</t>
+          <t>Bitmask DP</t>
         </is>
       </c>
       <c r="C172" s="31" t="n">
         <v>0</v>
       </c>
       <c r="D172" s="31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E172" s="31" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="173" s="32">
-      <c r="A173" s="31" t="inlineStr">
-        <is>
-          <t>21. Dynamic Programming</t>
-        </is>
-      </c>
-      <c r="B173" s="31" t="inlineStr">
-        <is>
-          <t>Bitmask DP</t>
-        </is>
-      </c>
-      <c r="C173" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="D173" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="E173" s="31" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Move Count Inversions from Core to Depth
It asks you to modify merge sort to count something, a real jump from
implementing it, and it landed at step 13 before any array work. Core's
Divide & Conquer now runs Merge Sort, Quick Sort, Sort an Array; Count
Inversions opens phase 1 Depth at step 87.

Steps 14-87 shift up by one. The workbook follows: Master rows, Path Stages
ranges and topics, Pattern Coverage counts, and Core 387 on Start Here and
in the README.
</commit_message>
<xml_diff>
--- a/DSA_Master_Sheet.xlsx
+++ b/DSA_Master_Sheet.xlsx
@@ -899,7 +899,7 @@
     <row r="9" ht="27.75" customHeight="1" s="32">
       <c r="C9" s="36" t="inlineStr">
         <is>
-          <t>Core (388) - the main track. It deliberately skips the advanced patterns (SCC, Euler path, bridges and articulation points, binary lifting, bitmask DP, and everything in Advanced DS); those live in Depth and Stretch. This is your actual target.</t>
+          <t>Core (387) - the main track. It deliberately skips the advanced patterns (SCC, Euler path, bridges and articulation points, binary lifting, bitmask DP, and everything in Advanced DS); those live in Depth and Stretch. This is your actual target.</t>
         </is>
       </c>
     </row>
@@ -1217,17 +1217,17 @@
       </c>
       <c r="B2" s="31" t="inlineStr">
         <is>
-          <t>1-87</t>
+          <t>1-86</t>
         </is>
       </c>
       <c r="C2" s="31" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D2" s="31" t="n">
         <v>52</v>
       </c>
       <c r="E2" s="31" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F2" s="31" t="n">
         <v>1</v>
@@ -1246,24 +1246,24 @@
       </c>
       <c r="B3" s="31" t="inlineStr">
         <is>
-          <t>88-153</t>
+          <t>87-153</t>
         </is>
       </c>
       <c r="C3" s="31" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D3" s="31" t="n">
         <v>14</v>
       </c>
       <c r="E3" s="31" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F3" s="31" t="n">
         <v>1</v>
       </c>
       <c r="G3" s="31" t="inlineStr">
         <is>
-          <t>Arrays &amp; Two Pointers, Sorting &amp; Cyclic Sort, Hashing, Prefix Sum &amp; Kadane, Sliding Window</t>
+          <t>Basics &amp; Recursion, Arrays &amp; Two Pointers, Sorting &amp; Cyclic Sort, Hashing, Prefix Sum &amp; Kadane, Sliding Window</t>
         </is>
       </c>
     </row>
@@ -2996,7 +2996,7 @@
       </c>
       <c r="E14" s="61" t="inlineStr">
         <is>
-          <t>Count Inversions</t>
+          <t>Sort an Array</t>
         </is>
       </c>
       <c r="F14" s="61" t="inlineStr">
@@ -3011,12 +3011,12 @@
       </c>
       <c r="H14" s="61" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I14" s="61" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/inversion-of-array-1587115620/1</t>
+          <t>https://leetcode.com/problems/sort-an-array/</t>
         </is>
       </c>
       <c r="J14" s="61" t="inlineStr">
@@ -3048,22 +3048,22 @@
       </c>
       <c r="C15" s="61" t="inlineStr">
         <is>
-          <t>01. Basics &amp; Recursion</t>
+          <t>02. Arrays &amp; Two Pointers</t>
         </is>
       </c>
       <c r="D15" s="61" t="inlineStr">
         <is>
-          <t>Divide &amp; Conquer</t>
+          <t>Basics</t>
         </is>
       </c>
       <c r="E15" s="61" t="inlineStr">
         <is>
-          <t>Sort an Array</t>
+          <t>Remove Element</t>
         </is>
       </c>
       <c r="F15" s="61" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G15" s="61" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="I15" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/sort-an-array/</t>
+          <t>https://leetcode.com/problems/remove-element/</t>
         </is>
       </c>
       <c r="J15" s="61" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="E16" s="61" t="inlineStr">
         <is>
-          <t>Remove Element</t>
+          <t>Plus One</t>
         </is>
       </c>
       <c r="F16" s="61" t="inlineStr">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="I16" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/remove-element/</t>
+          <t>https://leetcode.com/problems/plus-one/</t>
         </is>
       </c>
       <c r="J16" s="61" t="inlineStr">
@@ -3182,7 +3182,7 @@
       </c>
       <c r="E17" s="61" t="inlineStr">
         <is>
-          <t>Plus One</t>
+          <t>Third Maximum Number</t>
         </is>
       </c>
       <c r="F17" s="61" t="inlineStr">
@@ -3202,7 +3202,7 @@
       </c>
       <c r="I17" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/plus-one/</t>
+          <t>https://leetcode.com/problems/third-maximum-number/</t>
         </is>
       </c>
       <c r="J17" s="61" t="inlineStr">
@@ -3239,12 +3239,12 @@
       </c>
       <c r="D18" s="61" t="inlineStr">
         <is>
-          <t>Basics</t>
+          <t>Two pointers</t>
         </is>
       </c>
       <c r="E18" s="61" t="inlineStr">
         <is>
-          <t>Third Maximum Number</t>
+          <t>Remove Duplicates from Sorted Array</t>
         </is>
       </c>
       <c r="F18" s="61" t="inlineStr">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="I18" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/third-maximum-number/</t>
+          <t>https://leetcode.com/problems/remove-duplicates-from-sorted-array/</t>
         </is>
       </c>
       <c r="J18" s="61" t="inlineStr">
@@ -3306,7 +3306,7 @@
       </c>
       <c r="E19" s="61" t="inlineStr">
         <is>
-          <t>Remove Duplicates from Sorted Array</t>
+          <t>Move Zeroes</t>
         </is>
       </c>
       <c r="F19" s="61" t="inlineStr">
@@ -3326,7 +3326,7 @@
       </c>
       <c r="I19" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/remove-duplicates-from-sorted-array/</t>
+          <t>https://leetcode.com/problems/move-zeroes/</t>
         </is>
       </c>
       <c r="J19" s="61" t="inlineStr">
@@ -3368,7 +3368,7 @@
       </c>
       <c r="E20" s="61" t="inlineStr">
         <is>
-          <t>Move Zeroes</t>
+          <t>Sort Array By Parity</t>
         </is>
       </c>
       <c r="F20" s="61" t="inlineStr">
@@ -3388,7 +3388,7 @@
       </c>
       <c r="I20" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/move-zeroes/</t>
+          <t>https://leetcode.com/problems/sort-array-by-parity/</t>
         </is>
       </c>
       <c r="J20" s="61" t="inlineStr">
@@ -3430,12 +3430,12 @@
       </c>
       <c r="E21" s="61" t="inlineStr">
         <is>
-          <t>Sort Array By Parity</t>
+          <t>Two Sum II - Input Array Is Sorted</t>
         </is>
       </c>
       <c r="F21" s="61" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G21" s="61" t="inlineStr">
@@ -3450,7 +3450,7 @@
       </c>
       <c r="I21" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/sort-array-by-parity/</t>
+          <t>https://leetcode.com/problems/two-sum-ii-input-array-is-sorted/</t>
         </is>
       </c>
       <c r="J21" s="61" t="inlineStr">
@@ -3487,17 +3487,17 @@
       </c>
       <c r="D22" s="61" t="inlineStr">
         <is>
-          <t>Two pointers</t>
+          <t>Dutch National Flag</t>
         </is>
       </c>
       <c r="E22" s="61" t="inlineStr">
         <is>
-          <t>Two Sum II - Input Array Is Sorted</t>
+          <t>Segregate 0s and 1s</t>
         </is>
       </c>
       <c r="F22" s="61" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G22" s="61" t="inlineStr">
@@ -3507,12 +3507,12 @@
       </c>
       <c r="H22" s="61" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I22" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/two-sum-ii-input-array-is-sorted/</t>
+          <t>https://www.geeksforgeeks.org/problems/segregate-0s-and-1s5106/1</t>
         </is>
       </c>
       <c r="J22" s="61" t="inlineStr">
@@ -3554,12 +3554,12 @@
       </c>
       <c r="E23" s="61" t="inlineStr">
         <is>
-          <t>Segregate 0s and 1s</t>
+          <t>Sort Colors</t>
         </is>
       </c>
       <c r="F23" s="61" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G23" s="61" t="inlineStr">
@@ -3569,12 +3569,12 @@
       </c>
       <c r="H23" s="61" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I23" s="61" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/segregate-0s-and-1s5106/1</t>
+          <t>https://leetcode.com/problems/sort-colors/</t>
         </is>
       </c>
       <c r="J23" s="61" t="inlineStr">
@@ -3611,17 +3611,17 @@
       </c>
       <c r="D24" s="61" t="inlineStr">
         <is>
-          <t>Dutch National Flag</t>
+          <t>Frequency scan</t>
         </is>
       </c>
       <c r="E24" s="61" t="inlineStr">
         <is>
-          <t>Sort Colors</t>
+          <t>Element Appearing More Than 25% In Sorted Array</t>
         </is>
       </c>
       <c r="F24" s="61" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G24" s="61" t="inlineStr">
@@ -3636,7 +3636,7 @@
       </c>
       <c r="I24" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/sort-colors/</t>
+          <t>https://leetcode.com/problems/element-appearing-more-than-25-in-sorted-array/</t>
         </is>
       </c>
       <c r="J24" s="61" t="inlineStr">
@@ -3678,7 +3678,7 @@
       </c>
       <c r="E25" s="61" t="inlineStr">
         <is>
-          <t>Element Appearing More Than 25% In Sorted Array</t>
+          <t>Most Frequent Even Element</t>
         </is>
       </c>
       <c r="F25" s="61" t="inlineStr">
@@ -3698,7 +3698,7 @@
       </c>
       <c r="I25" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/element-appearing-more-than-25-in-sorted-array/</t>
+          <t>https://leetcode.com/problems/most-frequent-even-element/</t>
         </is>
       </c>
       <c r="J25" s="61" t="inlineStr">
@@ -3735,12 +3735,12 @@
       </c>
       <c r="D26" s="61" t="inlineStr">
         <is>
-          <t>Frequency scan</t>
+          <t>Voting / counting</t>
         </is>
       </c>
       <c r="E26" s="61" t="inlineStr">
         <is>
-          <t>Most Frequent Even Element</t>
+          <t>Majority Element</t>
         </is>
       </c>
       <c r="F26" s="61" t="inlineStr">
@@ -3760,7 +3760,7 @@
       </c>
       <c r="I26" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/most-frequent-even-element/</t>
+          <t>https://leetcode.com/problems/majority-element/</t>
         </is>
       </c>
       <c r="J26" s="61" t="inlineStr">
@@ -3802,12 +3802,12 @@
       </c>
       <c r="E27" s="61" t="inlineStr">
         <is>
-          <t>Majority Element</t>
+          <t>Majority Element II</t>
         </is>
       </c>
       <c r="F27" s="61" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G27" s="61" t="inlineStr">
@@ -3822,7 +3822,7 @@
       </c>
       <c r="I27" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/majority-element/</t>
+          <t>https://leetcode.com/problems/majority-element-ii/</t>
         </is>
       </c>
       <c r="J27" s="61" t="inlineStr">
@@ -3859,12 +3859,12 @@
       </c>
       <c r="D28" s="61" t="inlineStr">
         <is>
-          <t>Voting / counting</t>
+          <t>Rearrangement</t>
         </is>
       </c>
       <c r="E28" s="61" t="inlineStr">
         <is>
-          <t>Majority Element II</t>
+          <t>Rotate Array</t>
         </is>
       </c>
       <c r="F28" s="61" t="inlineStr">
@@ -3884,7 +3884,7 @@
       </c>
       <c r="I28" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/majority-element-ii/</t>
+          <t>https://leetcode.com/problems/rotate-array/</t>
         </is>
       </c>
       <c r="J28" s="61" t="inlineStr">
@@ -3926,7 +3926,7 @@
       </c>
       <c r="E29" s="61" t="inlineStr">
         <is>
-          <t>Rotate Array</t>
+          <t>Next Permutation</t>
         </is>
       </c>
       <c r="F29" s="61" t="inlineStr">
@@ -3946,7 +3946,7 @@
       </c>
       <c r="I29" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/rotate-array/</t>
+          <t>https://leetcode.com/problems/next-permutation/</t>
         </is>
       </c>
       <c r="J29" s="61" t="inlineStr">
@@ -3983,17 +3983,17 @@
       </c>
       <c r="D30" s="61" t="inlineStr">
         <is>
-          <t>Rearrangement</t>
+          <t>K-Sum</t>
         </is>
       </c>
       <c r="E30" s="61" t="inlineStr">
         <is>
-          <t>Next Permutation</t>
+          <t>Number of Arithmetic Triplets</t>
         </is>
       </c>
       <c r="F30" s="61" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G30" s="61" t="inlineStr">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="I30" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/next-permutation/</t>
+          <t>https://leetcode.com/problems/number-of-arithmetic-triplets/</t>
         </is>
       </c>
       <c r="J30" s="61" t="inlineStr">
@@ -4050,12 +4050,12 @@
       </c>
       <c r="E31" s="61" t="inlineStr">
         <is>
-          <t>Number of Arithmetic Triplets</t>
+          <t>3Sum</t>
         </is>
       </c>
       <c r="F31" s="61" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G31" s="61" t="inlineStr">
@@ -4070,7 +4070,7 @@
       </c>
       <c r="I31" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/number-of-arithmetic-triplets/</t>
+          <t>https://leetcode.com/problems/3sum/</t>
         </is>
       </c>
       <c r="J31" s="61" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="E32" s="61" t="inlineStr">
         <is>
-          <t>3Sum</t>
+          <t>3Sum Closest</t>
         </is>
       </c>
       <c r="F32" s="61" t="inlineStr">
@@ -4132,7 +4132,7 @@
       </c>
       <c r="I32" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/3sum/</t>
+          <t>https://leetcode.com/problems/3sum-closest/</t>
         </is>
       </c>
       <c r="J32" s="61" t="inlineStr">
@@ -4164,22 +4164,22 @@
       </c>
       <c r="C33" s="61" t="inlineStr">
         <is>
-          <t>02. Arrays &amp; Two Pointers</t>
+          <t>03. Sorting &amp; Cyclic Sort</t>
         </is>
       </c>
       <c r="D33" s="61" t="inlineStr">
         <is>
-          <t>K-Sum</t>
+          <t>Custom comparator</t>
         </is>
       </c>
       <c r="E33" s="61" t="inlineStr">
         <is>
-          <t>3Sum Closest</t>
+          <t>Relative Sort Array</t>
         </is>
       </c>
       <c r="F33" s="61" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G33" s="61" t="inlineStr">
@@ -4194,7 +4194,7 @@
       </c>
       <c r="I33" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/3sum-closest/</t>
+          <t>https://leetcode.com/problems/relative-sort-array/</t>
         </is>
       </c>
       <c r="J33" s="61" t="inlineStr">
@@ -4236,7 +4236,7 @@
       </c>
       <c r="E34" s="61" t="inlineStr">
         <is>
-          <t>Relative Sort Array</t>
+          <t>Rank Transform of an Array</t>
         </is>
       </c>
       <c r="F34" s="61" t="inlineStr">
@@ -4256,7 +4256,7 @@
       </c>
       <c r="I34" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/relative-sort-array/</t>
+          <t>https://leetcode.com/problems/rank-transform-of-an-array/</t>
         </is>
       </c>
       <c r="J34" s="61" t="inlineStr">
@@ -4298,12 +4298,12 @@
       </c>
       <c r="E35" s="61" t="inlineStr">
         <is>
-          <t>Rank Transform of an Array</t>
+          <t>Largest Number</t>
         </is>
       </c>
       <c r="F35" s="61" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G35" s="61" t="inlineStr">
@@ -4318,7 +4318,7 @@
       </c>
       <c r="I35" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/rank-transform-of-an-array/</t>
+          <t>https://leetcode.com/problems/largest-number/</t>
         </is>
       </c>
       <c r="J35" s="61" t="inlineStr">
@@ -4355,17 +4355,17 @@
       </c>
       <c r="D36" s="61" t="inlineStr">
         <is>
-          <t>Custom comparator</t>
+          <t>Counting sort</t>
         </is>
       </c>
       <c r="E36" s="61" t="inlineStr">
         <is>
-          <t>Largest Number</t>
+          <t>Sort an Array by Increasing Frequency</t>
         </is>
       </c>
       <c r="F36" s="61" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G36" s="61" t="inlineStr">
@@ -4380,7 +4380,7 @@
       </c>
       <c r="I36" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/largest-number/</t>
+          <t>https://leetcode.com/problems/sort-array-by-increasing-frequency/</t>
         </is>
       </c>
       <c r="J36" s="61" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="E37" s="61" t="inlineStr">
         <is>
-          <t>Sort an Array by Increasing Frequency</t>
+          <t>Height Checker</t>
         </is>
       </c>
       <c r="F37" s="61" t="inlineStr">
@@ -4442,7 +4442,7 @@
       </c>
       <c r="I37" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/sort-array-by-increasing-frequency/</t>
+          <t>https://leetcode.com/problems/height-checker/</t>
         </is>
       </c>
       <c r="J37" s="61" t="inlineStr">
@@ -4484,7 +4484,7 @@
       </c>
       <c r="E38" s="61" t="inlineStr">
         <is>
-          <t>Height Checker</t>
+          <t>Sort Even and Odd Indices Independently</t>
         </is>
       </c>
       <c r="F38" s="61" t="inlineStr">
@@ -4504,7 +4504,7 @@
       </c>
       <c r="I38" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/height-checker/</t>
+          <t>https://leetcode.com/problems/sort-even-and-odd-indices-independently/</t>
         </is>
       </c>
       <c r="J38" s="61" t="inlineStr">
@@ -4546,7 +4546,7 @@
       </c>
       <c r="E39" s="61" t="inlineStr">
         <is>
-          <t>Sort Even and Odd Indices Independently</t>
+          <t>Maximum Number of Balls in a Box</t>
         </is>
       </c>
       <c r="F39" s="61" t="inlineStr">
@@ -4566,7 +4566,7 @@
       </c>
       <c r="I39" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/sort-even-and-odd-indices-independently/</t>
+          <t>https://leetcode.com/problems/maximum-number-of-balls-in-a-box/</t>
         </is>
       </c>
       <c r="J39" s="61" t="inlineStr">
@@ -4603,12 +4603,12 @@
       </c>
       <c r="D40" s="61" t="inlineStr">
         <is>
-          <t>Counting sort</t>
+          <t>Cyclic sort</t>
         </is>
       </c>
       <c r="E40" s="61" t="inlineStr">
         <is>
-          <t>Maximum Number of Balls in a Box</t>
+          <t>Missing Number</t>
         </is>
       </c>
       <c r="F40" s="61" t="inlineStr">
@@ -4628,7 +4628,7 @@
       </c>
       <c r="I40" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/maximum-number-of-balls-in-a-box/</t>
+          <t>https://leetcode.com/problems/missing-number/</t>
         </is>
       </c>
       <c r="J40" s="61" t="inlineStr">
@@ -4670,7 +4670,7 @@
       </c>
       <c r="E41" s="61" t="inlineStr">
         <is>
-          <t>Missing Number</t>
+          <t>Find All Numbers Disappeared in an Array</t>
         </is>
       </c>
       <c r="F41" s="61" t="inlineStr">
@@ -4690,7 +4690,7 @@
       </c>
       <c r="I41" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/missing-number/</t>
+          <t>https://leetcode.com/problems/find-all-numbers-disappeared-in-an-array/</t>
         </is>
       </c>
       <c r="J41" s="61" t="inlineStr">
@@ -4727,12 +4727,12 @@
       </c>
       <c r="D42" s="61" t="inlineStr">
         <is>
-          <t>Cyclic sort</t>
+          <t>Sorting application</t>
         </is>
       </c>
       <c r="E42" s="61" t="inlineStr">
         <is>
-          <t>Find All Numbers Disappeared in an Array</t>
+          <t>Largest Perimeter Triangle</t>
         </is>
       </c>
       <c r="F42" s="61" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="I42" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/find-all-numbers-disappeared-in-an-array/</t>
+          <t>https://leetcode.com/problems/largest-perimeter-triangle/</t>
         </is>
       </c>
       <c r="J42" s="61" t="inlineStr">
@@ -4794,7 +4794,7 @@
       </c>
       <c r="E43" s="61" t="inlineStr">
         <is>
-          <t>Largest Perimeter Triangle</t>
+          <t>Minimum Absolute Difference</t>
         </is>
       </c>
       <c r="F43" s="61" t="inlineStr">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="I43" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/largest-perimeter-triangle/</t>
+          <t>https://leetcode.com/problems/minimum-absolute-difference/</t>
         </is>
       </c>
       <c r="J43" s="61" t="inlineStr">
@@ -4856,12 +4856,12 @@
       </c>
       <c r="E44" s="61" t="inlineStr">
         <is>
-          <t>Minimum Absolute Difference</t>
+          <t>H-Index</t>
         </is>
       </c>
       <c r="F44" s="61" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G44" s="61" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="I44" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/minimum-absolute-difference/</t>
+          <t>https://leetcode.com/problems/h-index/</t>
         </is>
       </c>
       <c r="J44" s="61" t="inlineStr">
@@ -4918,7 +4918,7 @@
       </c>
       <c r="E45" s="61" t="inlineStr">
         <is>
-          <t>H-Index</t>
+          <t>Wiggle Sort</t>
         </is>
       </c>
       <c r="F45" s="61" t="inlineStr">
@@ -4933,12 +4933,12 @@
       </c>
       <c r="H45" s="61" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I45" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/h-index/</t>
+          <t>https://www.geeksforgeeks.org/problems/convert-array-into-zig-zag-fashion1638/1</t>
         </is>
       </c>
       <c r="J45" s="61" t="inlineStr">
@@ -4970,22 +4970,22 @@
       </c>
       <c r="C46" s="61" t="inlineStr">
         <is>
-          <t>03. Sorting &amp; Cyclic Sort</t>
+          <t>04. Hashing</t>
         </is>
       </c>
       <c r="D46" s="61" t="inlineStr">
         <is>
-          <t>Sorting application</t>
+          <t>Set basics</t>
         </is>
       </c>
       <c r="E46" s="61" t="inlineStr">
         <is>
-          <t>Wiggle Sort</t>
+          <t>Contains Duplicate</t>
         </is>
       </c>
       <c r="F46" s="61" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G46" s="61" t="inlineStr">
@@ -4995,12 +4995,12 @@
       </c>
       <c r="H46" s="61" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I46" s="61" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/convert-array-into-zig-zag-fashion1638/1</t>
+          <t>https://leetcode.com/problems/contains-duplicate/</t>
         </is>
       </c>
       <c r="J46" s="61" t="inlineStr">
@@ -5042,7 +5042,7 @@
       </c>
       <c r="E47" s="61" t="inlineStr">
         <is>
-          <t>Contains Duplicate</t>
+          <t>Contains Duplicate II</t>
         </is>
       </c>
       <c r="F47" s="61" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="I47" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/contains-duplicate/</t>
+          <t>https://leetcode.com/problems/contains-duplicate-ii/</t>
         </is>
       </c>
       <c r="J47" s="61" t="inlineStr">
@@ -5104,7 +5104,7 @@
       </c>
       <c r="E48" s="61" t="inlineStr">
         <is>
-          <t>Contains Duplicate II</t>
+          <t>Unique Number of Occurrences</t>
         </is>
       </c>
       <c r="F48" s="61" t="inlineStr">
@@ -5124,7 +5124,7 @@
       </c>
       <c r="I48" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/contains-duplicate-ii/</t>
+          <t>https://leetcode.com/problems/unique-number-of-occurrences/</t>
         </is>
       </c>
       <c r="J48" s="61" t="inlineStr">
@@ -5166,7 +5166,7 @@
       </c>
       <c r="E49" s="61" t="inlineStr">
         <is>
-          <t>Unique Number of Occurrences</t>
+          <t>Check If N and Its Double Exist</t>
         </is>
       </c>
       <c r="F49" s="61" t="inlineStr">
@@ -5186,7 +5186,7 @@
       </c>
       <c r="I49" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/unique-number-of-occurrences/</t>
+          <t>https://leetcode.com/problems/check-if-n-and-its-double-exist/</t>
         </is>
       </c>
       <c r="J49" s="61" t="inlineStr">
@@ -5223,12 +5223,12 @@
       </c>
       <c r="D50" s="61" t="inlineStr">
         <is>
-          <t>Set basics</t>
+          <t>Complement lookup</t>
         </is>
       </c>
       <c r="E50" s="61" t="inlineStr">
         <is>
-          <t>Check If N and Its Double Exist</t>
+          <t>Two Sum</t>
         </is>
       </c>
       <c r="F50" s="61" t="inlineStr">
@@ -5248,7 +5248,7 @@
       </c>
       <c r="I50" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/check-if-n-and-its-double-exist/</t>
+          <t>https://leetcode.com/problems/two-sum/</t>
         </is>
       </c>
       <c r="J50" s="61" t="inlineStr">
@@ -5285,12 +5285,12 @@
       </c>
       <c r="D51" s="61" t="inlineStr">
         <is>
-          <t>Complement lookup</t>
+          <t>Frequency map</t>
         </is>
       </c>
       <c r="E51" s="61" t="inlineStr">
         <is>
-          <t>Two Sum</t>
+          <t>First Unique Character in a String</t>
         </is>
       </c>
       <c r="F51" s="61" t="inlineStr">
@@ -5310,7 +5310,7 @@
       </c>
       <c r="I51" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/two-sum/</t>
+          <t>https://leetcode.com/problems/first-unique-character-in-a-string/</t>
         </is>
       </c>
       <c r="J51" s="61" t="inlineStr">
@@ -5352,7 +5352,7 @@
       </c>
       <c r="E52" s="61" t="inlineStr">
         <is>
-          <t>First Unique Character in a String</t>
+          <t>Ransom Note</t>
         </is>
       </c>
       <c r="F52" s="61" t="inlineStr">
@@ -5372,7 +5372,7 @@
       </c>
       <c r="I52" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/first-unique-character-in-a-string/</t>
+          <t>https://leetcode.com/problems/ransom-note/</t>
         </is>
       </c>
       <c r="J52" s="61" t="inlineStr">
@@ -5409,12 +5409,12 @@
       </c>
       <c r="D53" s="61" t="inlineStr">
         <is>
-          <t>Frequency map</t>
+          <t>Set + scan</t>
         </is>
       </c>
       <c r="E53" s="61" t="inlineStr">
         <is>
-          <t>Ransom Note</t>
+          <t>Distribute Candies</t>
         </is>
       </c>
       <c r="F53" s="61" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="I53" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/ransom-note/</t>
+          <t>https://leetcode.com/problems/distribute-candies/</t>
         </is>
       </c>
       <c r="J53" s="61" t="inlineStr">
@@ -5476,7 +5476,7 @@
       </c>
       <c r="E54" s="61" t="inlineStr">
         <is>
-          <t>Distribute Candies</t>
+          <t>Maximum Number of Pairs in Array</t>
         </is>
       </c>
       <c r="F54" s="61" t="inlineStr">
@@ -5496,7 +5496,7 @@
       </c>
       <c r="I54" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/distribute-candies/</t>
+          <t>https://leetcode.com/problems/maximum-number-of-pairs-in-array/</t>
         </is>
       </c>
       <c r="J54" s="61" t="inlineStr">
@@ -5538,7 +5538,7 @@
       </c>
       <c r="E55" s="61" t="inlineStr">
         <is>
-          <t>Maximum Number of Pairs in Array</t>
+          <t>Longest Harmonious Subsequence</t>
         </is>
       </c>
       <c r="F55" s="61" t="inlineStr">
@@ -5558,7 +5558,7 @@
       </c>
       <c r="I55" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/maximum-number-of-pairs-in-array/</t>
+          <t>https://leetcode.com/problems/longest-harmonious-subsequence/</t>
         </is>
       </c>
       <c r="J55" s="61" t="inlineStr">
@@ -5600,12 +5600,12 @@
       </c>
       <c r="E56" s="61" t="inlineStr">
         <is>
-          <t>Longest Harmonious Subsequence</t>
+          <t>Longest Consecutive Sequence</t>
         </is>
       </c>
       <c r="F56" s="61" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G56" s="61" t="inlineStr">
@@ -5620,7 +5620,7 @@
       </c>
       <c r="I56" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/longest-harmonious-subsequence/</t>
+          <t>https://leetcode.com/problems/longest-consecutive-sequence/</t>
         </is>
       </c>
       <c r="J56" s="61" t="inlineStr">
@@ -5657,17 +5657,17 @@
       </c>
       <c r="D57" s="61" t="inlineStr">
         <is>
-          <t>Set + scan</t>
+          <t>Cycle detection</t>
         </is>
       </c>
       <c r="E57" s="61" t="inlineStr">
         <is>
-          <t>Longest Consecutive Sequence</t>
+          <t>Happy Number</t>
         </is>
       </c>
       <c r="F57" s="61" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G57" s="61" t="inlineStr">
@@ -5682,7 +5682,7 @@
       </c>
       <c r="I57" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/longest-consecutive-sequence/</t>
+          <t>https://leetcode.com/problems/happy-number/</t>
         </is>
       </c>
       <c r="J57" s="61" t="inlineStr">
@@ -5719,12 +5719,12 @@
       </c>
       <c r="D58" s="61" t="inlineStr">
         <is>
-          <t>Cycle detection</t>
+          <t>Grid hashing</t>
         </is>
       </c>
       <c r="E58" s="61" t="inlineStr">
         <is>
-          <t>Happy Number</t>
+          <t>Number of Equivalent Domino Pairs</t>
         </is>
       </c>
       <c r="F58" s="61" t="inlineStr">
@@ -5744,7 +5744,7 @@
       </c>
       <c r="I58" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/happy-number/</t>
+          <t>https://leetcode.com/problems/number-of-equivalent-domino-pairs/</t>
         </is>
       </c>
       <c r="J58" s="61" t="inlineStr">
@@ -5786,7 +5786,7 @@
       </c>
       <c r="E59" s="61" t="inlineStr">
         <is>
-          <t>Number of Equivalent Domino Pairs</t>
+          <t>Check if Every Row and Column Contains All Numbers</t>
         </is>
       </c>
       <c r="F59" s="61" t="inlineStr">
@@ -5806,7 +5806,7 @@
       </c>
       <c r="I59" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/number-of-equivalent-domino-pairs/</t>
+          <t>https://leetcode.com/problems/check-if-every-row-and-column-contains-all-numbers/</t>
         </is>
       </c>
       <c r="J59" s="61" t="inlineStr">
@@ -5848,12 +5848,12 @@
       </c>
       <c r="E60" s="61" t="inlineStr">
         <is>
-          <t>Check if Every Row and Column Contains All Numbers</t>
+          <t>Valid Sudoku</t>
         </is>
       </c>
       <c r="F60" s="61" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G60" s="61" t="inlineStr">
@@ -5868,7 +5868,7 @@
       </c>
       <c r="I60" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/check-if-every-row-and-column-contains-all-numbers/</t>
+          <t>https://leetcode.com/problems/valid-sudoku/</t>
         </is>
       </c>
       <c r="J60" s="61" t="inlineStr">
@@ -5905,17 +5905,17 @@
       </c>
       <c r="D61" s="61" t="inlineStr">
         <is>
-          <t>Grid hashing</t>
+          <t>Line hashing</t>
         </is>
       </c>
       <c r="E61" s="61" t="inlineStr">
         <is>
-          <t>Valid Sudoku</t>
+          <t>Check If It Is a Straight Line</t>
         </is>
       </c>
       <c r="F61" s="61" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G61" s="61" t="inlineStr">
@@ -5930,7 +5930,7 @@
       </c>
       <c r="I61" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/valid-sudoku/</t>
+          <t>https://leetcode.com/problems/check-if-it-is-a-straight-line/</t>
         </is>
       </c>
       <c r="J61" s="61" t="inlineStr">
@@ -5972,12 +5972,12 @@
       </c>
       <c r="E62" s="61" t="inlineStr">
         <is>
-          <t>Check If It Is a Straight Line</t>
+          <t>Brick Wall</t>
         </is>
       </c>
       <c r="F62" s="61" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G62" s="61" t="inlineStr">
@@ -5992,7 +5992,7 @@
       </c>
       <c r="I62" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/check-if-it-is-a-straight-line/</t>
+          <t>https://leetcode.com/problems/brick-wall/</t>
         </is>
       </c>
       <c r="J62" s="61" t="inlineStr">
@@ -6029,12 +6029,12 @@
       </c>
       <c r="D63" s="61" t="inlineStr">
         <is>
-          <t>Line hashing</t>
+          <t>Meet in the middle</t>
         </is>
       </c>
       <c r="E63" s="61" t="inlineStr">
         <is>
-          <t>Brick Wall</t>
+          <t>4Sum II</t>
         </is>
       </c>
       <c r="F63" s="61" t="inlineStr">
@@ -6054,7 +6054,7 @@
       </c>
       <c r="I63" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/brick-wall/</t>
+          <t>https://leetcode.com/problems/4sum-ii/</t>
         </is>
       </c>
       <c r="J63" s="61" t="inlineStr">
@@ -6086,22 +6086,22 @@
       </c>
       <c r="C64" s="61" t="inlineStr">
         <is>
-          <t>04. Hashing</t>
+          <t>05. Prefix Sum &amp; Kadane</t>
         </is>
       </c>
       <c r="D64" s="61" t="inlineStr">
         <is>
-          <t>Meet in the middle</t>
+          <t>Prefix basics</t>
         </is>
       </c>
       <c r="E64" s="61" t="inlineStr">
         <is>
-          <t>4Sum II</t>
+          <t>Running Sum of 1d Array</t>
         </is>
       </c>
       <c r="F64" s="61" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G64" s="61" t="inlineStr">
@@ -6116,7 +6116,7 @@
       </c>
       <c r="I64" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/4sum-ii/</t>
+          <t>https://leetcode.com/problems/running-sum-of-1d-array/</t>
         </is>
       </c>
       <c r="J64" s="61" t="inlineStr">
@@ -6158,7 +6158,7 @@
       </c>
       <c r="E65" s="61" t="inlineStr">
         <is>
-          <t>Running Sum of 1d Array</t>
+          <t>Find Pivot Index</t>
         </is>
       </c>
       <c r="F65" s="61" t="inlineStr">
@@ -6178,7 +6178,7 @@
       </c>
       <c r="I65" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/running-sum-of-1d-array/</t>
+          <t>https://leetcode.com/problems/find-pivot-index/</t>
         </is>
       </c>
       <c r="J65" s="61" t="inlineStr">
@@ -6220,12 +6220,12 @@
       </c>
       <c r="E66" s="61" t="inlineStr">
         <is>
-          <t>Find Pivot Index</t>
+          <t>Product of Array Except Self</t>
         </is>
       </c>
       <c r="F66" s="61" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G66" s="61" t="inlineStr">
@@ -6240,7 +6240,7 @@
       </c>
       <c r="I66" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/find-pivot-index/</t>
+          <t>https://leetcode.com/problems/product-of-array-except-self/</t>
         </is>
       </c>
       <c r="J66" s="61" t="inlineStr">
@@ -6277,12 +6277,12 @@
       </c>
       <c r="D67" s="61" t="inlineStr">
         <is>
-          <t>Prefix basics</t>
+          <t>Kadane</t>
         </is>
       </c>
       <c r="E67" s="61" t="inlineStr">
         <is>
-          <t>Product of Array Except Self</t>
+          <t>Maximum Subarray</t>
         </is>
       </c>
       <c r="F67" s="61" t="inlineStr">
@@ -6302,7 +6302,7 @@
       </c>
       <c r="I67" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/product-of-array-except-self/</t>
+          <t>https://leetcode.com/problems/maximum-subarray/</t>
         </is>
       </c>
       <c r="J67" s="61" t="inlineStr">
@@ -6344,12 +6344,12 @@
       </c>
       <c r="E68" s="61" t="inlineStr">
         <is>
-          <t>Maximum Subarray</t>
+          <t>Best Time to Buy and Sell Stock</t>
         </is>
       </c>
       <c r="F68" s="61" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G68" s="61" t="inlineStr">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="I68" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/maximum-subarray/</t>
+          <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock/</t>
         </is>
       </c>
       <c r="J68" s="61" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="E69" s="61" t="inlineStr">
         <is>
-          <t>Best Time to Buy and Sell Stock</t>
+          <t>Smallest Sum Contiguous Subarray</t>
         </is>
       </c>
       <c r="F69" s="61" t="inlineStr">
@@ -6421,12 +6421,12 @@
       </c>
       <c r="H69" s="61" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I69" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock/</t>
+          <t>https://www.geeksforgeeks.org/problems/smallest-sum-contiguous-subarray/1</t>
         </is>
       </c>
       <c r="J69" s="61" t="inlineStr">
@@ -6468,12 +6468,12 @@
       </c>
       <c r="E70" s="61" t="inlineStr">
         <is>
-          <t>Smallest Sum Contiguous Subarray</t>
+          <t>Maximum Product Subarray</t>
         </is>
       </c>
       <c r="F70" s="61" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G70" s="61" t="inlineStr">
@@ -6483,12 +6483,12 @@
       </c>
       <c r="H70" s="61" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I70" s="61" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/smallest-sum-contiguous-subarray/1</t>
+          <t>https://leetcode.com/problems/maximum-product-subarray/</t>
         </is>
       </c>
       <c r="J70" s="61" t="inlineStr">
@@ -6525,12 +6525,12 @@
       </c>
       <c r="D71" s="61" t="inlineStr">
         <is>
-          <t>Kadane</t>
+          <t>Prefix + HashMap</t>
         </is>
       </c>
       <c r="E71" s="61" t="inlineStr">
         <is>
-          <t>Maximum Product Subarray</t>
+          <t>Subarray Sum Equals K</t>
         </is>
       </c>
       <c r="F71" s="61" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="I71" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/maximum-product-subarray/</t>
+          <t>https://leetcode.com/problems/subarray-sum-equals-k/</t>
         </is>
       </c>
       <c r="J71" s="61" t="inlineStr">
@@ -6592,7 +6592,7 @@
       </c>
       <c r="E72" s="61" t="inlineStr">
         <is>
-          <t>Subarray Sum Equals K</t>
+          <t>Subarray Sums Divisible by K</t>
         </is>
       </c>
       <c r="F72" s="61" t="inlineStr">
@@ -6612,7 +6612,7 @@
       </c>
       <c r="I72" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/subarray-sum-equals-k/</t>
+          <t>https://leetcode.com/problems/subarray-sums-divisible-by-k/</t>
         </is>
       </c>
       <c r="J72" s="61" t="inlineStr">
@@ -6649,17 +6649,17 @@
       </c>
       <c r="D73" s="61" t="inlineStr">
         <is>
-          <t>Prefix + HashMap</t>
+          <t>Difference array</t>
         </is>
       </c>
       <c r="E73" s="61" t="inlineStr">
         <is>
-          <t>Subarray Sums Divisible by K</t>
+          <t>Maximum Population Year</t>
         </is>
       </c>
       <c r="F73" s="61" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G73" s="61" t="inlineStr">
@@ -6674,7 +6674,7 @@
       </c>
       <c r="I73" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/subarray-sums-divisible-by-k/</t>
+          <t>https://leetcode.com/problems/maximum-population-year/</t>
         </is>
       </c>
       <c r="J73" s="61" t="inlineStr">
@@ -6716,12 +6716,12 @@
       </c>
       <c r="E74" s="61" t="inlineStr">
         <is>
-          <t>Maximum Population Year</t>
+          <t>Corporate Flight Bookings</t>
         </is>
       </c>
       <c r="F74" s="61" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G74" s="61" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="I74" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/maximum-population-year/</t>
+          <t>https://leetcode.com/problems/corporate-flight-bookings/</t>
         </is>
       </c>
       <c r="J74" s="61" t="inlineStr">
@@ -6778,7 +6778,7 @@
       </c>
       <c r="E75" s="61" t="inlineStr">
         <is>
-          <t>Corporate Flight Bookings</t>
+          <t>Car Pooling</t>
         </is>
       </c>
       <c r="F75" s="61" t="inlineStr">
@@ -6798,7 +6798,7 @@
       </c>
       <c r="I75" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/corporate-flight-bookings/</t>
+          <t>https://leetcode.com/problems/car-pooling/</t>
         </is>
       </c>
       <c r="J75" s="61" t="inlineStr">
@@ -6830,22 +6830,22 @@
       </c>
       <c r="C76" s="61" t="inlineStr">
         <is>
-          <t>05. Prefix Sum &amp; Kadane</t>
+          <t>06. Sliding Window</t>
         </is>
       </c>
       <c r="D76" s="61" t="inlineStr">
         <is>
-          <t>Difference array</t>
+          <t>Fixed window</t>
         </is>
       </c>
       <c r="E76" s="61" t="inlineStr">
         <is>
-          <t>Car Pooling</t>
+          <t>Maximum Average Subarray I</t>
         </is>
       </c>
       <c r="F76" s="61" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G76" s="61" t="inlineStr">
@@ -6860,7 +6860,7 @@
       </c>
       <c r="I76" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/car-pooling/</t>
+          <t>https://leetcode.com/problems/maximum-average-subarray-i/</t>
         </is>
       </c>
       <c r="J76" s="61" t="inlineStr">
@@ -6902,7 +6902,7 @@
       </c>
       <c r="E77" s="61" t="inlineStr">
         <is>
-          <t>Maximum Average Subarray I</t>
+          <t>Max Sum Subarray of Size K</t>
         </is>
       </c>
       <c r="F77" s="61" t="inlineStr">
@@ -6917,12 +6917,12 @@
       </c>
       <c r="H77" s="61" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I77" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/maximum-average-subarray-i/</t>
+          <t>https://www.geeksforgeeks.org/problems/max-sum-subarray-of-size-k5313/1</t>
         </is>
       </c>
       <c r="J77" s="61" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="E78" s="61" t="inlineStr">
         <is>
-          <t>Max Sum Subarray of Size K</t>
+          <t>Substrings of Size Three with Distinct Characters</t>
         </is>
       </c>
       <c r="F78" s="61" t="inlineStr">
@@ -6979,12 +6979,12 @@
       </c>
       <c r="H78" s="61" t="inlineStr">
         <is>
-          <t>GeeksforGeeks</t>
+          <t>LeetCode</t>
         </is>
       </c>
       <c r="I78" s="61" t="inlineStr">
         <is>
-          <t>https://www.geeksforgeeks.org/problems/max-sum-subarray-of-size-k5313/1</t>
+          <t>https://leetcode.com/problems/substrings-of-size-three-with-distinct-characters/</t>
         </is>
       </c>
       <c r="J78" s="61" t="inlineStr">
@@ -7021,17 +7021,17 @@
       </c>
       <c r="D79" s="61" t="inlineStr">
         <is>
-          <t>Fixed window</t>
+          <t>Variable window</t>
         </is>
       </c>
       <c r="E79" s="61" t="inlineStr">
         <is>
-          <t>Substrings of Size Three with Distinct Characters</t>
+          <t>Minimum Size Subarray Sum</t>
         </is>
       </c>
       <c r="F79" s="61" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G79" s="61" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="I79" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/substrings-of-size-three-with-distinct-characters/</t>
+          <t>https://leetcode.com/problems/minimum-size-subarray-sum/</t>
         </is>
       </c>
       <c r="J79" s="61" t="inlineStr">
@@ -7088,7 +7088,7 @@
       </c>
       <c r="E80" s="61" t="inlineStr">
         <is>
-          <t>Minimum Size Subarray Sum</t>
+          <t>Longest Substring Without Repeating Characters</t>
         </is>
       </c>
       <c r="F80" s="61" t="inlineStr">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="I80" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/minimum-size-subarray-sum/</t>
+          <t>https://leetcode.com/problems/longest-substring-without-repeating-characters/</t>
         </is>
       </c>
       <c r="J80" s="61" t="inlineStr">
@@ -7150,7 +7150,7 @@
       </c>
       <c r="E81" s="61" t="inlineStr">
         <is>
-          <t>Longest Substring Without Repeating Characters</t>
+          <t>Longest Repeating Character Replacement</t>
         </is>
       </c>
       <c r="F81" s="61" t="inlineStr">
@@ -7170,7 +7170,7 @@
       </c>
       <c r="I81" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/longest-substring-without-repeating-characters/</t>
+          <t>https://leetcode.com/problems/longest-repeating-character-replacement/</t>
         </is>
       </c>
       <c r="J81" s="61" t="inlineStr">
@@ -7212,7 +7212,7 @@
       </c>
       <c r="E82" s="61" t="inlineStr">
         <is>
-          <t>Longest Repeating Character Replacement</t>
+          <t>Max Consecutive Ones III</t>
         </is>
       </c>
       <c r="F82" s="61" t="inlineStr">
@@ -7232,7 +7232,7 @@
       </c>
       <c r="I82" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/longest-repeating-character-replacement/</t>
+          <t>https://leetcode.com/problems/max-consecutive-ones-iii/</t>
         </is>
       </c>
       <c r="J82" s="61" t="inlineStr">
@@ -7269,12 +7269,12 @@
       </c>
       <c r="D83" s="61" t="inlineStr">
         <is>
-          <t>Variable window</t>
+          <t>Anagram window</t>
         </is>
       </c>
       <c r="E83" s="61" t="inlineStr">
         <is>
-          <t>Max Consecutive Ones III</t>
+          <t>Permutation in String</t>
         </is>
       </c>
       <c r="F83" s="61" t="inlineStr">
@@ -7294,7 +7294,7 @@
       </c>
       <c r="I83" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/max-consecutive-ones-iii/</t>
+          <t>https://leetcode.com/problems/permutation-in-string/</t>
         </is>
       </c>
       <c r="J83" s="61" t="inlineStr">
@@ -7336,7 +7336,7 @@
       </c>
       <c r="E84" s="61" t="inlineStr">
         <is>
-          <t>Permutation in String</t>
+          <t>Find All Anagrams in a String</t>
         </is>
       </c>
       <c r="F84" s="61" t="inlineStr">
@@ -7356,7 +7356,7 @@
       </c>
       <c r="I84" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/permutation-in-string/</t>
+          <t>https://leetcode.com/problems/find-all-anagrams-in-a-string/</t>
         </is>
       </c>
       <c r="J84" s="61" t="inlineStr">
@@ -7393,12 +7393,12 @@
       </c>
       <c r="D85" s="61" t="inlineStr">
         <is>
-          <t>Anagram window</t>
+          <t>Count exactly-K trick</t>
         </is>
       </c>
       <c r="E85" s="61" t="inlineStr">
         <is>
-          <t>Find All Anagrams in a String</t>
+          <t>Binary Subarrays With Sum</t>
         </is>
       </c>
       <c r="F85" s="61" t="inlineStr">
@@ -7418,7 +7418,7 @@
       </c>
       <c r="I85" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/find-all-anagrams-in-a-string/</t>
+          <t>https://leetcode.com/problems/binary-subarrays-with-sum/</t>
         </is>
       </c>
       <c r="J85" s="61" t="inlineStr">
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E86" s="61" t="inlineStr">
         <is>
-          <t>Binary Subarrays With Sum</t>
+          <t>Count Number of Nice Subarrays</t>
         </is>
       </c>
       <c r="F86" s="61" t="inlineStr">
@@ -7480,7 +7480,7 @@
       </c>
       <c r="I86" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/binary-subarrays-with-sum/</t>
+          <t>https://leetcode.com/problems/count-number-of-nice-subarrays/</t>
         </is>
       </c>
       <c r="J86" s="61" t="inlineStr">
@@ -7517,17 +7517,17 @@
       </c>
       <c r="D87" s="61" t="inlineStr">
         <is>
-          <t>Count exactly-K trick</t>
+          <t>Hard window</t>
         </is>
       </c>
       <c r="E87" s="61" t="inlineStr">
         <is>
-          <t>Count Number of Nice Subarrays</t>
+          <t>Minimum Window Substring</t>
         </is>
       </c>
       <c r="F87" s="61" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="G87" s="61" t="inlineStr">
@@ -7542,7 +7542,7 @@
       </c>
       <c r="I87" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/count-number-of-nice-subarrays/</t>
+          <t>https://leetcode.com/problems/minimum-window-substring/</t>
         </is>
       </c>
       <c r="J87" s="61" t="inlineStr">
@@ -7569,42 +7569,42 @@
       </c>
       <c r="B88" s="61" t="inlineStr">
         <is>
-          <t>1. Foundations - Core</t>
+          <t>1. Foundations - Depth</t>
         </is>
       </c>
       <c r="C88" s="61" t="inlineStr">
         <is>
-          <t>06. Sliding Window</t>
+          <t>01. Basics &amp; Recursion</t>
         </is>
       </c>
       <c r="D88" s="61" t="inlineStr">
         <is>
-          <t>Hard window</t>
+          <t>Divide &amp; Conquer</t>
         </is>
       </c>
       <c r="E88" s="61" t="inlineStr">
         <is>
-          <t>Minimum Window Substring</t>
+          <t>Count Inversions</t>
         </is>
       </c>
       <c r="F88" s="61" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G88" s="61" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Depth</t>
         </is>
       </c>
       <c r="H88" s="61" t="inlineStr">
         <is>
-          <t>LeetCode</t>
+          <t>GeeksforGeeks</t>
         </is>
       </c>
       <c r="I88" s="61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/minimum-window-substring/</t>
+          <t>https://www.geeksforgeeks.org/problems/inversion-of-array-1587115620/1</t>
         </is>
       </c>
       <c r="J88" s="61" t="inlineStr">
@@ -65959,10 +65959,10 @@
         </is>
       </c>
       <c r="C3" s="31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D3" s="31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" s="31" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Count the Plan tab by stage and fix the Core tooltip
The Plan tab's formulas hardcoded every topic name with its v3 number, so
after the v4 renumbering only topics 01, 02 and 23 matched and the per-phase
Core counts were wrong. Core Qs and Done now count Master's Stage column
("1. Foundations - Core" and so on), which doesn't depend on topic names.
They read 86, 94, 46, 44, 77, 40 (387). The topics-covered text follows the
v4 phases.

The "Core only" tooltip no longer claims two problems per pattern.
</commit_message>
<xml_diff>
--- a/DSA_Master_Sheet.xlsx
+++ b/DSA_Master_Sheet.xlsx
@@ -1848,11 +1848,11 @@
       </c>
       <c r="C9" s="42" t="inlineStr">
         <is>
-          <t>01 - 05: Basics &amp; Recursion, Arrays &amp; Two Pointers, Sliding Window, Prefix Sum &amp; Kadane, Sorting &amp; Cyclic Sort</t>
+          <t>01 - 06: Basics &amp; Recursion, Arrays &amp; Two Pointers, Sorting &amp; Cyclic Sort, Hashing, Prefix Sum &amp; Kadane, Sliding Window</t>
         </is>
       </c>
       <c r="D9" s="43">
-        <f>COUNTIFS(Master!$C$2:$C$918,"01. Basics &amp; Recursion",Master!$G$2:$G$918,"Core")+COUNTIFS(Master!$C$2:$C$918,"02. Arrays &amp; Two Pointers",Master!$G$2:$G$918,"Core")+COUNTIFS(Master!$C$2:$C$918,"03. Sliding Window",Master!$G$2:$G$918,"Core")+COUNTIFS(Master!$C$2:$C$918,"04. Prefix Sum &amp; Kadane",Master!$G$2:$G$918,"Core")+COUNTIFS(Master!$C$2:$C$918,"05. Sorting &amp; Cyclic Sort",Master!$G$2:$G$918,"Core")</f>
+        <f>COUNTIF(Master!$B$2:$B$918,"1. Foundations - Core")</f>
         <v/>
       </c>
       <c r="E9" s="43">
@@ -1868,7 +1868,7 @@
         <v/>
       </c>
       <c r="H9" s="43">
-        <f>COUNTIFS(Master!$C$2:$C$918,"01. Basics &amp; Recursion",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"01. Basics &amp; Recursion",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")+COUNTIFS(Master!$C$2:$C$918,"02. Arrays &amp; Two Pointers",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"02. Arrays &amp; Two Pointers",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")+COUNTIFS(Master!$C$2:$C$918,"03. Sliding Window",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"03. Sliding Window",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")+COUNTIFS(Master!$C$2:$C$918,"04. Prefix Sum &amp; Kadane",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"04. Prefix Sum &amp; Kadane",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")+COUNTIFS(Master!$C$2:$C$918,"05. Sorting &amp; Cyclic Sort",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"05. Sorting &amp; Cyclic Sort",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")</f>
+        <f>COUNTIFS(Master!$B$2:$B$918,"1. Foundations - Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$B$2:$B$918,"1. Foundations - Core",Master!$J$2:$J$918,"Mastered")</f>
         <v/>
       </c>
       <c r="I9" s="45">
@@ -1884,11 +1884,11 @@
       </c>
       <c r="C10" s="42" t="inlineStr">
         <is>
-          <t>06 - 09: Binary Search, Strings, Hashing, Matrix / 2D</t>
+          <t>07 - 11: Binary Search, Strings, Bit Manipulation, Math &amp; Number Theory, Matrix / 2D</t>
         </is>
       </c>
       <c r="D10" s="43">
-        <f>COUNTIFS(Master!$C$2:$C$918,"06. Binary Search",Master!$G$2:$G$918,"Core")+COUNTIFS(Master!$C$2:$C$918,"07. Strings",Master!$G$2:$G$918,"Core")+COUNTIFS(Master!$C$2:$C$918,"08. Hashing",Master!$G$2:$G$918,"Core")+COUNTIFS(Master!$C$2:$C$918,"09. Matrix / 2D",Master!$G$2:$G$918,"Core")</f>
+        <f>COUNTIF(Master!$B$2:$B$918,"2. Search, Strings &amp; Math - Core")</f>
         <v/>
       </c>
       <c r="E10" s="43">
@@ -1904,7 +1904,7 @@
         <v/>
       </c>
       <c r="H10" s="43">
-        <f>COUNTIFS(Master!$C$2:$C$918,"06. Binary Search",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"06. Binary Search",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")+COUNTIFS(Master!$C$2:$C$918,"07. Strings",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"07. Strings",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")+COUNTIFS(Master!$C$2:$C$918,"08. Hashing",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"08. Hashing",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")+COUNTIFS(Master!$C$2:$C$918,"09. Matrix / 2D",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"09. Matrix / 2D",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")</f>
+        <f>COUNTIFS(Master!$B$2:$B$918,"2. Search, Strings &amp; Math - Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$B$2:$B$918,"2. Search, Strings &amp; Math - Core",Master!$J$2:$J$918,"Mastered")</f>
         <v/>
       </c>
       <c r="I10" s="45">
@@ -1920,11 +1920,11 @@
       </c>
       <c r="C11" s="42" t="inlineStr">
         <is>
-          <t>10 - 12: Linked List, Stack &amp; Queue, Heap &amp; Priority Queue</t>
+          <t>12 - 14: Linked List, Stack &amp; Queue, Heap &amp; Priority Queue</t>
         </is>
       </c>
       <c r="D11" s="43">
-        <f>COUNTIFS(Master!$C$2:$C$918,"10. Linked List",Master!$G$2:$G$918,"Core")+COUNTIFS(Master!$C$2:$C$918,"11. Stack &amp; Queue",Master!$G$2:$G$918,"Core")+COUNTIFS(Master!$C$2:$C$918,"12. Heap &amp; Priority Queue",Master!$G$2:$G$918,"Core")</f>
+        <f>COUNTIF(Master!$B$2:$B$918,"3. Linear DS - Core")</f>
         <v/>
       </c>
       <c r="E11" s="43">
@@ -1940,7 +1940,7 @@
         <v/>
       </c>
       <c r="H11" s="43">
-        <f>COUNTIFS(Master!$C$2:$C$918,"10. Linked List",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"10. Linked List",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")+COUNTIFS(Master!$C$2:$C$918,"11. Stack &amp; Queue",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"11. Stack &amp; Queue",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")+COUNTIFS(Master!$C$2:$C$918,"12. Heap &amp; Priority Queue",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"12. Heap &amp; Priority Queue",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")</f>
+        <f>COUNTIFS(Master!$B$2:$B$918,"3. Linear DS - Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$B$2:$B$918,"3. Linear DS - Core",Master!$J$2:$J$918,"Mastered")</f>
         <v/>
       </c>
       <c r="I11" s="45">
@@ -1956,11 +1956,11 @@
       </c>
       <c r="C12" s="42" t="inlineStr">
         <is>
-          <t>13 - 14: Greedy, Backtracking</t>
+          <t>15 - 17: Intervals, Greedy, Backtracking</t>
         </is>
       </c>
       <c r="D12" s="43">
-        <f>COUNTIFS(Master!$C$2:$C$918,"13. Greedy",Master!$G$2:$G$918,"Core")+COUNTIFS(Master!$C$2:$C$918,"14. Backtracking",Master!$G$2:$G$918,"Core")</f>
+        <f>COUNTIF(Master!$B$2:$B$918,"4. Greedy &amp; Backtracking - Core")</f>
         <v/>
       </c>
       <c r="E12" s="43">
@@ -1976,7 +1976,7 @@
         <v/>
       </c>
       <c r="H12" s="43">
-        <f>COUNTIFS(Master!$C$2:$C$918,"13. Greedy",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"13. Greedy",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")+COUNTIFS(Master!$C$2:$C$918,"14. Backtracking",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"14. Backtracking",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")</f>
+        <f>COUNTIFS(Master!$B$2:$B$918,"4. Greedy &amp; Backtracking - Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$B$2:$B$918,"4. Greedy &amp; Backtracking - Core",Master!$J$2:$J$918,"Mastered")</f>
         <v/>
       </c>
       <c r="I12" s="45">
@@ -1992,11 +1992,11 @@
       </c>
       <c r="C13" s="42" t="inlineStr">
         <is>
-          <t>15 - 17: Trees &amp; BST, Tries, Graphs</t>
+          <t>18 - 20: Trees &amp; BST, Tries, Graphs</t>
         </is>
       </c>
       <c r="D13" s="43">
-        <f>COUNTIFS(Master!$C$2:$C$918,"15. Trees &amp; BST",Master!$G$2:$G$918,"Core")+COUNTIFS(Master!$C$2:$C$918,"16. Tries",Master!$G$2:$G$918,"Core")+COUNTIFS(Master!$C$2:$C$918,"17. Graphs",Master!$G$2:$G$918,"Core")</f>
+        <f>COUNTIF(Master!$B$2:$B$918,"5. Trees &amp; Graphs - Core")</f>
         <v/>
       </c>
       <c r="E13" s="43">
@@ -2012,7 +2012,7 @@
         <v/>
       </c>
       <c r="H13" s="43">
-        <f>COUNTIFS(Master!$C$2:$C$918,"15. Trees &amp; BST",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"15. Trees &amp; BST",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")+COUNTIFS(Master!$C$2:$C$918,"16. Tries",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"16. Tries",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")+COUNTIFS(Master!$C$2:$C$918,"17. Graphs",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"17. Graphs",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")</f>
+        <f>COUNTIFS(Master!$B$2:$B$918,"5. Trees &amp; Graphs - Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$B$2:$B$918,"5. Trees &amp; Graphs - Core",Master!$J$2:$J$918,"Mastered")</f>
         <v/>
       </c>
       <c r="I13" s="45">
@@ -2028,11 +2028,11 @@
       </c>
       <c r="C14" s="42" t="inlineStr">
         <is>
-          <t>18 - 23: Dynamic Programming, Bit Manipulation, Math &amp; Number Theory, Intervals, Design, Advanced DS</t>
+          <t>21 - 23: Dynamic Programming, Design, Advanced DS</t>
         </is>
       </c>
       <c r="D14" s="43">
-        <f>COUNTIFS(Master!$C$2:$C$918,"18. Dynamic Programming",Master!$G$2:$G$918,"Core")+COUNTIFS(Master!$C$2:$C$918,"19. Bit Manipulation",Master!$G$2:$G$918,"Core")+COUNTIFS(Master!$C$2:$C$918,"20. Math &amp; Number Theory",Master!$G$2:$G$918,"Core")+COUNTIFS(Master!$C$2:$C$918,"21. Intervals",Master!$G$2:$G$918,"Core")+COUNTIFS(Master!$C$2:$C$918,"22. Design",Master!$G$2:$G$918,"Core")+COUNTIFS(Master!$C$2:$C$918,"23. Advanced DS",Master!$G$2:$G$918,"Core")</f>
+        <f>COUNTIF(Master!$B$2:$B$918,"6. DP &amp; Closers - Core")</f>
         <v/>
       </c>
       <c r="E14" s="43">
@@ -2048,7 +2048,7 @@
         <v/>
       </c>
       <c r="H14" s="43">
-        <f>COUNTIFS(Master!$C$2:$C$918,"18. Dynamic Programming",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"18. Dynamic Programming",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")+COUNTIFS(Master!$C$2:$C$918,"19. Bit Manipulation",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"19. Bit Manipulation",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")+COUNTIFS(Master!$C$2:$C$918,"20. Math &amp; Number Theory",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"20. Math &amp; Number Theory",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")+COUNTIFS(Master!$C$2:$C$918,"21. Intervals",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"21. Intervals",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")+COUNTIFS(Master!$C$2:$C$918,"22. Design",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"22. Design",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")+COUNTIFS(Master!$C$2:$C$918,"23. Advanced DS",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$C$2:$C$918,"23. Advanced DS",Master!$G$2:$G$918,"Core",Master!$J$2:$J$918,"Mastered")</f>
+        <f>COUNTIFS(Master!$B$2:$B$918,"6. DP &amp; Closers - Core",Master!$J$2:$J$918,"Solved")+COUNTIFS(Master!$B$2:$B$918,"6. DP &amp; Closers - Core",Master!$J$2:$J$918,"Mastered")</f>
         <v/>
       </c>
       <c r="I14" s="45">

</xml_diff>

<commit_message>
Store the Plan start date as a date and fix the phase 2 label
Plan!C5 held the text "2026-09-15", so every Target finish (=$C$5+$F<row>)
relied on locale-dependent text-to-date coercion. It is now the date value,
shown the same through its yyyy-mm-dd format. B10 takes the v4 phase name,
Search, Strings & Math.
</commit_message>
<xml_diff>
--- a/DSA_Master_Sheet.xlsx
+++ b/DSA_Master_Sheet.xlsx
@@ -1776,10 +1776,8 @@
           <t>Start date</t>
         </is>
       </c>
-      <c r="C5" s="38" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
+      <c r="C5" s="38" t="n">
+        <v>46280</v>
       </c>
       <c r="D5" s="39" t="inlineStr">
         <is>
@@ -1879,7 +1877,7 @@
     <row r="10" ht="15" customHeight="1" s="32">
       <c r="B10" s="37" t="inlineStr">
         <is>
-          <t>Phase 2 - Search &amp; Strings</t>
+          <t>Phase 2 - Search, Strings &amp; Math</t>
         </is>
       </c>
       <c r="C10" s="42" t="inlineStr">

</xml_diff>